<commit_message>
Add Great Blue Heron to animals tab
Signed-off-by: Connor Graydon <connorj@bully4u.com>
</commit_message>
<xml_diff>
--- a/chinuk_vocab_gold.xlsx
+++ b/chinuk_vocab_gold.xlsx
@@ -1,43 +1,44 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/connor/Desktop/work/chinuk_vocab_repo/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/connor/Work/chinuk_vocab_repo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3870862F-5F68-7A45-BB35-04CBA5463104}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{748EA4B4-9A5C-6946-BD62-5598C16181A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-39040" yWindow="2040" windowWidth="35160" windowHeight="26700" activeTab="2" xr2:uid="{7DFB5DAA-41FE-8F4C-ADA0-7B74441B15D5}"/>
+    <workbookView xWindow="-52180" yWindow="3860" windowWidth="42960" windowHeight="24520" activeTab="17" xr2:uid="{7DFB5DAA-41FE-8F4C-ADA0-7B74441B15D5}"/>
   </bookViews>
   <sheets>
     <sheet name="Grammar" sheetId="33" r:id="rId1"/>
     <sheet name="Question_words" sheetId="8" r:id="rId2"/>
-    <sheet name="Vocab" sheetId="2" r:id="rId3"/>
-    <sheet name="Handy" sheetId="32" r:id="rId4"/>
-    <sheet name="Learning" sheetId="25" r:id="rId5"/>
-    <sheet name="verbs" sheetId="6" r:id="rId6"/>
-    <sheet name="foods" sheetId="12" r:id="rId7"/>
-    <sheet name="plants" sheetId="11" r:id="rId8"/>
-    <sheet name="Auxilary Words" sheetId="26" r:id="rId9"/>
-    <sheet name="parts of day" sheetId="5" r:id="rId10"/>
-    <sheet name="Days of Week" sheetId="18" r:id="rId11"/>
-    <sheet name="adjectives" sheetId="15" r:id="rId12"/>
-    <sheet name="adverbs" sheetId="7" r:id="rId13"/>
-    <sheet name="misc" sheetId="4" r:id="rId14"/>
-    <sheet name="colors" sheetId="16" r:id="rId15"/>
-    <sheet name="x̣əlel-ikta" sheetId="1" r:id="rId16"/>
-    <sheet name="qʰata mayka" sheetId="20" r:id="rId17"/>
-    <sheet name="House " sheetId="23" r:id="rId18"/>
-    <sheet name="bathroom" sheetId="9" r:id="rId19"/>
-    <sheet name="body_parts" sheetId="19" r:id="rId20"/>
-    <sheet name="Directions" sheetId="22" r:id="rId21"/>
-    <sheet name="PlaceNames" sheetId="24" r:id="rId22"/>
-    <sheet name="tilixam" sheetId="13" r:id="rId23"/>
-    <sheet name="plant_pres_vocab" sheetId="17" r:id="rId24"/>
-    <sheet name="template" sheetId="14" r:id="rId25"/>
+    <sheet name="book" sheetId="34" r:id="rId3"/>
+    <sheet name="Vocab" sheetId="2" r:id="rId4"/>
+    <sheet name="Handy" sheetId="32" r:id="rId5"/>
+    <sheet name="Learning" sheetId="25" r:id="rId6"/>
+    <sheet name="verbs" sheetId="6" r:id="rId7"/>
+    <sheet name="foods" sheetId="12" r:id="rId8"/>
+    <sheet name="plants" sheetId="11" r:id="rId9"/>
+    <sheet name="Auxilary Words" sheetId="26" r:id="rId10"/>
+    <sheet name="parts of day" sheetId="5" r:id="rId11"/>
+    <sheet name="tilixam" sheetId="13" r:id="rId12"/>
+    <sheet name="Days of Week" sheetId="18" r:id="rId13"/>
+    <sheet name="adjectives" sheetId="15" r:id="rId14"/>
+    <sheet name="adverbs" sheetId="7" r:id="rId15"/>
+    <sheet name="misc" sheetId="4" r:id="rId16"/>
+    <sheet name="colors" sheetId="16" r:id="rId17"/>
+    <sheet name="x̣əlel-ikta" sheetId="1" r:id="rId18"/>
+    <sheet name="qʰata mayka" sheetId="20" r:id="rId19"/>
+    <sheet name="House " sheetId="23" r:id="rId20"/>
+    <sheet name="bathroom" sheetId="9" r:id="rId21"/>
+    <sheet name="body_parts" sheetId="19" r:id="rId22"/>
+    <sheet name="Directions" sheetId="22" r:id="rId23"/>
+    <sheet name="PlaceNames" sheetId="24" r:id="rId24"/>
+    <sheet name="plant_pres_vocab" sheetId="17" r:id="rId25"/>
+    <sheet name="template" sheetId="14" r:id="rId26"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -60,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2157" uniqueCount="1777">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2187" uniqueCount="1799">
   <si>
     <t>tʼsiqʰwaʔ</t>
   </si>
@@ -5401,6 +5402,72 @@
   </si>
   <si>
     <t>See also "letter."</t>
+  </si>
+  <si>
+    <t>t’ɬunas maybe, who knows but that…</t>
+  </si>
+  <si>
+    <t>t’ɬunas</t>
+  </si>
+  <si>
+    <t>t’ɬunas qʰənchi-lili alta wəx̣t yaka hayu-nanich…</t>
+  </si>
+  <si>
+    <t>Who knows how long a time, then again she’s looking…. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">t’ɬunas qʰənchi-hayu tilixam wəx̣t kʰapá. </t>
+  </si>
+  <si>
+    <t>I don’t know how many people were also over there.  </t>
+  </si>
+  <si>
+    <t>t’ɬunas-qʰa alta ya t’ɬap ɬaska.</t>
+  </si>
+  <si>
+    <t>Then somewhere or other she found them.  </t>
+  </si>
+  <si>
+    <t>Some thing arrived where we were, I don’t know what. </t>
+  </si>
+  <si>
+    <t>t’ɬunas-ikta ya q’uʔ kʰapa ntsayka.</t>
+  </si>
+  <si>
+    <t>From pipa5-6_cw103_sp2023.pdf</t>
+  </si>
+  <si>
+    <t>iləp-pus</t>
+  </si>
+  <si>
+    <t>alikʰuchik</t>
+  </si>
+  <si>
+    <t>large dentailium</t>
+  </si>
+  <si>
+    <t>shawash-iliʔi tilixam</t>
+  </si>
+  <si>
+    <t>valuables</t>
+  </si>
+  <si>
+    <t>lak'mayut-iliʔi</t>
+  </si>
+  <si>
+    <t>Luckiamuite Land</t>
+  </si>
+  <si>
+    <t>iqsix</t>
+  </si>
+  <si>
+    <t>son in law</t>
+  </si>
+  <si>
+    <t>qʰwashqʰwash </t>
+  </si>
+  <si>
+    <t>Great Blue Heron</t>
   </si>
 </sst>
 </file>
@@ -5780,7 +5847,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -5909,6 +5976,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6453,6 +6523,574 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD9AAA77-1A26-CF4D-855B-50339A62BDBB}">
+  <sheetPr codeName="Sheet5"/>
+  <dimension ref="A1:H26"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="39.75" defaultRowHeight="21"/>
+  <cols>
+    <col min="1" max="1" width="14.25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="37.125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="37.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.875" customWidth="1"/>
+    <col min="8" max="8" width="37.375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="25">
+      <c r="A1" s="50" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="51" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1" s="51" t="s">
+        <v>77</v>
+      </c>
+      <c r="D1" s="51" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" s="51" t="s">
+        <v>77</v>
+      </c>
+      <c r="F1" s="51" t="s">
+        <v>78</v>
+      </c>
+      <c r="G1" s="52"/>
+      <c r="H1" s="52"/>
+    </row>
+    <row r="2" spans="1:8" ht="25">
+      <c r="A2" s="53" t="s">
+        <v>1599</v>
+      </c>
+      <c r="B2" s="54" t="s">
+        <v>1600</v>
+      </c>
+      <c r="C2" s="54" t="s">
+        <v>283</v>
+      </c>
+      <c r="D2" s="54" t="s">
+        <v>284</v>
+      </c>
+      <c r="E2" s="54" t="s">
+        <v>281</v>
+      </c>
+      <c r="F2" s="54" t="s">
+        <v>282</v>
+      </c>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+    </row>
+    <row r="3" spans="1:8" ht="50">
+      <c r="A3" s="53" t="s">
+        <v>1601</v>
+      </c>
+      <c r="B3" s="54" t="s">
+        <v>1602</v>
+      </c>
+      <c r="C3" s="54" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D3" s="54" t="s">
+        <v>1604</v>
+      </c>
+      <c r="E3" s="54" t="s">
+        <v>1605</v>
+      </c>
+      <c r="F3" s="54" t="s">
+        <v>1602</v>
+      </c>
+      <c r="G3" s="52"/>
+      <c r="H3" s="55" t="s">
+        <v>1606</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="25">
+      <c r="A4" s="53" t="s">
+        <v>1607</v>
+      </c>
+      <c r="B4" s="54" t="s">
+        <v>1608</v>
+      </c>
+      <c r="C4" s="54" t="s">
+        <v>1609</v>
+      </c>
+      <c r="D4" s="54" t="s">
+        <v>1610</v>
+      </c>
+      <c r="E4" s="54" t="s">
+        <v>1611</v>
+      </c>
+      <c r="F4" s="54" t="s">
+        <v>1612</v>
+      </c>
+      <c r="G4" s="52"/>
+      <c r="H4" s="52"/>
+    </row>
+    <row r="5" spans="1:8" ht="25">
+      <c r="A5" s="53" t="s">
+        <v>1613</v>
+      </c>
+      <c r="B5" s="54" t="s">
+        <v>1614</v>
+      </c>
+      <c r="C5" s="54" t="s">
+        <v>1615</v>
+      </c>
+      <c r="D5" s="54" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E5" s="54" t="s">
+        <v>1617</v>
+      </c>
+      <c r="F5" s="54" t="s">
+        <v>1618</v>
+      </c>
+      <c r="G5" s="52"/>
+      <c r="H5" s="52"/>
+    </row>
+    <row r="6" spans="1:8" ht="25">
+      <c r="A6" s="53" t="s">
+        <v>1619</v>
+      </c>
+      <c r="B6" s="54" t="s">
+        <v>1620</v>
+      </c>
+      <c r="C6" s="54" t="s">
+        <v>1621</v>
+      </c>
+      <c r="D6" s="54" t="s">
+        <v>1622</v>
+      </c>
+      <c r="E6" s="54" t="s">
+        <v>1623</v>
+      </c>
+      <c r="F6" s="54" t="s">
+        <v>1624</v>
+      </c>
+      <c r="G6" s="52"/>
+      <c r="H6" s="52"/>
+    </row>
+    <row r="7" spans="1:8" ht="25">
+      <c r="A7" s="53" t="s">
+        <v>1625</v>
+      </c>
+      <c r="B7" s="54" t="s">
+        <v>1626</v>
+      </c>
+      <c r="C7" s="54" t="s">
+        <v>1627</v>
+      </c>
+      <c r="D7" s="54" t="s">
+        <v>1628</v>
+      </c>
+      <c r="E7" s="56"/>
+      <c r="F7" s="56"/>
+      <c r="G7" s="52"/>
+      <c r="H7" s="52"/>
+    </row>
+    <row r="8" spans="1:8" ht="25">
+      <c r="A8" s="53" t="s">
+        <v>1629</v>
+      </c>
+      <c r="B8" s="54" t="s">
+        <v>1630</v>
+      </c>
+      <c r="C8" s="54" t="s">
+        <v>1631</v>
+      </c>
+      <c r="D8" s="54" t="s">
+        <v>1632</v>
+      </c>
+      <c r="E8" s="54" t="s">
+        <v>1633</v>
+      </c>
+      <c r="F8" s="54" t="s">
+        <v>1634</v>
+      </c>
+      <c r="G8" s="52"/>
+      <c r="H8" s="52"/>
+    </row>
+    <row r="9" spans="1:8" ht="50">
+      <c r="A9" s="53" t="s">
+        <v>1635</v>
+      </c>
+      <c r="B9" s="54" t="s">
+        <v>1636</v>
+      </c>
+      <c r="C9" s="54" t="s">
+        <v>1637</v>
+      </c>
+      <c r="D9" s="54" t="s">
+        <v>1638</v>
+      </c>
+      <c r="E9" s="56"/>
+      <c r="F9" s="56"/>
+      <c r="G9" s="52"/>
+      <c r="H9" s="52"/>
+    </row>
+    <row r="10" spans="1:8" ht="25">
+      <c r="A10" s="53" t="s">
+        <v>1639</v>
+      </c>
+      <c r="B10" s="54" t="s">
+        <v>1640</v>
+      </c>
+      <c r="C10" s="54" t="s">
+        <v>1641</v>
+      </c>
+      <c r="D10" s="54" t="s">
+        <v>1642</v>
+      </c>
+      <c r="E10" s="56"/>
+      <c r="F10" s="56"/>
+      <c r="G10" s="52"/>
+      <c r="H10" s="52"/>
+    </row>
+    <row r="11" spans="1:8" ht="25">
+      <c r="A11" s="53" t="s">
+        <v>1643</v>
+      </c>
+      <c r="B11" s="54" t="s">
+        <v>1644</v>
+      </c>
+      <c r="C11" s="54" t="s">
+        <v>1470</v>
+      </c>
+      <c r="D11" s="54" t="s">
+        <v>1645</v>
+      </c>
+      <c r="E11" s="54" t="s">
+        <v>1646</v>
+      </c>
+      <c r="F11" s="54" t="s">
+        <v>1647</v>
+      </c>
+      <c r="G11" s="52"/>
+      <c r="H11" s="52"/>
+    </row>
+    <row r="12" spans="1:8" ht="25">
+      <c r="A12" s="53" t="s">
+        <v>1648</v>
+      </c>
+      <c r="B12" s="54" t="s">
+        <v>1649</v>
+      </c>
+      <c r="C12" s="54" t="s">
+        <v>1650</v>
+      </c>
+      <c r="D12" s="54" t="s">
+        <v>1651</v>
+      </c>
+      <c r="E12" s="54" t="s">
+        <v>1652</v>
+      </c>
+      <c r="F12" s="54" t="s">
+        <v>1653</v>
+      </c>
+      <c r="G12" s="52"/>
+      <c r="H12" s="52"/>
+    </row>
+    <row r="13" spans="1:8" ht="25">
+      <c r="A13" s="53" t="s">
+        <v>1654</v>
+      </c>
+      <c r="B13" s="54" t="s">
+        <v>1655</v>
+      </c>
+      <c r="C13" s="54" t="s">
+        <v>1491</v>
+      </c>
+      <c r="D13" s="54" t="s">
+        <v>1492</v>
+      </c>
+      <c r="E13" s="54" t="s">
+        <v>1493</v>
+      </c>
+      <c r="F13" s="54" t="s">
+        <v>1463</v>
+      </c>
+      <c r="G13" s="52"/>
+      <c r="H13" s="52"/>
+    </row>
+    <row r="14" spans="1:8" ht="25">
+      <c r="A14" s="53" t="s">
+        <v>1656</v>
+      </c>
+      <c r="B14" s="54" t="s">
+        <v>1497</v>
+      </c>
+      <c r="C14" s="54" t="s">
+        <v>1657</v>
+      </c>
+      <c r="D14" s="54" t="s">
+        <v>1658</v>
+      </c>
+      <c r="E14" s="54" t="s">
+        <v>1659</v>
+      </c>
+      <c r="F14" s="54" t="s">
+        <v>1660</v>
+      </c>
+      <c r="G14" s="52"/>
+      <c r="H14" s="52"/>
+    </row>
+    <row r="15" spans="1:8" ht="25">
+      <c r="A15" s="53" t="s">
+        <v>1661</v>
+      </c>
+      <c r="B15" s="54" t="s">
+        <v>1662</v>
+      </c>
+      <c r="C15" s="54" t="s">
+        <v>1663</v>
+      </c>
+      <c r="D15" s="54" t="s">
+        <v>1664</v>
+      </c>
+      <c r="E15" s="54" t="s">
+        <v>1665</v>
+      </c>
+      <c r="F15" s="54" t="s">
+        <v>1666</v>
+      </c>
+      <c r="G15" s="52"/>
+      <c r="H15" s="52"/>
+    </row>
+    <row r="16" spans="1:8" ht="25">
+      <c r="A16" s="53" t="s">
+        <v>1667</v>
+      </c>
+      <c r="B16" s="54" t="s">
+        <v>1513</v>
+      </c>
+      <c r="C16" s="54" t="s">
+        <v>1668</v>
+      </c>
+      <c r="D16" s="54" t="s">
+        <v>1668</v>
+      </c>
+      <c r="E16" s="54" t="s">
+        <v>1669</v>
+      </c>
+      <c r="F16" s="54" t="s">
+        <v>1670</v>
+      </c>
+      <c r="G16" s="52"/>
+      <c r="H16" s="52"/>
+    </row>
+    <row r="17" spans="1:8" ht="25">
+      <c r="A17" s="53" t="s">
+        <v>1671</v>
+      </c>
+      <c r="B17" s="54" t="s">
+        <v>336</v>
+      </c>
+      <c r="C17" s="54" t="s">
+        <v>1444</v>
+      </c>
+      <c r="D17" s="54" t="s">
+        <v>1672</v>
+      </c>
+      <c r="E17" s="54" t="s">
+        <v>1673</v>
+      </c>
+      <c r="F17" s="54" t="s">
+        <v>1674</v>
+      </c>
+      <c r="G17" s="52"/>
+      <c r="H17" s="52"/>
+    </row>
+    <row r="18" spans="1:8" ht="25">
+      <c r="A18" s="53" t="s">
+        <v>1675</v>
+      </c>
+      <c r="B18" s="54" t="s">
+        <v>1676</v>
+      </c>
+      <c r="C18" s="54" t="s">
+        <v>1528</v>
+      </c>
+      <c r="D18" s="54" t="s">
+        <v>1677</v>
+      </c>
+      <c r="E18" s="54" t="s">
+        <v>1529</v>
+      </c>
+      <c r="F18" s="54" t="s">
+        <v>1678</v>
+      </c>
+      <c r="G18" s="52"/>
+      <c r="H18" s="52"/>
+    </row>
+    <row r="19" spans="1:8" ht="50">
+      <c r="A19" s="53" t="s">
+        <v>1679</v>
+      </c>
+      <c r="B19" s="54" t="s">
+        <v>1680</v>
+      </c>
+      <c r="C19" s="54" t="s">
+        <v>922</v>
+      </c>
+      <c r="D19" s="54" t="s">
+        <v>1681</v>
+      </c>
+      <c r="E19" s="54" t="s">
+        <v>1682</v>
+      </c>
+      <c r="F19" s="54" t="s">
+        <v>1683</v>
+      </c>
+      <c r="G19" s="52"/>
+      <c r="H19" s="52"/>
+    </row>
+    <row r="20" spans="1:8" ht="50">
+      <c r="A20" s="53" t="s">
+        <v>1684</v>
+      </c>
+      <c r="B20" s="54" t="s">
+        <v>1685</v>
+      </c>
+      <c r="C20" s="54" t="s">
+        <v>1686</v>
+      </c>
+      <c r="D20" s="54" t="s">
+        <v>1687</v>
+      </c>
+      <c r="E20" s="54" t="s">
+        <v>1688</v>
+      </c>
+      <c r="F20" s="54" t="s">
+        <v>1689</v>
+      </c>
+      <c r="G20" s="52"/>
+      <c r="H20" s="52"/>
+    </row>
+    <row r="21" spans="1:8" ht="50">
+      <c r="A21" s="53" t="s">
+        <v>1690</v>
+      </c>
+      <c r="B21" s="54" t="s">
+        <v>1691</v>
+      </c>
+      <c r="C21" s="54" t="s">
+        <v>1692</v>
+      </c>
+      <c r="D21" s="54" t="s">
+        <v>1693</v>
+      </c>
+      <c r="E21" s="54" t="s">
+        <v>1694</v>
+      </c>
+      <c r="F21" s="54" t="s">
+        <v>1695</v>
+      </c>
+      <c r="G21" s="52"/>
+      <c r="H21" s="52"/>
+    </row>
+    <row r="22" spans="1:8" ht="25">
+      <c r="A22" s="53" t="s">
+        <v>1696</v>
+      </c>
+      <c r="B22" s="54" t="s">
+        <v>1544</v>
+      </c>
+      <c r="C22" s="54" t="s">
+        <v>1697</v>
+      </c>
+      <c r="D22" s="54" t="s">
+        <v>1698</v>
+      </c>
+      <c r="E22" s="54" t="s">
+        <v>1699</v>
+      </c>
+      <c r="F22" s="54" t="s">
+        <v>1700</v>
+      </c>
+      <c r="G22" s="52"/>
+      <c r="H22" s="52"/>
+    </row>
+    <row r="23" spans="1:8" ht="25">
+      <c r="A23" s="53" t="s">
+        <v>1701</v>
+      </c>
+      <c r="B23" s="54" t="s">
+        <v>1702</v>
+      </c>
+      <c r="C23" s="54" t="s">
+        <v>1554</v>
+      </c>
+      <c r="D23" s="54" t="s">
+        <v>1703</v>
+      </c>
+      <c r="E23" s="56"/>
+      <c r="F23" s="56"/>
+      <c r="G23" s="52"/>
+      <c r="H23" s="52"/>
+    </row>
+    <row r="24" spans="1:8" ht="25">
+      <c r="A24" s="53" t="s">
+        <v>1704</v>
+      </c>
+      <c r="B24" s="54" t="s">
+        <v>1705</v>
+      </c>
+      <c r="C24" s="54" t="s">
+        <v>1706</v>
+      </c>
+      <c r="D24" s="54" t="s">
+        <v>1707</v>
+      </c>
+      <c r="E24" s="56"/>
+      <c r="F24" s="56"/>
+      <c r="G24" s="52"/>
+      <c r="H24" s="52"/>
+    </row>
+    <row r="25" spans="1:8" ht="25">
+      <c r="A25" s="53" t="s">
+        <v>1708</v>
+      </c>
+      <c r="B25" s="54" t="s">
+        <v>1709</v>
+      </c>
+      <c r="C25" s="54" t="s">
+        <v>1710</v>
+      </c>
+      <c r="D25" s="54" t="s">
+        <v>1711</v>
+      </c>
+      <c r="E25" s="56"/>
+      <c r="F25" s="56"/>
+      <c r="G25" s="52"/>
+      <c r="H25" s="52"/>
+    </row>
+    <row r="26" spans="1:8" ht="25">
+      <c r="A26" s="53" t="s">
+        <v>1712</v>
+      </c>
+      <c r="B26" s="54" t="s">
+        <v>1713</v>
+      </c>
+      <c r="C26" s="54" t="s">
+        <v>1567</v>
+      </c>
+      <c r="D26" s="54" t="s">
+        <v>1714</v>
+      </c>
+      <c r="E26" s="56"/>
+      <c r="F26" s="56"/>
+      <c r="G26" s="52"/>
+      <c r="H26" s="52"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0621B05F-84D3-C041-A876-6535B8901E4C}">
   <sheetPr codeName="Sheet6"/>
   <dimension ref="A2:C14"/>
@@ -6580,7 +7218,237 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F53271B7-0EAD-D94F-8AA6-BD76BFA13A48}">
+  <sheetPr codeName="Sheet26"/>
+  <dimension ref="A2:C26"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="21"/>
+  <cols>
+    <col min="1" max="1" width="21.625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:3" ht="31">
+      <c r="A2" s="19" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="24">
+      <c r="A4" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="B4" s="29" t="s">
+        <v>78</v>
+      </c>
+      <c r="C4" s="29" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="24">
+      <c r="A5" s="30" t="s">
+        <v>815</v>
+      </c>
+      <c r="B5" s="31" t="s">
+        <v>816</v>
+      </c>
+      <c r="C5" s="12"/>
+    </row>
+    <row r="6" spans="1:3" ht="24">
+      <c r="A6" s="13" t="s">
+        <v>504</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>505</v>
+      </c>
+      <c r="C6" s="32"/>
+    </row>
+    <row r="7" spans="1:3" ht="24">
+      <c r="A7" s="13" t="s">
+        <v>506</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>507</v>
+      </c>
+      <c r="C7" s="14"/>
+    </row>
+    <row r="8" spans="1:3" ht="24">
+      <c r="A8" s="13" t="s">
+        <v>508</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>509</v>
+      </c>
+      <c r="C8" s="14"/>
+    </row>
+    <row r="9" spans="1:3" ht="24">
+      <c r="A9" s="13" t="s">
+        <v>809</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>810</v>
+      </c>
+      <c r="C9" s="14"/>
+    </row>
+    <row r="10" spans="1:3" ht="24">
+      <c r="A10" s="13" t="s">
+        <v>510</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>511</v>
+      </c>
+      <c r="C10" s="14"/>
+    </row>
+    <row r="11" spans="1:3" ht="24">
+      <c r="A11" s="13" t="s">
+        <v>811</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>812</v>
+      </c>
+      <c r="C11" s="14"/>
+    </row>
+    <row r="12" spans="1:3" ht="24">
+      <c r="A12" s="13" t="s">
+        <v>512</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>513</v>
+      </c>
+      <c r="C12" s="14"/>
+    </row>
+    <row r="13" spans="1:3" ht="24">
+      <c r="A13" s="14" t="s">
+        <v>817</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>819</v>
+      </c>
+      <c r="C13" s="14"/>
+    </row>
+    <row r="14" spans="1:3" ht="24">
+      <c r="A14" s="14" t="s">
+        <v>818</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>820</v>
+      </c>
+      <c r="C14" s="14"/>
+    </row>
+    <row r="15" spans="1:3" ht="24">
+      <c r="A15" s="13" t="s">
+        <v>514</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>515</v>
+      </c>
+      <c r="C15" s="14"/>
+    </row>
+    <row r="16" spans="1:3" ht="24">
+      <c r="A16" s="13" t="s">
+        <v>516</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>517</v>
+      </c>
+      <c r="C16" s="14"/>
+    </row>
+    <row r="17" spans="1:3" ht="24">
+      <c r="A17" s="13" t="s">
+        <v>518</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>519</v>
+      </c>
+      <c r="C17" s="14"/>
+    </row>
+    <row r="18" spans="1:3" ht="24">
+      <c r="A18" s="13" t="s">
+        <v>520</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>521</v>
+      </c>
+      <c r="C18" s="14"/>
+    </row>
+    <row r="19" spans="1:3" ht="24">
+      <c r="A19" s="30" t="s">
+        <v>805</v>
+      </c>
+      <c r="B19" s="31" t="s">
+        <v>806</v>
+      </c>
+      <c r="C19" s="14"/>
+    </row>
+    <row r="20" spans="1:3" ht="24">
+      <c r="A20" s="13" t="s">
+        <v>807</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>808</v>
+      </c>
+      <c r="C20" s="32"/>
+    </row>
+    <row r="21" spans="1:3" ht="24">
+      <c r="A21" s="13" t="s">
+        <v>813</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>814</v>
+      </c>
+      <c r="C21" s="32"/>
+    </row>
+    <row r="22" spans="1:3" ht="24">
+      <c r="A22" s="13" t="s">
+        <v>1449</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>1448</v>
+      </c>
+      <c r="C22" s="32"/>
+    </row>
+    <row r="23" spans="1:3" ht="24">
+      <c r="A23" s="13" t="s">
+        <v>821</v>
+      </c>
+      <c r="B23" s="14" t="s">
+        <v>822</v>
+      </c>
+      <c r="C23" s="32"/>
+    </row>
+    <row r="24" spans="1:3" ht="24">
+      <c r="A24" s="13" t="s">
+        <v>821</v>
+      </c>
+      <c r="B24" s="14" t="s">
+        <v>822</v>
+      </c>
+      <c r="C24" s="14"/>
+    </row>
+    <row r="25" spans="1:3" ht="24">
+      <c r="A25" s="13" t="s">
+        <v>1451</v>
+      </c>
+      <c r="B25" s="14" t="s">
+        <v>1450</v>
+      </c>
+      <c r="C25" s="14"/>
+    </row>
+    <row r="26" spans="1:3" ht="24">
+      <c r="A26" s="13" t="s">
+        <v>1795</v>
+      </c>
+      <c r="B26" s="14" t="s">
+        <v>1796</v>
+      </c>
+      <c r="C26" s="14"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F67C7AAB-967B-5045-BDCA-9F7B04711E90}">
   <sheetPr codeName="Sheet7"/>
   <dimension ref="A3:C29"/>
@@ -6800,7 +7668,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D11FE1F-F4A2-4243-AD49-0AE386224F39}">
   <sheetPr codeName="Sheet8"/>
   <dimension ref="A2:C38"/>
@@ -7115,7 +7983,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F29A4BE1-9EDE-B14C-A890-3CF582053E14}">
   <sheetPr codeName="Sheet9"/>
   <dimension ref="A1:E26"/>
@@ -7376,7 +8244,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B3091FA-FA4D-C844-8EC8-A36691B6A574}">
   <sheetPr codeName="Sheet10"/>
   <dimension ref="A2:H96"/>
@@ -8288,7 +9156,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B274FF1E-1838-214B-B5DD-642DFDA172AC}">
   <sheetPr codeName="Sheet11"/>
   <dimension ref="A2:C13"/>
@@ -8408,10 +9276,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE17E8DC-C5DA-1E49-AE1C-D1A03DE11DA3}">
   <sheetPr codeName="Sheet12"/>
-  <dimension ref="A1:X38"/>
+  <dimension ref="A1:X39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="21"/>
   <cols>
     <col min="1" max="2" width="30.25" customWidth="1"/>
@@ -8466,10 +9334,10 @@
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="5" t="s">
-        <v>6</v>
+        <v>305</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>133</v>
+        <v>304</v>
       </c>
       <c r="I4" s="4"/>
       <c r="J4" s="1"/>
@@ -8504,10 +9372,10 @@
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>101</v>
+        <v>6</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>133</v>
       </c>
       <c r="I5" s="4"/>
       <c r="J5" s="1"/>
@@ -8542,10 +9410,10 @@
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>124</v>
+        <v>23</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>101</v>
       </c>
       <c r="I6" s="4"/>
       <c r="J6" s="1"/>
@@ -8580,10 +9448,10 @@
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="5" t="s">
-        <v>1716</v>
+        <v>11</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="I7" s="4"/>
       <c r="J7" s="1"/>
@@ -8618,10 +9486,10 @@
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="5" t="s">
-        <v>70</v>
+        <v>1716</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>137</v>
+        <v>118</v>
       </c>
       <c r="I8" s="4"/>
       <c r="J8" s="1"/>
@@ -8656,10 +9524,10 @@
       </c>
       <c r="F9" s="1"/>
       <c r="G9" s="5" t="s">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>118</v>
+        <v>137</v>
       </c>
       <c r="I9" s="4"/>
       <c r="J9" s="1"/>
@@ -8694,10 +9562,10 @@
       </c>
       <c r="F10" s="1"/>
       <c r="G10" s="5" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I10" s="4"/>
       <c r="J10" s="1"/>
@@ -8732,10 +9600,10 @@
       </c>
       <c r="F11" s="1"/>
       <c r="G11" s="5" t="s">
-        <v>67</v>
+        <v>27</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>83</v>
+        <v>122</v>
       </c>
       <c r="I11" s="4"/>
       <c r="J11" s="1"/>
@@ -8770,10 +9638,10 @@
       </c>
       <c r="F12" s="1"/>
       <c r="G12" s="5" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>125</v>
+        <v>83</v>
       </c>
       <c r="I12" s="4"/>
       <c r="J12" s="1"/>
@@ -8808,10 +9676,10 @@
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="5" t="s">
-        <v>1322</v>
+        <v>64</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>1323</v>
+        <v>125</v>
       </c>
       <c r="I13" s="4"/>
       <c r="J13" s="1"/>
@@ -8846,10 +9714,10 @@
       </c>
       <c r="F14" s="1"/>
       <c r="G14" s="5" t="s">
-        <v>17</v>
+        <v>1322</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>117</v>
+        <v>1323</v>
       </c>
       <c r="I14" s="4"/>
       <c r="J14" s="1"/>
@@ -8884,10 +9752,10 @@
       </c>
       <c r="F15" s="1"/>
       <c r="G15" s="5" t="s">
-        <v>157</v>
+        <v>17</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>158</v>
+        <v>117</v>
       </c>
       <c r="I15" s="4"/>
       <c r="J15" s="1"/>
@@ -8922,10 +9790,10 @@
       </c>
       <c r="F16" s="1"/>
       <c r="G16" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>98</v>
+        <v>157</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>158</v>
       </c>
       <c r="I16" s="4"/>
       <c r="J16" s="1"/>
@@ -8960,10 +9828,10 @@
       </c>
       <c r="F17" s="1"/>
       <c r="G17" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="H17" s="5" t="s">
-        <v>95</v>
+        <v>38</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>98</v>
       </c>
       <c r="I17" s="4"/>
       <c r="J17" s="1"/>
@@ -8998,10 +9866,10 @@
       </c>
       <c r="F18" s="1"/>
       <c r="G18" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="H18" s="6" t="s">
-        <v>100</v>
+        <v>0</v>
+      </c>
+      <c r="H18" s="5" t="s">
+        <v>95</v>
       </c>
       <c r="I18" s="4"/>
       <c r="J18" s="1"/>
@@ -9035,11 +9903,11 @@
         <v>123</v>
       </c>
       <c r="F19" s="1"/>
-      <c r="G19" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="H19" s="7" t="s">
-        <v>154</v>
+      <c r="G19" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>100</v>
       </c>
       <c r="I19" s="4"/>
       <c r="J19" s="1"/>
@@ -9067,17 +9935,17 @@
       </c>
       <c r="C20" s="1"/>
       <c r="D20" s="5" t="s">
-        <v>48</v>
+        <v>1797</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>119</v>
+        <v>1798</v>
       </c>
       <c r="F20" s="1"/>
-      <c r="G20" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="H20" s="6" t="s">
-        <v>108</v>
+      <c r="G20" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>154</v>
       </c>
       <c r="I20" s="4"/>
       <c r="J20" s="1"/>
@@ -9105,17 +9973,17 @@
       </c>
       <c r="C21" s="1"/>
       <c r="D21" s="5" t="s">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>81</v>
+        <v>119</v>
       </c>
       <c r="F21" s="1"/>
-      <c r="G21" s="45" t="s">
-        <v>522</v>
-      </c>
-      <c r="H21" s="45" t="s">
-        <v>523</v>
+      <c r="G21" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>108</v>
       </c>
       <c r="I21" s="4"/>
       <c r="J21" s="1"/>
@@ -9143,17 +10011,17 @@
       </c>
       <c r="C22" s="1"/>
       <c r="D22" s="5" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>143</v>
+        <v>81</v>
       </c>
       <c r="F22" s="1"/>
-      <c r="G22" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="H22" s="6" t="s">
-        <v>104</v>
+      <c r="G22" s="45" t="s">
+        <v>522</v>
+      </c>
+      <c r="H22" s="45" t="s">
+        <v>523</v>
       </c>
       <c r="I22" s="4"/>
       <c r="J22" s="1"/>
@@ -9181,17 +10049,17 @@
       </c>
       <c r="C23" s="1"/>
       <c r="D23" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="E23" s="6" t="s">
-        <v>128</v>
+        <v>54</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>143</v>
       </c>
       <c r="F23" s="1"/>
       <c r="G23" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="H23" s="5" t="s">
-        <v>145</v>
+        <v>5</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>104</v>
       </c>
       <c r="I23" s="4"/>
       <c r="J23" s="1"/>
@@ -9219,17 +10087,17 @@
       </c>
       <c r="C24" s="1"/>
       <c r="D24" s="5" t="s">
-        <v>71</v>
+        <v>50</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>102</v>
+        <v>128</v>
       </c>
       <c r="F24" s="1"/>
       <c r="G24" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="H24" s="6" t="s">
-        <v>113</v>
+        <v>72</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>145</v>
       </c>
       <c r="I24" s="4"/>
       <c r="J24" s="1"/>
@@ -9257,17 +10125,17 @@
       </c>
       <c r="C25" s="1"/>
       <c r="D25" s="5" t="s">
-        <v>12</v>
+        <v>71</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="F25" s="1"/>
       <c r="G25" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="H25" s="5" t="s">
-        <v>97</v>
+        <v>16</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>113</v>
       </c>
       <c r="I25" s="4"/>
       <c r="J25" s="1"/>
@@ -9295,17 +10163,17 @@
       </c>
       <c r="C26" s="1"/>
       <c r="D26" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="E26" s="5" t="s">
-        <v>96</v>
+        <v>12</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>99</v>
       </c>
       <c r="F26" s="1"/>
       <c r="G26" s="5" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>132</v>
+        <v>97</v>
       </c>
       <c r="I26" s="4"/>
       <c r="J26" s="1"/>
@@ -9333,17 +10201,17 @@
       </c>
       <c r="C27" s="1"/>
       <c r="D27" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="E27" s="6" t="s">
-        <v>152</v>
+        <v>4</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>96</v>
       </c>
       <c r="F27" s="1"/>
       <c r="G27" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="H27" s="6" t="s">
-        <v>107</v>
+        <v>68</v>
+      </c>
+      <c r="H27" s="5" t="s">
+        <v>132</v>
       </c>
       <c r="I27" s="4"/>
       <c r="J27" s="1"/>
@@ -9371,17 +10239,17 @@
       </c>
       <c r="C28" s="1"/>
       <c r="D28" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="E28" s="5" t="s">
-        <v>151</v>
+        <v>2</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>152</v>
       </c>
       <c r="F28" s="1"/>
       <c r="G28" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="H28" s="5" t="s">
-        <v>90</v>
+        <v>73</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>107</v>
       </c>
       <c r="I28" s="4"/>
       <c r="J28" s="1"/>
@@ -9409,17 +10277,17 @@
       </c>
       <c r="C29" s="1"/>
       <c r="D29" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="E29" s="6" t="s">
-        <v>93</v>
+        <v>35</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>151</v>
       </c>
       <c r="F29" s="1"/>
       <c r="G29" s="5" t="s">
-        <v>15</v>
+        <v>74</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>115</v>
+        <v>90</v>
       </c>
       <c r="I29" s="4"/>
       <c r="J29" s="1"/>
@@ -9447,17 +10315,17 @@
       </c>
       <c r="C30" s="1"/>
       <c r="D30" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E30" s="5" t="s">
-        <v>109</v>
+        <v>58</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>93</v>
       </c>
       <c r="F30" s="1"/>
       <c r="G30" s="5" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="I30" s="4"/>
       <c r="J30" s="1"/>
@@ -9485,17 +10353,17 @@
       </c>
       <c r="C31" s="1"/>
       <c r="D31" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>131</v>
+        <v>42</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>109</v>
       </c>
       <c r="F31" s="1"/>
       <c r="G31" s="5" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="I31" s="4"/>
       <c r="J31" s="1"/>
@@ -9523,12 +10391,18 @@
       </c>
       <c r="C32" s="1"/>
       <c r="D32" s="5" t="s">
-        <v>305</v>
-      </c>
-      <c r="E32" s="5" t="s">
-        <v>304</v>
+        <v>26</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>131</v>
       </c>
       <c r="F32" s="1"/>
+      <c r="G32" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H32" s="5" t="s">
+        <v>82</v>
+      </c>
       <c r="I32" s="4"/>
       <c r="J32" s="1"/>
       <c r="K32" s="1"/>
@@ -9550,8 +10424,6 @@
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
-      <c r="D33" s="1"/>
-      <c r="E33" s="1"/>
       <c r="F33" s="1"/>
       <c r="I33" s="1"/>
       <c r="J33" s="1"/>
@@ -9574,8 +10446,8 @@
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
-      <c r="D34" s="3"/>
-      <c r="E34" s="3"/>
+      <c r="D34" s="1"/>
+      <c r="E34" s="1"/>
       <c r="F34" s="3"/>
       <c r="I34" s="1"/>
       <c r="J34" s="1"/>
@@ -9594,15 +10466,13 @@
       <c r="W34" s="1"/>
       <c r="X34" s="1"/>
     </row>
-    <row r="35" spans="1:24" ht="24">
+    <row r="35" spans="1:24">
       <c r="A35" s="3"/>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
-      <c r="G35" s="45"/>
-      <c r="H35" s="45"/>
       <c r="I35" s="1"/>
       <c r="J35" s="1"/>
       <c r="K35" s="1"/>
@@ -9620,11 +10490,13 @@
       <c r="W35" s="1"/>
       <c r="X35" s="1"/>
     </row>
-    <row r="36" spans="1:24">
+    <row r="36" spans="1:24" ht="24">
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
+      <c r="G36" s="45"/>
+      <c r="H36" s="45"/>
       <c r="I36" s="1"/>
       <c r="J36" s="1"/>
       <c r="K36" s="1"/>
@@ -9665,8 +10537,12 @@
       <c r="V37" s="1"/>
     </row>
     <row r="38" spans="1:24">
-      <c r="G38" s="1"/>
-      <c r="H38" s="1"/>
+      <c r="D38" s="3"/>
+      <c r="E38" s="3"/>
+    </row>
+    <row r="39" spans="1:24">
+      <c r="G39" s="1"/>
+      <c r="H39" s="1"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:B31">
@@ -9677,7 +10553,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE750D78-E2F3-B742-B882-1710CECA9C5E}">
   <sheetPr codeName="Sheet18"/>
   <dimension ref="A2:C20"/>
@@ -9860,7 +10736,369 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{958F5EED-587F-4E45-80B8-2EABD5CA4158}">
+  <sheetPr codeName="Sheet1"/>
+  <dimension ref="A2:H29"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="21"/>
+  <cols>
+    <col min="1" max="1" width="21.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="45.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="53.75" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="31.875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:8" ht="31">
+      <c r="A2" s="19" t="s">
+        <v>456</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1447</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="31">
+      <c r="A3" s="19"/>
+    </row>
+    <row r="4" spans="1:8" ht="24">
+      <c r="A4" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>457</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="24">
+      <c r="A5" s="21" t="s">
+        <v>177</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>409</v>
+      </c>
+      <c r="C5" s="21"/>
+      <c r="F5" s="21" t="s">
+        <v>1177</v>
+      </c>
+      <c r="G5" s="21" t="s">
+        <v>1178</v>
+      </c>
+      <c r="H5" s="21"/>
+    </row>
+    <row r="6" spans="1:8" ht="24">
+      <c r="A6" s="21" t="s">
+        <v>410</v>
+      </c>
+      <c r="B6" s="21" t="s">
+        <v>411</v>
+      </c>
+      <c r="C6" s="21"/>
+      <c r="F6" s="21" t="s">
+        <v>566</v>
+      </c>
+      <c r="G6" s="21" t="s">
+        <v>1345</v>
+      </c>
+      <c r="H6" s="21"/>
+    </row>
+    <row r="7" spans="1:8" ht="24">
+      <c r="A7" s="21" t="s">
+        <v>412</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>413</v>
+      </c>
+      <c r="C7" s="21"/>
+      <c r="F7" s="21" t="s">
+        <v>1132</v>
+      </c>
+      <c r="G7" s="21" t="s">
+        <v>1133</v>
+      </c>
+      <c r="H7" s="21"/>
+    </row>
+    <row r="8" spans="1:8" ht="24">
+      <c r="A8" s="21" t="s">
+        <v>251</v>
+      </c>
+      <c r="B8" s="21" t="s">
+        <v>252</v>
+      </c>
+      <c r="C8" s="21"/>
+      <c r="F8" s="21" t="s">
+        <v>1185</v>
+      </c>
+      <c r="G8" s="21" t="s">
+        <v>1186</v>
+      </c>
+      <c r="H8" s="21"/>
+    </row>
+    <row r="9" spans="1:8" ht="24">
+      <c r="A9" s="21" t="s">
+        <v>414</v>
+      </c>
+      <c r="B9" s="21" t="s">
+        <v>415</v>
+      </c>
+      <c r="C9" s="21"/>
+    </row>
+    <row r="10" spans="1:8" ht="24">
+      <c r="A10" s="21" t="s">
+        <v>417</v>
+      </c>
+      <c r="B10" s="21" t="s">
+        <v>416</v>
+      </c>
+      <c r="C10" s="21"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="21"/>
+      <c r="H10" s="21"/>
+    </row>
+    <row r="11" spans="1:8" ht="24">
+      <c r="A11" s="21" t="s">
+        <v>418</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>419</v>
+      </c>
+      <c r="C11" s="21"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="21"/>
+      <c r="H11" s="21"/>
+    </row>
+    <row r="12" spans="1:8" ht="24">
+      <c r="A12" s="21" t="s">
+        <v>179</v>
+      </c>
+      <c r="B12" s="21" t="s">
+        <v>170</v>
+      </c>
+      <c r="C12" s="21"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="21"/>
+      <c r="H12" s="21"/>
+    </row>
+    <row r="13" spans="1:8" ht="24">
+      <c r="A13" s="21" t="s">
+        <v>1168</v>
+      </c>
+      <c r="B13" s="21" t="s">
+        <v>1169</v>
+      </c>
+      <c r="C13" s="21"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="21"/>
+      <c r="H13" s="21"/>
+    </row>
+    <row r="14" spans="1:8" ht="24">
+      <c r="A14" s="21" t="s">
+        <v>1170</v>
+      </c>
+      <c r="B14" s="21" t="s">
+        <v>1171</v>
+      </c>
+      <c r="C14" s="21"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="21"/>
+    </row>
+    <row r="15" spans="1:8" ht="24">
+      <c r="A15" s="21" t="s">
+        <v>1172</v>
+      </c>
+      <c r="B15" s="21" t="s">
+        <v>1173</v>
+      </c>
+      <c r="C15" s="21"/>
+    </row>
+    <row r="16" spans="1:8" ht="24">
+      <c r="A16" s="21" t="s">
+        <v>1174</v>
+      </c>
+      <c r="B16" s="21" t="s">
+        <v>1175</v>
+      </c>
+      <c r="C16" s="21"/>
+    </row>
+    <row r="17" spans="1:8" ht="24">
+      <c r="A17" s="9"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+    </row>
+    <row r="18" spans="1:8" ht="31">
+      <c r="A18" s="9"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="9"/>
+      <c r="F18" s="19" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="31">
+      <c r="A19" s="19" t="s">
+        <v>1176</v>
+      </c>
+      <c r="F19" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="H19" s="10" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="24">
+      <c r="A20" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>457</v>
+      </c>
+      <c r="F20" s="21" t="s">
+        <v>1778</v>
+      </c>
+      <c r="G20" s="21" t="s">
+        <v>1777</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="26">
+      <c r="A21" s="44" t="s">
+        <v>1179</v>
+      </c>
+      <c r="B21" s="44" t="s">
+        <v>1180</v>
+      </c>
+      <c r="C21" s="44"/>
+      <c r="F21" s="21" t="s">
+        <v>1786</v>
+      </c>
+      <c r="G21" s="21" t="s">
+        <v>1785</v>
+      </c>
+      <c r="H21" s="21" t="s">
+        <v>1787</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="26">
+      <c r="A22" s="44" t="s">
+        <v>1181</v>
+      </c>
+      <c r="B22" s="44" t="s">
+        <v>1182</v>
+      </c>
+      <c r="C22" s="44"/>
+      <c r="F22" s="21" t="s">
+        <v>1783</v>
+      </c>
+      <c r="G22" s="21" t="s">
+        <v>1784</v>
+      </c>
+      <c r="H22" s="21"/>
+    </row>
+    <row r="23" spans="1:8" ht="26">
+      <c r="A23" s="44" t="s">
+        <v>1183</v>
+      </c>
+      <c r="B23" s="44" t="s">
+        <v>1184</v>
+      </c>
+      <c r="C23" s="44"/>
+      <c r="F23" s="21" t="s">
+        <v>1781</v>
+      </c>
+      <c r="G23" s="21" t="s">
+        <v>1782</v>
+      </c>
+      <c r="H23" s="21"/>
+    </row>
+    <row r="24" spans="1:8" ht="26">
+      <c r="A24" s="44" t="s">
+        <v>1187</v>
+      </c>
+      <c r="B24" s="44" t="s">
+        <v>1188</v>
+      </c>
+      <c r="C24" s="44"/>
+      <c r="F24" s="21" t="s">
+        <v>1779</v>
+      </c>
+      <c r="G24" s="21" t="s">
+        <v>1780</v>
+      </c>
+      <c r="H24" s="21"/>
+    </row>
+    <row r="25" spans="1:8" ht="26">
+      <c r="A25" s="44" t="s">
+        <v>1177</v>
+      </c>
+      <c r="B25" s="44" t="s">
+        <v>1178</v>
+      </c>
+      <c r="C25" s="44" t="s">
+        <v>1189</v>
+      </c>
+      <c r="F25" s="21"/>
+      <c r="G25" s="21"/>
+      <c r="H25" s="21"/>
+    </row>
+    <row r="26" spans="1:8" ht="26">
+      <c r="A26" s="44" t="s">
+        <v>1190</v>
+      </c>
+      <c r="B26" s="44" t="s">
+        <v>1191</v>
+      </c>
+      <c r="C26" s="44"/>
+      <c r="F26" s="21"/>
+      <c r="G26" s="21"/>
+      <c r="H26" s="21"/>
+    </row>
+    <row r="27" spans="1:8" ht="24">
+      <c r="A27" s="23"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="21"/>
+      <c r="H27" s="21"/>
+    </row>
+    <row r="28" spans="1:8" ht="24">
+      <c r="A28" s="21"/>
+      <c r="B28" s="21"/>
+      <c r="C28" s="21"/>
+      <c r="F28" s="21"/>
+      <c r="G28" s="21"/>
+      <c r="H28" s="21"/>
+    </row>
+    <row r="29" spans="1:8" ht="24">
+      <c r="A29" s="21"/>
+      <c r="B29" s="21"/>
+      <c r="C29" s="21"/>
+      <c r="F29" s="21"/>
+      <c r="G29" s="21"/>
+      <c r="H29" s="21"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B72F937A-4684-FC4D-BDC3-F85FA5A8BEEC}">
   <sheetPr codeName="Sheet19"/>
   <dimension ref="A2:C46"/>
@@ -10279,7 +11517,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D371A750-118C-6F46-8EB6-D8BED82A7A0D}">
   <sheetPr codeName="Sheet20"/>
   <dimension ref="A2:D42"/>
@@ -10569,303 +11807,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{958F5EED-587F-4E45-80B8-2EABD5CA4158}">
-  <sheetPr codeName="Sheet1"/>
-  <dimension ref="A2:H28"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="21"/>
-  <cols>
-    <col min="1" max="1" width="21.75" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.75" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="1:8" ht="31">
-      <c r="A2" s="19" t="s">
-        <v>456</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1447</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="31">
-      <c r="A3" s="19"/>
-    </row>
-    <row r="4" spans="1:8" ht="24">
-      <c r="A4" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>457</v>
-      </c>
-      <c r="F4" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="G4" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="H4" s="10" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="24">
-      <c r="A5" s="21" t="s">
-        <v>177</v>
-      </c>
-      <c r="B5" s="21" t="s">
-        <v>409</v>
-      </c>
-      <c r="C5" s="21"/>
-      <c r="F5" s="21" t="s">
-        <v>1177</v>
-      </c>
-      <c r="G5" s="21" t="s">
-        <v>1178</v>
-      </c>
-      <c r="H5" s="21"/>
-    </row>
-    <row r="6" spans="1:8" ht="24">
-      <c r="A6" s="21" t="s">
-        <v>410</v>
-      </c>
-      <c r="B6" s="21" t="s">
-        <v>411</v>
-      </c>
-      <c r="C6" s="21"/>
-      <c r="F6" s="21" t="s">
-        <v>566</v>
-      </c>
-      <c r="G6" s="21" t="s">
-        <v>1345</v>
-      </c>
-      <c r="H6" s="21"/>
-    </row>
-    <row r="7" spans="1:8" ht="24">
-      <c r="A7" s="21" t="s">
-        <v>412</v>
-      </c>
-      <c r="B7" s="21" t="s">
-        <v>413</v>
-      </c>
-      <c r="C7" s="21"/>
-      <c r="F7" s="21" t="s">
-        <v>1132</v>
-      </c>
-      <c r="G7" s="21" t="s">
-        <v>1133</v>
-      </c>
-      <c r="H7" s="21"/>
-    </row>
-    <row r="8" spans="1:8" ht="24">
-      <c r="A8" s="21" t="s">
-        <v>251</v>
-      </c>
-      <c r="B8" s="21" t="s">
-        <v>252</v>
-      </c>
-      <c r="C8" s="21"/>
-      <c r="F8" s="21" t="s">
-        <v>1185</v>
-      </c>
-      <c r="G8" s="21" t="s">
-        <v>1186</v>
-      </c>
-      <c r="H8" s="21"/>
-    </row>
-    <row r="9" spans="1:8" ht="24">
-      <c r="A9" s="21" t="s">
-        <v>414</v>
-      </c>
-      <c r="B9" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="C9" s="21"/>
-    </row>
-    <row r="10" spans="1:8" ht="24">
-      <c r="A10" s="21" t="s">
-        <v>417</v>
-      </c>
-      <c r="B10" s="21" t="s">
-        <v>416</v>
-      </c>
-      <c r="C10" s="21"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
-      <c r="H10" s="21"/>
-    </row>
-    <row r="11" spans="1:8" ht="24">
-      <c r="A11" s="21" t="s">
-        <v>418</v>
-      </c>
-      <c r="B11" s="21" t="s">
-        <v>419</v>
-      </c>
-      <c r="C11" s="21"/>
-      <c r="F11" s="21"/>
-      <c r="G11" s="21"/>
-      <c r="H11" s="21"/>
-    </row>
-    <row r="12" spans="1:8" ht="24">
-      <c r="A12" s="21" t="s">
-        <v>179</v>
-      </c>
-      <c r="B12" s="21" t="s">
-        <v>170</v>
-      </c>
-      <c r="C12" s="21"/>
-      <c r="F12" s="21"/>
-      <c r="G12" s="21"/>
-      <c r="H12" s="21"/>
-    </row>
-    <row r="13" spans="1:8" ht="24">
-      <c r="A13" s="21" t="s">
-        <v>1168</v>
-      </c>
-      <c r="B13" s="21" t="s">
-        <v>1169</v>
-      </c>
-      <c r="C13" s="21"/>
-      <c r="F13" s="21"/>
-      <c r="G13" s="21"/>
-      <c r="H13" s="21"/>
-    </row>
-    <row r="14" spans="1:8" ht="24">
-      <c r="A14" s="21" t="s">
-        <v>1170</v>
-      </c>
-      <c r="B14" s="21" t="s">
-        <v>1171</v>
-      </c>
-      <c r="C14" s="21"/>
-      <c r="F14" s="21"/>
-      <c r="G14" s="21"/>
-      <c r="H14" s="21"/>
-    </row>
-    <row r="15" spans="1:8" ht="24">
-      <c r="A15" s="21" t="s">
-        <v>1172</v>
-      </c>
-      <c r="B15" s="21" t="s">
-        <v>1173</v>
-      </c>
-      <c r="C15" s="21"/>
-    </row>
-    <row r="16" spans="1:8" ht="24">
-      <c r="A16" s="21" t="s">
-        <v>1174</v>
-      </c>
-      <c r="B16" s="21" t="s">
-        <v>1175</v>
-      </c>
-      <c r="C16" s="21"/>
-    </row>
-    <row r="17" spans="1:8" ht="24">
-      <c r="A17" s="9"/>
-      <c r="B17" s="9"/>
-      <c r="C17" s="9"/>
-    </row>
-    <row r="18" spans="1:8" ht="31">
-      <c r="A18" s="9"/>
-      <c r="B18" s="9"/>
-      <c r="C18" s="9"/>
-      <c r="F18" s="19" t="s">
-        <v>1176</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="24">
-      <c r="F19" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="G19" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="H19" s="10" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="26">
-      <c r="F20" s="44" t="s">
-        <v>1179</v>
-      </c>
-      <c r="G20" s="44" t="s">
-        <v>1180</v>
-      </c>
-      <c r="H20" s="44"/>
-    </row>
-    <row r="21" spans="1:8" ht="26">
-      <c r="F21" s="44" t="s">
-        <v>1181</v>
-      </c>
-      <c r="G21" s="44" t="s">
-        <v>1182</v>
-      </c>
-      <c r="H21" s="44"/>
-    </row>
-    <row r="22" spans="1:8" ht="26">
-      <c r="F22" s="44" t="s">
-        <v>1183</v>
-      </c>
-      <c r="G22" s="44" t="s">
-        <v>1184</v>
-      </c>
-      <c r="H22" s="44"/>
-    </row>
-    <row r="23" spans="1:8" ht="26">
-      <c r="F23" s="44" t="s">
-        <v>1187</v>
-      </c>
-      <c r="G23" s="44" t="s">
-        <v>1188</v>
-      </c>
-      <c r="H23" s="44"/>
-    </row>
-    <row r="24" spans="1:8" ht="26">
-      <c r="F24" s="44" t="s">
-        <v>1177</v>
-      </c>
-      <c r="G24" s="44" t="s">
-        <v>1178</v>
-      </c>
-      <c r="H24" s="44" t="s">
-        <v>1189</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="26">
-      <c r="F25" s="44" t="s">
-        <v>1190</v>
-      </c>
-      <c r="G25" s="44" t="s">
-        <v>1191</v>
-      </c>
-      <c r="H25" s="44"/>
-    </row>
-    <row r="26" spans="1:8" ht="24">
-      <c r="F26" s="23"/>
-      <c r="G26" s="21"/>
-      <c r="H26" s="21"/>
-    </row>
-    <row r="27" spans="1:8" ht="24">
-      <c r="F27" s="21"/>
-      <c r="G27" s="21"/>
-      <c r="H27" s="21"/>
-    </row>
-    <row r="28" spans="1:8" ht="24">
-      <c r="F28" s="21"/>
-      <c r="G28" s="21"/>
-      <c r="H28" s="21"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F683013-E274-BC4D-AA3D-D4742589A444}">
   <sheetPr codeName="Sheet21"/>
   <dimension ref="A2:C17"/>
@@ -11024,7 +11966,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{350DAC63-F1A9-8847-8991-89A792935208}">
   <sheetPr codeName="Sheet24"/>
   <dimension ref="A2:C18"/>
@@ -11172,7 +12114,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A8189FA-8DE2-CE4D-844B-A846D91C12A6}">
   <sheetPr codeName="Sheet25"/>
   <dimension ref="A1:E16"/>
@@ -11334,228 +12276,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F53271B7-0EAD-D94F-8AA6-BD76BFA13A48}">
-  <sheetPr codeName="Sheet26"/>
-  <dimension ref="A2:C25"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="21"/>
-  <cols>
-    <col min="1" max="1" width="21.625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="1:3" ht="31">
-      <c r="A2" s="19" t="s">
-        <v>501</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="24">
-      <c r="A4" s="28" t="s">
-        <v>77</v>
-      </c>
-      <c r="B4" s="29" t="s">
-        <v>78</v>
-      </c>
-      <c r="C4" s="29" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="24">
-      <c r="A5" s="30" t="s">
-        <v>815</v>
-      </c>
-      <c r="B5" s="31" t="s">
-        <v>816</v>
-      </c>
-      <c r="C5" s="12"/>
-    </row>
-    <row r="6" spans="1:3" ht="24">
-      <c r="A6" s="13" t="s">
-        <v>504</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>505</v>
-      </c>
-      <c r="C6" s="32"/>
-    </row>
-    <row r="7" spans="1:3" ht="24">
-      <c r="A7" s="13" t="s">
-        <v>506</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>507</v>
-      </c>
-      <c r="C7" s="14"/>
-    </row>
-    <row r="8" spans="1:3" ht="24">
-      <c r="A8" s="13" t="s">
-        <v>508</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>509</v>
-      </c>
-      <c r="C8" s="14"/>
-    </row>
-    <row r="9" spans="1:3" ht="24">
-      <c r="A9" s="13" t="s">
-        <v>809</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>810</v>
-      </c>
-      <c r="C9" s="14"/>
-    </row>
-    <row r="10" spans="1:3" ht="24">
-      <c r="A10" s="13" t="s">
-        <v>510</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>511</v>
-      </c>
-      <c r="C10" s="14"/>
-    </row>
-    <row r="11" spans="1:3" ht="24">
-      <c r="A11" s="13" t="s">
-        <v>811</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>812</v>
-      </c>
-      <c r="C11" s="14"/>
-    </row>
-    <row r="12" spans="1:3" ht="24">
-      <c r="A12" s="13" t="s">
-        <v>512</v>
-      </c>
-      <c r="B12" s="14" t="s">
-        <v>513</v>
-      </c>
-      <c r="C12" s="14"/>
-    </row>
-    <row r="13" spans="1:3" ht="24">
-      <c r="A13" s="14" t="s">
-        <v>817</v>
-      </c>
-      <c r="B13" s="14" t="s">
-        <v>819</v>
-      </c>
-      <c r="C13" s="14"/>
-    </row>
-    <row r="14" spans="1:3" ht="24">
-      <c r="A14" s="14" t="s">
-        <v>818</v>
-      </c>
-      <c r="B14" s="14" t="s">
-        <v>820</v>
-      </c>
-      <c r="C14" s="14"/>
-    </row>
-    <row r="15" spans="1:3" ht="24">
-      <c r="A15" s="13" t="s">
-        <v>514</v>
-      </c>
-      <c r="B15" s="14" t="s">
-        <v>515</v>
-      </c>
-      <c r="C15" s="14"/>
-    </row>
-    <row r="16" spans="1:3" ht="24">
-      <c r="A16" s="13" t="s">
-        <v>516</v>
-      </c>
-      <c r="B16" s="14" t="s">
-        <v>517</v>
-      </c>
-      <c r="C16" s="14"/>
-    </row>
-    <row r="17" spans="1:3" ht="24">
-      <c r="A17" s="13" t="s">
-        <v>518</v>
-      </c>
-      <c r="B17" s="14" t="s">
-        <v>519</v>
-      </c>
-      <c r="C17" s="14"/>
-    </row>
-    <row r="18" spans="1:3" ht="24">
-      <c r="A18" s="13" t="s">
-        <v>520</v>
-      </c>
-      <c r="B18" s="14" t="s">
-        <v>521</v>
-      </c>
-      <c r="C18" s="14"/>
-    </row>
-    <row r="19" spans="1:3" ht="24">
-      <c r="A19" s="30" t="s">
-        <v>805</v>
-      </c>
-      <c r="B19" s="31" t="s">
-        <v>806</v>
-      </c>
-      <c r="C19" s="14"/>
-    </row>
-    <row r="20" spans="1:3" ht="24">
-      <c r="A20" s="13" t="s">
-        <v>807</v>
-      </c>
-      <c r="B20" s="14" t="s">
-        <v>808</v>
-      </c>
-      <c r="C20" s="32"/>
-    </row>
-    <row r="21" spans="1:3" ht="24">
-      <c r="A21" s="13" t="s">
-        <v>813</v>
-      </c>
-      <c r="B21" s="14" t="s">
-        <v>814</v>
-      </c>
-      <c r="C21" s="32"/>
-    </row>
-    <row r="22" spans="1:3" ht="24">
-      <c r="A22" s="13" t="s">
-        <v>1449</v>
-      </c>
-      <c r="B22" s="14" t="s">
-        <v>1448</v>
-      </c>
-      <c r="C22" s="32"/>
-    </row>
-    <row r="23" spans="1:3" ht="24">
-      <c r="A23" s="13" t="s">
-        <v>821</v>
-      </c>
-      <c r="B23" s="14" t="s">
-        <v>822</v>
-      </c>
-      <c r="C23" s="32"/>
-    </row>
-    <row r="24" spans="1:3" ht="24">
-      <c r="A24" s="13" t="s">
-        <v>821</v>
-      </c>
-      <c r="B24" s="14" t="s">
-        <v>822</v>
-      </c>
-      <c r="C24" s="14"/>
-    </row>
-    <row r="25" spans="1:3" ht="24">
-      <c r="A25" s="13" t="s">
-        <v>1451</v>
-      </c>
-      <c r="B25" s="14" t="s">
-        <v>1450</v>
-      </c>
-      <c r="C25" s="14"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1446148E-86CD-C745-8E28-605EED3FB402}">
   <sheetPr codeName="Sheet27"/>
   <dimension ref="A2:D64"/>
@@ -12069,7 +12790,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{515B1972-D3D7-3442-9E74-B079BA9D4035}">
   <sheetPr codeName="Sheet28"/>
   <dimension ref="A2:C38"/>
@@ -12280,6 +13001,108 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7129155C-C3C0-6742-97C5-B521174141C9}">
+  <dimension ref="A2:C17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="21"/>
+  <cols>
+    <col min="1" max="1" width="19.625" customWidth="1"/>
+    <col min="2" max="2" width="17.125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:3" ht="24">
+      <c r="A2" s="64" t="s">
+        <v>1791</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="24">
+      <c r="A5" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="24">
+      <c r="A6" s="21" t="s">
+        <v>1789</v>
+      </c>
+      <c r="B6" s="21" t="s">
+        <v>1790</v>
+      </c>
+      <c r="C6" s="21"/>
+    </row>
+    <row r="7" spans="1:3" ht="24">
+      <c r="A7" s="21" t="s">
+        <v>530</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>1792</v>
+      </c>
+      <c r="C7" s="21"/>
+    </row>
+    <row r="8" spans="1:3" ht="24">
+      <c r="A8" s="21" t="s">
+        <v>1793</v>
+      </c>
+      <c r="B8" s="21" t="s">
+        <v>1794</v>
+      </c>
+      <c r="C8" s="21"/>
+    </row>
+    <row r="9" spans="1:3" ht="24">
+      <c r="A9" s="21"/>
+      <c r="B9" s="21"/>
+      <c r="C9" s="21"/>
+    </row>
+    <row r="10" spans="1:3" ht="24">
+      <c r="A10" s="21"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+    </row>
+    <row r="11" spans="1:3" ht="24">
+      <c r="A11" s="21"/>
+      <c r="B11" s="21"/>
+      <c r="C11" s="21"/>
+    </row>
+    <row r="12" spans="1:3" ht="24">
+      <c r="A12" s="21"/>
+      <c r="B12" s="21"/>
+      <c r="C12" s="21"/>
+    </row>
+    <row r="13" spans="1:3" ht="24">
+      <c r="A13" s="21"/>
+      <c r="B13" s="21"/>
+      <c r="C13" s="21"/>
+    </row>
+    <row r="14" spans="1:3" ht="24">
+      <c r="A14" s="21"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="21"/>
+    </row>
+    <row r="15" spans="1:3" ht="24">
+      <c r="A15" s="21"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
+    </row>
+    <row r="16" spans="1:3" ht="24">
+      <c r="A16" s="21"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="21"/>
+    </row>
+    <row r="17" spans="1:3" ht="24">
+      <c r="A17" s="21"/>
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB36050E-0104-0341-9D1D-396F77732371}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A2:O246"/>
@@ -14320,7 +15143,9 @@
       <c r="C167" s="21"/>
     </row>
     <row r="168" spans="1:3" ht="24">
-      <c r="A168" s="21"/>
+      <c r="A168" s="21" t="s">
+        <v>1788</v>
+      </c>
       <c r="B168" s="21"/>
       <c r="C168" s="21"/>
     </row>
@@ -14723,7 +15548,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68999D53-424B-0B43-BD8A-F8C773239393}">
   <dimension ref="A1:C37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="21"/>
@@ -15042,7 +15867,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{163338F1-8B10-E648-8B00-E5D51E4474AF}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A3:E39"/>
@@ -15266,7 +16091,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E34B8B3C-4FB9-F34F-BE43-E919C8031462}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A2:T143"/>
@@ -16703,7 +17528,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{986BFAB8-2551-5F4B-8E86-4BE2D8B7FB94}">
   <sheetPr codeName="Sheet22"/>
   <dimension ref="A2:E20"/>
@@ -16920,7 +17745,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA7AA6E8-CA82-4143-AC8B-E58D08BD738E}">
   <sheetPr codeName="Sheet23"/>
   <dimension ref="A2:K31"/>
@@ -17497,572 +18322,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD9AAA77-1A26-CF4D-855B-50339A62BDBB}">
-  <sheetPr codeName="Sheet5"/>
-  <dimension ref="A1:H26"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="39.75" defaultRowHeight="21"/>
-  <cols>
-    <col min="1" max="1" width="14.25" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.75" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="37.125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="37.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.875" customWidth="1"/>
-    <col min="8" max="8" width="37.375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" ht="25">
-      <c r="A1" s="50" t="s">
-        <v>77</v>
-      </c>
-      <c r="B1" s="51" t="s">
-        <v>78</v>
-      </c>
-      <c r="C1" s="51" t="s">
-        <v>77</v>
-      </c>
-      <c r="D1" s="51" t="s">
-        <v>78</v>
-      </c>
-      <c r="E1" s="51" t="s">
-        <v>77</v>
-      </c>
-      <c r="F1" s="51" t="s">
-        <v>78</v>
-      </c>
-      <c r="G1" s="52"/>
-      <c r="H1" s="52"/>
-    </row>
-    <row r="2" spans="1:8" ht="25">
-      <c r="A2" s="53" t="s">
-        <v>1599</v>
-      </c>
-      <c r="B2" s="54" t="s">
-        <v>1600</v>
-      </c>
-      <c r="C2" s="54" t="s">
-        <v>283</v>
-      </c>
-      <c r="D2" s="54" t="s">
-        <v>284</v>
-      </c>
-      <c r="E2" s="54" t="s">
-        <v>281</v>
-      </c>
-      <c r="F2" s="54" t="s">
-        <v>282</v>
-      </c>
-      <c r="G2" s="52"/>
-      <c r="H2" s="52"/>
-    </row>
-    <row r="3" spans="1:8" ht="50">
-      <c r="A3" s="53" t="s">
-        <v>1601</v>
-      </c>
-      <c r="B3" s="54" t="s">
-        <v>1602</v>
-      </c>
-      <c r="C3" s="54" t="s">
-        <v>1603</v>
-      </c>
-      <c r="D3" s="54" t="s">
-        <v>1604</v>
-      </c>
-      <c r="E3" s="54" t="s">
-        <v>1605</v>
-      </c>
-      <c r="F3" s="54" t="s">
-        <v>1602</v>
-      </c>
-      <c r="G3" s="52"/>
-      <c r="H3" s="55" t="s">
-        <v>1606</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="25">
-      <c r="A4" s="53" t="s">
-        <v>1607</v>
-      </c>
-      <c r="B4" s="54" t="s">
-        <v>1608</v>
-      </c>
-      <c r="C4" s="54" t="s">
-        <v>1609</v>
-      </c>
-      <c r="D4" s="54" t="s">
-        <v>1610</v>
-      </c>
-      <c r="E4" s="54" t="s">
-        <v>1611</v>
-      </c>
-      <c r="F4" s="54" t="s">
-        <v>1612</v>
-      </c>
-      <c r="G4" s="52"/>
-      <c r="H4" s="52"/>
-    </row>
-    <row r="5" spans="1:8" ht="25">
-      <c r="A5" s="53" t="s">
-        <v>1613</v>
-      </c>
-      <c r="B5" s="54" t="s">
-        <v>1614</v>
-      </c>
-      <c r="C5" s="54" t="s">
-        <v>1615</v>
-      </c>
-      <c r="D5" s="54" t="s">
-        <v>1616</v>
-      </c>
-      <c r="E5" s="54" t="s">
-        <v>1617</v>
-      </c>
-      <c r="F5" s="54" t="s">
-        <v>1618</v>
-      </c>
-      <c r="G5" s="52"/>
-      <c r="H5" s="52"/>
-    </row>
-    <row r="6" spans="1:8" ht="25">
-      <c r="A6" s="53" t="s">
-        <v>1619</v>
-      </c>
-      <c r="B6" s="54" t="s">
-        <v>1620</v>
-      </c>
-      <c r="C6" s="54" t="s">
-        <v>1621</v>
-      </c>
-      <c r="D6" s="54" t="s">
-        <v>1622</v>
-      </c>
-      <c r="E6" s="54" t="s">
-        <v>1623</v>
-      </c>
-      <c r="F6" s="54" t="s">
-        <v>1624</v>
-      </c>
-      <c r="G6" s="52"/>
-      <c r="H6" s="52"/>
-    </row>
-    <row r="7" spans="1:8" ht="25">
-      <c r="A7" s="53" t="s">
-        <v>1625</v>
-      </c>
-      <c r="B7" s="54" t="s">
-        <v>1626</v>
-      </c>
-      <c r="C7" s="54" t="s">
-        <v>1627</v>
-      </c>
-      <c r="D7" s="54" t="s">
-        <v>1628</v>
-      </c>
-      <c r="E7" s="56"/>
-      <c r="F7" s="56"/>
-      <c r="G7" s="52"/>
-      <c r="H7" s="52"/>
-    </row>
-    <row r="8" spans="1:8" ht="25">
-      <c r="A8" s="53" t="s">
-        <v>1629</v>
-      </c>
-      <c r="B8" s="54" t="s">
-        <v>1630</v>
-      </c>
-      <c r="C8" s="54" t="s">
-        <v>1631</v>
-      </c>
-      <c r="D8" s="54" t="s">
-        <v>1632</v>
-      </c>
-      <c r="E8" s="54" t="s">
-        <v>1633</v>
-      </c>
-      <c r="F8" s="54" t="s">
-        <v>1634</v>
-      </c>
-      <c r="G8" s="52"/>
-      <c r="H8" s="52"/>
-    </row>
-    <row r="9" spans="1:8" ht="50">
-      <c r="A9" s="53" t="s">
-        <v>1635</v>
-      </c>
-      <c r="B9" s="54" t="s">
-        <v>1636</v>
-      </c>
-      <c r="C9" s="54" t="s">
-        <v>1637</v>
-      </c>
-      <c r="D9" s="54" t="s">
-        <v>1638</v>
-      </c>
-      <c r="E9" s="56"/>
-      <c r="F9" s="56"/>
-      <c r="G9" s="52"/>
-      <c r="H9" s="52"/>
-    </row>
-    <row r="10" spans="1:8" ht="25">
-      <c r="A10" s="53" t="s">
-        <v>1639</v>
-      </c>
-      <c r="B10" s="54" t="s">
-        <v>1640</v>
-      </c>
-      <c r="C10" s="54" t="s">
-        <v>1641</v>
-      </c>
-      <c r="D10" s="54" t="s">
-        <v>1642</v>
-      </c>
-      <c r="E10" s="56"/>
-      <c r="F10" s="56"/>
-      <c r="G10" s="52"/>
-      <c r="H10" s="52"/>
-    </row>
-    <row r="11" spans="1:8" ht="25">
-      <c r="A11" s="53" t="s">
-        <v>1643</v>
-      </c>
-      <c r="B11" s="54" t="s">
-        <v>1644</v>
-      </c>
-      <c r="C11" s="54" t="s">
-        <v>1470</v>
-      </c>
-      <c r="D11" s="54" t="s">
-        <v>1645</v>
-      </c>
-      <c r="E11" s="54" t="s">
-        <v>1646</v>
-      </c>
-      <c r="F11" s="54" t="s">
-        <v>1647</v>
-      </c>
-      <c r="G11" s="52"/>
-      <c r="H11" s="52"/>
-    </row>
-    <row r="12" spans="1:8" ht="25">
-      <c r="A12" s="53" t="s">
-        <v>1648</v>
-      </c>
-      <c r="B12" s="54" t="s">
-        <v>1649</v>
-      </c>
-      <c r="C12" s="54" t="s">
-        <v>1650</v>
-      </c>
-      <c r="D12" s="54" t="s">
-        <v>1651</v>
-      </c>
-      <c r="E12" s="54" t="s">
-        <v>1652</v>
-      </c>
-      <c r="F12" s="54" t="s">
-        <v>1653</v>
-      </c>
-      <c r="G12" s="52"/>
-      <c r="H12" s="52"/>
-    </row>
-    <row r="13" spans="1:8" ht="25">
-      <c r="A13" s="53" t="s">
-        <v>1654</v>
-      </c>
-      <c r="B13" s="54" t="s">
-        <v>1655</v>
-      </c>
-      <c r="C13" s="54" t="s">
-        <v>1491</v>
-      </c>
-      <c r="D13" s="54" t="s">
-        <v>1492</v>
-      </c>
-      <c r="E13" s="54" t="s">
-        <v>1493</v>
-      </c>
-      <c r="F13" s="54" t="s">
-        <v>1463</v>
-      </c>
-      <c r="G13" s="52"/>
-      <c r="H13" s="52"/>
-    </row>
-    <row r="14" spans="1:8" ht="25">
-      <c r="A14" s="53" t="s">
-        <v>1656</v>
-      </c>
-      <c r="B14" s="54" t="s">
-        <v>1497</v>
-      </c>
-      <c r="C14" s="54" t="s">
-        <v>1657</v>
-      </c>
-      <c r="D14" s="54" t="s">
-        <v>1658</v>
-      </c>
-      <c r="E14" s="54" t="s">
-        <v>1659</v>
-      </c>
-      <c r="F14" s="54" t="s">
-        <v>1660</v>
-      </c>
-      <c r="G14" s="52"/>
-      <c r="H14" s="52"/>
-    </row>
-    <row r="15" spans="1:8" ht="25">
-      <c r="A15" s="53" t="s">
-        <v>1661</v>
-      </c>
-      <c r="B15" s="54" t="s">
-        <v>1662</v>
-      </c>
-      <c r="C15" s="54" t="s">
-        <v>1663</v>
-      </c>
-      <c r="D15" s="54" t="s">
-        <v>1664</v>
-      </c>
-      <c r="E15" s="54" t="s">
-        <v>1665</v>
-      </c>
-      <c r="F15" s="54" t="s">
-        <v>1666</v>
-      </c>
-      <c r="G15" s="52"/>
-      <c r="H15" s="52"/>
-    </row>
-    <row r="16" spans="1:8" ht="25">
-      <c r="A16" s="53" t="s">
-        <v>1667</v>
-      </c>
-      <c r="B16" s="54" t="s">
-        <v>1513</v>
-      </c>
-      <c r="C16" s="54" t="s">
-        <v>1668</v>
-      </c>
-      <c r="D16" s="54" t="s">
-        <v>1668</v>
-      </c>
-      <c r="E16" s="54" t="s">
-        <v>1669</v>
-      </c>
-      <c r="F16" s="54" t="s">
-        <v>1670</v>
-      </c>
-      <c r="G16" s="52"/>
-      <c r="H16" s="52"/>
-    </row>
-    <row r="17" spans="1:8" ht="25">
-      <c r="A17" s="53" t="s">
-        <v>1671</v>
-      </c>
-      <c r="B17" s="54" t="s">
-        <v>336</v>
-      </c>
-      <c r="C17" s="54" t="s">
-        <v>1444</v>
-      </c>
-      <c r="D17" s="54" t="s">
-        <v>1672</v>
-      </c>
-      <c r="E17" s="54" t="s">
-        <v>1673</v>
-      </c>
-      <c r="F17" s="54" t="s">
-        <v>1674</v>
-      </c>
-      <c r="G17" s="52"/>
-      <c r="H17" s="52"/>
-    </row>
-    <row r="18" spans="1:8" ht="25">
-      <c r="A18" s="53" t="s">
-        <v>1675</v>
-      </c>
-      <c r="B18" s="54" t="s">
-        <v>1676</v>
-      </c>
-      <c r="C18" s="54" t="s">
-        <v>1528</v>
-      </c>
-      <c r="D18" s="54" t="s">
-        <v>1677</v>
-      </c>
-      <c r="E18" s="54" t="s">
-        <v>1529</v>
-      </c>
-      <c r="F18" s="54" t="s">
-        <v>1678</v>
-      </c>
-      <c r="G18" s="52"/>
-      <c r="H18" s="52"/>
-    </row>
-    <row r="19" spans="1:8" ht="50">
-      <c r="A19" s="53" t="s">
-        <v>1679</v>
-      </c>
-      <c r="B19" s="54" t="s">
-        <v>1680</v>
-      </c>
-      <c r="C19" s="54" t="s">
-        <v>922</v>
-      </c>
-      <c r="D19" s="54" t="s">
-        <v>1681</v>
-      </c>
-      <c r="E19" s="54" t="s">
-        <v>1682</v>
-      </c>
-      <c r="F19" s="54" t="s">
-        <v>1683</v>
-      </c>
-      <c r="G19" s="52"/>
-      <c r="H19" s="52"/>
-    </row>
-    <row r="20" spans="1:8" ht="50">
-      <c r="A20" s="53" t="s">
-        <v>1684</v>
-      </c>
-      <c r="B20" s="54" t="s">
-        <v>1685</v>
-      </c>
-      <c r="C20" s="54" t="s">
-        <v>1686</v>
-      </c>
-      <c r="D20" s="54" t="s">
-        <v>1687</v>
-      </c>
-      <c r="E20" s="54" t="s">
-        <v>1688</v>
-      </c>
-      <c r="F20" s="54" t="s">
-        <v>1689</v>
-      </c>
-      <c r="G20" s="52"/>
-      <c r="H20" s="52"/>
-    </row>
-    <row r="21" spans="1:8" ht="50">
-      <c r="A21" s="53" t="s">
-        <v>1690</v>
-      </c>
-      <c r="B21" s="54" t="s">
-        <v>1691</v>
-      </c>
-      <c r="C21" s="54" t="s">
-        <v>1692</v>
-      </c>
-      <c r="D21" s="54" t="s">
-        <v>1693</v>
-      </c>
-      <c r="E21" s="54" t="s">
-        <v>1694</v>
-      </c>
-      <c r="F21" s="54" t="s">
-        <v>1695</v>
-      </c>
-      <c r="G21" s="52"/>
-      <c r="H21" s="52"/>
-    </row>
-    <row r="22" spans="1:8" ht="25">
-      <c r="A22" s="53" t="s">
-        <v>1696</v>
-      </c>
-      <c r="B22" s="54" t="s">
-        <v>1544</v>
-      </c>
-      <c r="C22" s="54" t="s">
-        <v>1697</v>
-      </c>
-      <c r="D22" s="54" t="s">
-        <v>1698</v>
-      </c>
-      <c r="E22" s="54" t="s">
-        <v>1699</v>
-      </c>
-      <c r="F22" s="54" t="s">
-        <v>1700</v>
-      </c>
-      <c r="G22" s="52"/>
-      <c r="H22" s="52"/>
-    </row>
-    <row r="23" spans="1:8" ht="25">
-      <c r="A23" s="53" t="s">
-        <v>1701</v>
-      </c>
-      <c r="B23" s="54" t="s">
-        <v>1702</v>
-      </c>
-      <c r="C23" s="54" t="s">
-        <v>1554</v>
-      </c>
-      <c r="D23" s="54" t="s">
-        <v>1703</v>
-      </c>
-      <c r="E23" s="56"/>
-      <c r="F23" s="56"/>
-      <c r="G23" s="52"/>
-      <c r="H23" s="52"/>
-    </row>
-    <row r="24" spans="1:8" ht="25">
-      <c r="A24" s="53" t="s">
-        <v>1704</v>
-      </c>
-      <c r="B24" s="54" t="s">
-        <v>1705</v>
-      </c>
-      <c r="C24" s="54" t="s">
-        <v>1706</v>
-      </c>
-      <c r="D24" s="54" t="s">
-        <v>1707</v>
-      </c>
-      <c r="E24" s="56"/>
-      <c r="F24" s="56"/>
-      <c r="G24" s="52"/>
-      <c r="H24" s="52"/>
-    </row>
-    <row r="25" spans="1:8" ht="25">
-      <c r="A25" s="53" t="s">
-        <v>1708</v>
-      </c>
-      <c r="B25" s="54" t="s">
-        <v>1709</v>
-      </c>
-      <c r="C25" s="54" t="s">
-        <v>1710</v>
-      </c>
-      <c r="D25" s="54" t="s">
-        <v>1711</v>
-      </c>
-      <c r="E25" s="56"/>
-      <c r="F25" s="56"/>
-      <c r="G25" s="52"/>
-      <c r="H25" s="52"/>
-    </row>
-    <row r="26" spans="1:8" ht="25">
-      <c r="A26" s="53" t="s">
-        <v>1712</v>
-      </c>
-      <c r="B26" s="54" t="s">
-        <v>1713</v>
-      </c>
-      <c r="C26" s="54" t="s">
-        <v>1567</v>
-      </c>
-      <c r="D26" s="54" t="s">
-        <v>1714</v>
-      </c>
-      <c r="E26" s="56"/>
-      <c r="F26" s="56"/>
-      <c r="G26" s="52"/>
-      <c r="H26" s="52"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix formatting on animals tasb
Signed-off-by: Connor Graydon <connorj@bully4u.com>
</commit_message>
<xml_diff>
--- a/chinuk_vocab_gold.xlsx
+++ b/chinuk_vocab_gold.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/connor/Work/chinuk_vocab_repo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{748EA4B4-9A5C-6946-BD62-5598C16181A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A70A9281-D2C2-384B-9D44-86C7D1A9D85A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-52180" yWindow="3860" windowWidth="42960" windowHeight="24520" activeTab="17" xr2:uid="{7DFB5DAA-41FE-8F4C-ADA0-7B74441B15D5}"/>
+    <workbookView xWindow="-52180" yWindow="3860" windowWidth="42960" windowHeight="24520" activeTab="7" xr2:uid="{7DFB5DAA-41FE-8F4C-ADA0-7B74441B15D5}"/>
   </bookViews>
   <sheets>
     <sheet name="Grammar" sheetId="33" r:id="rId1"/>
@@ -10017,10 +10017,10 @@
         <v>81</v>
       </c>
       <c r="F22" s="1"/>
-      <c r="G22" s="45" t="s">
+      <c r="G22" s="5" t="s">
         <v>522</v>
       </c>
-      <c r="H22" s="45" t="s">
+      <c r="H22" s="6" t="s">
         <v>523</v>
       </c>
       <c r="I22" s="4"/>

</xml_diff>

<commit_message>
Added numbers to the day/momth tab.
Signed-off-by: Connor Graydon <connorj@bully4u.com>
</commit_message>
<xml_diff>
--- a/chinuk_vocab_gold.xlsx
+++ b/chinuk_vocab_gold.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/connor/Work/chinuk_vocab_repo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A70A9281-D2C2-384B-9D44-86C7D1A9D85A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB92F5D5-F0D3-6440-BA49-D48713C0D36D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-52180" yWindow="3860" windowWidth="42960" windowHeight="24520" activeTab="7" xr2:uid="{7DFB5DAA-41FE-8F4C-ADA0-7B74441B15D5}"/>
+    <workbookView xWindow="-52180" yWindow="3860" windowWidth="42960" windowHeight="24520" activeTab="12" xr2:uid="{7DFB5DAA-41FE-8F4C-ADA0-7B74441B15D5}"/>
   </bookViews>
   <sheets>
     <sheet name="Grammar" sheetId="33" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2187" uniqueCount="1799">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2235" uniqueCount="1844">
   <si>
     <t>tʼsiqʰwaʔ</t>
   </si>
@@ -5468,6 +5468,141 @@
   </si>
   <si>
     <t>Great Blue Heron</t>
+  </si>
+  <si>
+    <t>Numbers</t>
+  </si>
+  <si>
+    <t>ixt</t>
+  </si>
+  <si>
+    <t>one</t>
+  </si>
+  <si>
+    <t>makwst</t>
+  </si>
+  <si>
+    <t>two</t>
+  </si>
+  <si>
+    <t>three</t>
+  </si>
+  <si>
+    <t>four</t>
+  </si>
+  <si>
+    <t>five</t>
+  </si>
+  <si>
+    <t>six</t>
+  </si>
+  <si>
+    <t>seven</t>
+  </si>
+  <si>
+    <t>eight</t>
+  </si>
+  <si>
+    <t>nine</t>
+  </si>
+  <si>
+    <t>ten</t>
+  </si>
+  <si>
+    <t>eleven</t>
+  </si>
+  <si>
+    <t>twelve</t>
+  </si>
+  <si>
+    <t>thirteen</t>
+  </si>
+  <si>
+    <t>fourteen</t>
+  </si>
+  <si>
+    <t>fifteen</t>
+  </si>
+  <si>
+    <t>sixteen</t>
+  </si>
+  <si>
+    <t>seventeen</t>
+  </si>
+  <si>
+    <t>eighteen</t>
+  </si>
+  <si>
+    <t>nineteen</t>
+  </si>
+  <si>
+    <t>twenty</t>
+  </si>
+  <si>
+    <t>one hundred</t>
+  </si>
+  <si>
+    <t>ɬun</t>
+  </si>
+  <si>
+    <t>lakit</t>
+  </si>
+  <si>
+    <t>qwinəm</t>
+  </si>
+  <si>
+    <t>tax̣am</t>
+  </si>
+  <si>
+    <t>sinamakwst</t>
+  </si>
+  <si>
+    <t>stutkin</t>
+  </si>
+  <si>
+    <t>k'wayts</t>
+  </si>
+  <si>
+    <t>taɬlam</t>
+  </si>
+  <si>
+    <t>taɬlam pi ixt</t>
+  </si>
+  <si>
+    <t>taɬlam pi makwst</t>
+  </si>
+  <si>
+    <t>taɬlam pi ɬun</t>
+  </si>
+  <si>
+    <t>taɬlam pi lakit</t>
+  </si>
+  <si>
+    <t>taɬlam pi qwinəm</t>
+  </si>
+  <si>
+    <t>taɬtam pi tax̣am</t>
+  </si>
+  <si>
+    <t>taɬtlam pi sinamawkst</t>
+  </si>
+  <si>
+    <t>taɬlam pi stutkin</t>
+  </si>
+  <si>
+    <t>taɬlam pi k'wayts</t>
+  </si>
+  <si>
+    <t>makwst-taɬlam</t>
+  </si>
+  <si>
+    <t>tak'umunaq</t>
+  </si>
+  <si>
+    <t>makwst-tak'umunaq</t>
+  </si>
+  <si>
+    <t>two hundred</t>
   </si>
 </sst>
 </file>
@@ -5657,7 +5792,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -5834,20 +5969,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -5965,8 +6091,6 @@
     <xf numFmtId="0" fontId="12" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -6331,7 +6455,7 @@
       <c r="B4" s="21" t="s">
         <v>781</v>
       </c>
-      <c r="C4" s="59"/>
+      <c r="C4" s="57"/>
     </row>
     <row r="5" spans="1:3" ht="25">
       <c r="A5" s="13" t="s">
@@ -6340,7 +6464,7 @@
       <c r="B5" s="14" t="s">
         <v>1774</v>
       </c>
-      <c r="C5" s="59" t="s">
+      <c r="C5" s="57" t="s">
         <v>1776</v>
       </c>
     </row>
@@ -6351,7 +6475,7 @@
       <c r="B6" s="14" t="s">
         <v>1772</v>
       </c>
-      <c r="C6" s="59"/>
+      <c r="C6" s="57"/>
     </row>
     <row r="7" spans="1:3" ht="50">
       <c r="A7" s="13" t="s">
@@ -6360,7 +6484,7 @@
       <c r="B7" s="13" t="s">
         <v>1773</v>
       </c>
-      <c r="C7" s="59" t="s">
+      <c r="C7" s="57" t="s">
         <v>1775</v>
       </c>
     </row>
@@ -6371,7 +6495,7 @@
       <c r="B8" s="13" t="s">
         <v>775</v>
       </c>
-      <c r="C8" s="59"/>
+      <c r="C8" s="57"/>
     </row>
     <row r="9" spans="1:3" ht="24">
       <c r="A9" s="21" t="s">
@@ -6380,142 +6504,142 @@
       <c r="B9" s="21" t="s">
         <v>777</v>
       </c>
-      <c r="C9" s="59"/>
+      <c r="C9" s="57"/>
     </row>
     <row r="11" spans="1:3" ht="24">
       <c r="A11" s="13"/>
       <c r="B11" s="14"/>
-      <c r="C11" s="59"/>
+      <c r="C11" s="57"/>
     </row>
     <row r="12" spans="1:3" ht="24">
       <c r="A12" s="13"/>
       <c r="B12" s="14"/>
-      <c r="C12" s="59"/>
+      <c r="C12" s="57"/>
     </row>
     <row r="13" spans="1:3" ht="24">
       <c r="A13" s="13"/>
       <c r="B13" s="14"/>
-      <c r="C13" s="59"/>
+      <c r="C13" s="57"/>
     </row>
     <row r="14" spans="1:3" ht="24">
       <c r="A14" s="13"/>
       <c r="B14" s="21"/>
-      <c r="C14" s="59"/>
+      <c r="C14" s="57"/>
     </row>
     <row r="15" spans="1:3" ht="24">
       <c r="A15" s="13"/>
       <c r="B15" s="14"/>
-      <c r="C15" s="59"/>
+      <c r="C15" s="57"/>
     </row>
     <row r="16" spans="1:3" ht="24">
       <c r="A16" s="13"/>
       <c r="B16" s="14"/>
-      <c r="C16" s="59"/>
+      <c r="C16" s="57"/>
     </row>
     <row r="17" spans="1:3" ht="24">
       <c r="A17" s="13"/>
       <c r="B17" s="14"/>
-      <c r="C17" s="59"/>
+      <c r="C17" s="57"/>
     </row>
     <row r="18" spans="1:3" ht="24">
       <c r="A18" s="13"/>
       <c r="B18" s="14"/>
-      <c r="C18" s="59"/>
+      <c r="C18" s="57"/>
     </row>
     <row r="19" spans="1:3" ht="24">
       <c r="A19" s="13"/>
       <c r="B19" s="14"/>
-      <c r="C19" s="59"/>
+      <c r="C19" s="57"/>
     </row>
     <row r="20" spans="1:3" ht="24">
       <c r="A20" s="13"/>
       <c r="B20" s="14"/>
-      <c r="C20" s="59"/>
+      <c r="C20" s="57"/>
     </row>
     <row r="21" spans="1:3" ht="24">
       <c r="A21" s="13"/>
       <c r="B21" s="14"/>
-      <c r="C21" s="59"/>
+      <c r="C21" s="57"/>
     </row>
     <row r="22" spans="1:3" ht="24">
       <c r="A22" s="13"/>
       <c r="B22" s="14"/>
-      <c r="C22" s="59"/>
+      <c r="C22" s="57"/>
     </row>
     <row r="23" spans="1:3" ht="24">
       <c r="A23" s="13"/>
       <c r="B23" s="14"/>
-      <c r="C23" s="59"/>
+      <c r="C23" s="57"/>
     </row>
     <row r="24" spans="1:3" ht="24">
       <c r="A24" s="13"/>
       <c r="B24" s="14"/>
-      <c r="C24" s="59"/>
+      <c r="C24" s="57"/>
     </row>
     <row r="25" spans="1:3" ht="24">
       <c r="A25" s="13"/>
       <c r="B25" s="14"/>
-      <c r="C25" s="59"/>
+      <c r="C25" s="57"/>
     </row>
     <row r="26" spans="1:3" ht="24">
       <c r="A26" s="13"/>
       <c r="B26" s="14"/>
-      <c r="C26" s="59"/>
+      <c r="C26" s="57"/>
     </row>
     <row r="27" spans="1:3" ht="24">
       <c r="A27" s="13"/>
       <c r="B27" s="14"/>
-      <c r="C27" s="59"/>
+      <c r="C27" s="57"/>
     </row>
     <row r="28" spans="1:3" ht="24">
       <c r="A28" s="13"/>
       <c r="B28" s="14"/>
-      <c r="C28" s="59"/>
+      <c r="C28" s="57"/>
     </row>
     <row r="29" spans="1:3" ht="24">
       <c r="A29" s="13"/>
       <c r="B29" s="14"/>
-      <c r="C29" s="59"/>
+      <c r="C29" s="57"/>
     </row>
     <row r="30" spans="1:3" ht="24">
       <c r="A30" s="13"/>
       <c r="B30" s="14"/>
-      <c r="C30" s="59"/>
+      <c r="C30" s="57"/>
     </row>
     <row r="31" spans="1:3" ht="24">
       <c r="A31" s="13"/>
       <c r="B31" s="14"/>
-      <c r="C31" s="59"/>
+      <c r="C31" s="57"/>
     </row>
     <row r="32" spans="1:3" ht="24">
       <c r="A32" s="13"/>
       <c r="B32" s="14"/>
-      <c r="C32" s="59"/>
+      <c r="C32" s="57"/>
     </row>
     <row r="33" spans="1:3" ht="24">
       <c r="A33" s="13"/>
       <c r="B33" s="14"/>
-      <c r="C33" s="59"/>
+      <c r="C33" s="57"/>
     </row>
     <row r="34" spans="1:3" ht="24">
       <c r="A34" s="13"/>
       <c r="B34" s="14"/>
-      <c r="C34" s="59"/>
+      <c r="C34" s="57"/>
     </row>
     <row r="35" spans="1:3" ht="24">
       <c r="A35" s="13"/>
       <c r="B35" s="14"/>
-      <c r="C35" s="59"/>
+      <c r="C35" s="57"/>
     </row>
     <row r="36" spans="1:3" ht="24">
       <c r="A36" s="13"/>
       <c r="B36" s="14"/>
-      <c r="C36" s="59"/>
+      <c r="C36" s="57"/>
     </row>
     <row r="37" spans="1:3" ht="24">
       <c r="A37" s="13"/>
       <c r="B37" s="14"/>
-      <c r="C37" s="59"/>
+      <c r="C37" s="57"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7451,20 +7575,28 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F67C7AAB-967B-5045-BDCA-9F7B04711E90}">
   <sheetPr codeName="Sheet7"/>
-  <dimension ref="A3:C29"/>
+  <dimension ref="A3:G29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="21"/>
   <cols>
     <col min="1" max="1" width="23.25" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="6.625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.75" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:3" ht="31">
+    <row r="3" spans="1:7" ht="31">
       <c r="A3" s="19" t="s">
         <v>728</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="24">
+      <c r="E3" s="19" t="s">
+        <v>1799</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="31">
+      <c r="E4" s="19"/>
+    </row>
+    <row r="5" spans="1:7" ht="24">
       <c r="A5" s="11" t="s">
         <v>77</v>
       </c>
@@ -7474,8 +7606,17 @@
       <c r="C5" s="12" t="s">
         <v>457</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="24">
+      <c r="E5" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="24">
       <c r="A6" s="21" t="s">
         <v>729</v>
       </c>
@@ -7483,8 +7624,15 @@
         <v>736</v>
       </c>
       <c r="C6" s="21"/>
-    </row>
-    <row r="7" spans="1:3" ht="24">
+      <c r="E6" s="21" t="s">
+        <v>1800</v>
+      </c>
+      <c r="F6" s="21" t="s">
+        <v>1801</v>
+      </c>
+      <c r="G6" s="21"/>
+    </row>
+    <row r="7" spans="1:7" ht="24">
       <c r="A7" s="21" t="s">
         <v>730</v>
       </c>
@@ -7492,8 +7640,15 @@
         <v>737</v>
       </c>
       <c r="C7" s="21"/>
-    </row>
-    <row r="8" spans="1:3" ht="24">
+      <c r="E7" s="21" t="s">
+        <v>1802</v>
+      </c>
+      <c r="F7" s="21" t="s">
+        <v>1803</v>
+      </c>
+      <c r="G7" s="21"/>
+    </row>
+    <row r="8" spans="1:7" ht="24">
       <c r="A8" s="21" t="s">
         <v>731</v>
       </c>
@@ -7501,8 +7656,15 @@
         <v>738</v>
       </c>
       <c r="C8" s="21"/>
-    </row>
-    <row r="9" spans="1:3" ht="24">
+      <c r="E8" s="21" t="s">
+        <v>1823</v>
+      </c>
+      <c r="F8" s="21" t="s">
+        <v>1804</v>
+      </c>
+      <c r="G8" s="21"/>
+    </row>
+    <row r="9" spans="1:7" ht="24">
       <c r="A9" s="21" t="s">
         <v>732</v>
       </c>
@@ -7510,8 +7672,15 @@
         <v>739</v>
       </c>
       <c r="C9" s="21"/>
-    </row>
-    <row r="10" spans="1:3" ht="24">
+      <c r="E9" s="21" t="s">
+        <v>1824</v>
+      </c>
+      <c r="F9" s="21" t="s">
+        <v>1805</v>
+      </c>
+      <c r="G9" s="21"/>
+    </row>
+    <row r="10" spans="1:7" ht="24">
       <c r="A10" s="21" t="s">
         <v>733</v>
       </c>
@@ -7519,8 +7688,15 @@
         <v>740</v>
       </c>
       <c r="C10" s="21"/>
-    </row>
-    <row r="11" spans="1:3" ht="24">
+      <c r="E10" s="21" t="s">
+        <v>1825</v>
+      </c>
+      <c r="F10" s="21" t="s">
+        <v>1806</v>
+      </c>
+      <c r="G10" s="21"/>
+    </row>
+    <row r="11" spans="1:7" ht="24">
       <c r="A11" s="21" t="s">
         <v>734</v>
       </c>
@@ -7528,8 +7704,15 @@
         <v>741</v>
       </c>
       <c r="C11" s="21"/>
-    </row>
-    <row r="12" spans="1:3" ht="24">
+      <c r="E11" s="21" t="s">
+        <v>1826</v>
+      </c>
+      <c r="F11" s="21" t="s">
+        <v>1807</v>
+      </c>
+      <c r="G11" s="21"/>
+    </row>
+    <row r="12" spans="1:7" ht="24">
       <c r="A12" s="21" t="s">
         <v>735</v>
       </c>
@@ -7537,13 +7720,54 @@
         <v>742</v>
       </c>
       <c r="C12" s="21"/>
-    </row>
-    <row r="15" spans="1:3" ht="31">
+      <c r="E12" s="21" t="s">
+        <v>1827</v>
+      </c>
+      <c r="F12" s="21" t="s">
+        <v>1808</v>
+      </c>
+      <c r="G12" s="21"/>
+    </row>
+    <row r="13" spans="1:7" ht="24">
+      <c r="E13" s="21" t="s">
+        <v>1828</v>
+      </c>
+      <c r="F13" s="21" t="s">
+        <v>1809</v>
+      </c>
+      <c r="G13" s="21"/>
+    </row>
+    <row r="14" spans="1:7" ht="24">
+      <c r="E14" s="21" t="s">
+        <v>1829</v>
+      </c>
+      <c r="F14" s="21" t="s">
+        <v>1810</v>
+      </c>
+      <c r="G14" s="21"/>
+    </row>
+    <row r="15" spans="1:7" ht="31">
       <c r="A15" s="19" t="s">
         <v>963</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" ht="24">
+      <c r="E15" s="21" t="s">
+        <v>1830</v>
+      </c>
+      <c r="F15" s="21" t="s">
+        <v>1811</v>
+      </c>
+      <c r="G15" s="21"/>
+    </row>
+    <row r="16" spans="1:7" ht="24">
+      <c r="E16" s="21" t="s">
+        <v>1831</v>
+      </c>
+      <c r="F16" s="21" t="s">
+        <v>1812</v>
+      </c>
+      <c r="G16" s="21"/>
+    </row>
+    <row r="17" spans="1:7" ht="24">
       <c r="A17" s="11" t="s">
         <v>77</v>
       </c>
@@ -7553,8 +7777,15 @@
       <c r="C17" s="12" t="s">
         <v>457</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" ht="24">
+      <c r="E17" s="21" t="s">
+        <v>1832</v>
+      </c>
+      <c r="F17" s="21" t="s">
+        <v>1813</v>
+      </c>
+      <c r="G17" s="21"/>
+    </row>
+    <row r="18" spans="1:7" ht="24">
       <c r="A18" s="21" t="s">
         <v>964</v>
       </c>
@@ -7562,8 +7793,15 @@
         <v>976</v>
       </c>
       <c r="C18" s="21"/>
-    </row>
-    <row r="19" spans="1:3" ht="24">
+      <c r="E18" s="21" t="s">
+        <v>1833</v>
+      </c>
+      <c r="F18" s="21" t="s">
+        <v>1814</v>
+      </c>
+      <c r="G18" s="21"/>
+    </row>
+    <row r="19" spans="1:7" ht="24">
       <c r="A19" s="21" t="s">
         <v>965</v>
       </c>
@@ -7571,8 +7809,15 @@
         <v>977</v>
       </c>
       <c r="C19" s="21"/>
-    </row>
-    <row r="20" spans="1:3" ht="24">
+      <c r="E19" s="21" t="s">
+        <v>1834</v>
+      </c>
+      <c r="F19" s="21" t="s">
+        <v>1815</v>
+      </c>
+      <c r="G19" s="21"/>
+    </row>
+    <row r="20" spans="1:7" ht="24">
       <c r="A20" s="21" t="s">
         <v>966</v>
       </c>
@@ -7580,8 +7825,15 @@
         <v>978</v>
       </c>
       <c r="C20" s="21"/>
-    </row>
-    <row r="21" spans="1:3" ht="24">
+      <c r="E20" s="21" t="s">
+        <v>1835</v>
+      </c>
+      <c r="F20" s="21" t="s">
+        <v>1816</v>
+      </c>
+      <c r="G20" s="21"/>
+    </row>
+    <row r="21" spans="1:7" ht="24">
       <c r="A21" s="21" t="s">
         <v>967</v>
       </c>
@@ -7589,8 +7841,15 @@
         <v>979</v>
       </c>
       <c r="C21" s="21"/>
-    </row>
-    <row r="22" spans="1:3" ht="24">
+      <c r="E21" s="21" t="s">
+        <v>1836</v>
+      </c>
+      <c r="F21" s="21" t="s">
+        <v>1817</v>
+      </c>
+      <c r="G21" s="21"/>
+    </row>
+    <row r="22" spans="1:7" ht="24">
       <c r="A22" s="21" t="s">
         <v>968</v>
       </c>
@@ -7598,8 +7857,15 @@
         <v>980</v>
       </c>
       <c r="C22" s="21"/>
-    </row>
-    <row r="23" spans="1:3" ht="24">
+      <c r="E22" s="21" t="s">
+        <v>1837</v>
+      </c>
+      <c r="F22" s="21" t="s">
+        <v>1818</v>
+      </c>
+      <c r="G22" s="21"/>
+    </row>
+    <row r="23" spans="1:7" ht="24">
       <c r="A23" s="21" t="s">
         <v>969</v>
       </c>
@@ -7607,8 +7873,15 @@
         <v>981</v>
       </c>
       <c r="C23" s="21"/>
-    </row>
-    <row r="24" spans="1:3" ht="24">
+      <c r="E23" s="21" t="s">
+        <v>1838</v>
+      </c>
+      <c r="F23" s="21" t="s">
+        <v>1819</v>
+      </c>
+      <c r="G23" s="21"/>
+    </row>
+    <row r="24" spans="1:7" ht="24">
       <c r="A24" s="21" t="s">
         <v>970</v>
       </c>
@@ -7616,8 +7889,15 @@
         <v>982</v>
       </c>
       <c r="C24" s="21"/>
-    </row>
-    <row r="25" spans="1:3" ht="24">
+      <c r="E24" s="21" t="s">
+        <v>1839</v>
+      </c>
+      <c r="F24" s="21" t="s">
+        <v>1820</v>
+      </c>
+      <c r="G24" s="21"/>
+    </row>
+    <row r="25" spans="1:7" ht="24">
       <c r="A25" s="21" t="s">
         <v>971</v>
       </c>
@@ -7625,8 +7905,15 @@
         <v>983</v>
       </c>
       <c r="C25" s="21"/>
-    </row>
-    <row r="26" spans="1:3" ht="24">
+      <c r="E25" s="21" t="s">
+        <v>1840</v>
+      </c>
+      <c r="F25" s="21" t="s">
+        <v>1821</v>
+      </c>
+      <c r="G25" s="21"/>
+    </row>
+    <row r="26" spans="1:7" ht="24">
       <c r="A26" s="21" t="s">
         <v>972</v>
       </c>
@@ -7634,8 +7921,15 @@
         <v>984</v>
       </c>
       <c r="C26" s="21"/>
-    </row>
-    <row r="27" spans="1:3" ht="24">
+      <c r="E26" s="21" t="s">
+        <v>1841</v>
+      </c>
+      <c r="F26" s="21" t="s">
+        <v>1822</v>
+      </c>
+      <c r="G26" s="21"/>
+    </row>
+    <row r="27" spans="1:7" ht="24">
       <c r="A27" s="21" t="s">
         <v>973</v>
       </c>
@@ -7643,8 +7937,15 @@
         <v>985</v>
       </c>
       <c r="C27" s="21"/>
-    </row>
-    <row r="28" spans="1:3" ht="24">
+      <c r="E27" s="21" t="s">
+        <v>1842</v>
+      </c>
+      <c r="F27" s="21" t="s">
+        <v>1843</v>
+      </c>
+      <c r="G27" s="21"/>
+    </row>
+    <row r="28" spans="1:7" ht="24">
       <c r="A28" s="21" t="s">
         <v>974</v>
       </c>
@@ -7653,7 +7954,7 @@
       </c>
       <c r="C28" s="21"/>
     </row>
-    <row r="29" spans="1:3" ht="24">
+    <row r="29" spans="1:7" ht="24">
       <c r="A29" s="21" t="s">
         <v>975</v>
       </c>
@@ -13010,7 +13311,7 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:3" ht="24">
-      <c r="A2" s="64" t="s">
+      <c r="A2" s="62" t="s">
         <v>1791</v>
       </c>
     </row>
@@ -14985,10 +15286,10 @@
       <c r="C149" s="21"/>
     </row>
     <row r="150" spans="1:3" ht="25">
-      <c r="A150" s="62" t="s">
+      <c r="A150" s="60" t="s">
         <v>1587</v>
       </c>
-      <c r="B150" s="62" t="s">
+      <c r="B150" s="60" t="s">
         <v>1588</v>
       </c>
       <c r="C150" s="21"/>
@@ -15123,23 +15424,23 @@
       <c r="A165" s="21" t="s">
         <v>175</v>
       </c>
-      <c r="B165" s="63" t="s">
+      <c r="B165" s="61" t="s">
         <v>176</v>
       </c>
       <c r="C165" s="21"/>
     </row>
     <row r="166" spans="1:3" ht="24">
-      <c r="A166" s="61" t="s">
+      <c r="A166" s="59" t="s">
         <v>174</v>
       </c>
-      <c r="B166" s="61" t="s">
+      <c r="B166" s="59" t="s">
         <v>173</v>
       </c>
       <c r="C166" s="21"/>
     </row>
     <row r="167" spans="1:3" ht="24">
-      <c r="A167" s="60"/>
-      <c r="B167" s="61"/>
+      <c r="A167" s="58"/>
+      <c r="B167" s="59"/>
       <c r="C167" s="21"/>
     </row>
     <row r="168" spans="1:3" ht="24">
@@ -17689,10 +17990,10 @@
       <c r="B15" s="14" t="s">
         <v>455</v>
       </c>
-      <c r="D15" s="57" t="s">
+      <c r="D15" s="13" t="s">
         <v>1766</v>
       </c>
-      <c r="E15" s="58" t="s">
+      <c r="E15" s="13" t="s">
         <v>1767</v>
       </c>
     </row>
@@ -17703,6 +18004,8 @@
       <c r="B16" s="14" t="s">
         <v>450</v>
       </c>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
     </row>
     <row r="17" spans="1:2" ht="24">
       <c r="A17" s="13" t="s">

</xml_diff>

<commit_message>
Commit sticky ass bear story vocabulary
Signed-off-by: Connor Graydon <connorj@bully4u.com>
</commit_message>
<xml_diff>
--- a/chinuk_vocab_gold.xlsx
+++ b/chinuk_vocab_gold.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/connor/Work/chinuk_vocab_repo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB92F5D5-F0D3-6440-BA49-D48713C0D36D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5787A48D-671D-4F45-828B-E22572480B32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-52180" yWindow="3860" windowWidth="42960" windowHeight="24520" activeTab="12" xr2:uid="{7DFB5DAA-41FE-8F4C-ADA0-7B74441B15D5}"/>
+    <workbookView xWindow="-63920" yWindow="3200" windowWidth="34760" windowHeight="24520" activeTab="3" xr2:uid="{7DFB5DAA-41FE-8F4C-ADA0-7B74441B15D5}"/>
   </bookViews>
   <sheets>
     <sheet name="Grammar" sheetId="33" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2235" uniqueCount="1844">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2244" uniqueCount="1848">
   <si>
     <t>tʼsiqʰwaʔ</t>
   </si>
@@ -5437,9 +5437,6 @@
     <t>From pipa5-6_cw103_sp2023.pdf</t>
   </si>
   <si>
-    <t>iləp-pus</t>
-  </si>
-  <si>
     <t>alikʰuchik</t>
   </si>
   <si>
@@ -5603,6 +5600,21 @@
   </si>
   <si>
     <t>two hundred</t>
+  </si>
+  <si>
+    <t>only then</t>
+  </si>
+  <si>
+    <t>hayash-hayu</t>
+  </si>
+  <si>
+    <t>abundant</t>
+  </si>
+  <si>
+    <t>q'wetɬ-kakwa</t>
+  </si>
+  <si>
+    <t>sticky</t>
   </si>
 </sst>
 </file>
@@ -5973,7 +5985,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -6103,6 +6115,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7559,10 +7572,10 @@
     </row>
     <row r="26" spans="1:3" ht="24">
       <c r="A26" s="13" t="s">
+        <v>1794</v>
+      </c>
+      <c r="B26" s="14" t="s">
         <v>1795</v>
-      </c>
-      <c r="B26" s="14" t="s">
-        <v>1796</v>
       </c>
       <c r="C26" s="14"/>
     </row>
@@ -7590,7 +7603,7 @@
         <v>728</v>
       </c>
       <c r="E3" s="19" t="s">
-        <v>1799</v>
+        <v>1798</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="31">
@@ -7625,10 +7638,10 @@
       </c>
       <c r="C6" s="21"/>
       <c r="E6" s="21" t="s">
+        <v>1799</v>
+      </c>
+      <c r="F6" s="21" t="s">
         <v>1800</v>
-      </c>
-      <c r="F6" s="21" t="s">
-        <v>1801</v>
       </c>
       <c r="G6" s="21"/>
     </row>
@@ -7641,10 +7654,10 @@
       </c>
       <c r="C7" s="21"/>
       <c r="E7" s="21" t="s">
+        <v>1801</v>
+      </c>
+      <c r="F7" s="21" t="s">
         <v>1802</v>
-      </c>
-      <c r="F7" s="21" t="s">
-        <v>1803</v>
       </c>
       <c r="G7" s="21"/>
     </row>
@@ -7657,10 +7670,10 @@
       </c>
       <c r="C8" s="21"/>
       <c r="E8" s="21" t="s">
-        <v>1823</v>
+        <v>1822</v>
       </c>
       <c r="F8" s="21" t="s">
-        <v>1804</v>
+        <v>1803</v>
       </c>
       <c r="G8" s="21"/>
     </row>
@@ -7673,10 +7686,10 @@
       </c>
       <c r="C9" s="21"/>
       <c r="E9" s="21" t="s">
-        <v>1824</v>
+        <v>1823</v>
       </c>
       <c r="F9" s="21" t="s">
-        <v>1805</v>
+        <v>1804</v>
       </c>
       <c r="G9" s="21"/>
     </row>
@@ -7689,10 +7702,10 @@
       </c>
       <c r="C10" s="21"/>
       <c r="E10" s="21" t="s">
-        <v>1825</v>
+        <v>1824</v>
       </c>
       <c r="F10" s="21" t="s">
-        <v>1806</v>
+        <v>1805</v>
       </c>
       <c r="G10" s="21"/>
     </row>
@@ -7705,10 +7718,10 @@
       </c>
       <c r="C11" s="21"/>
       <c r="E11" s="21" t="s">
-        <v>1826</v>
+        <v>1825</v>
       </c>
       <c r="F11" s="21" t="s">
-        <v>1807</v>
+        <v>1806</v>
       </c>
       <c r="G11" s="21"/>
     </row>
@@ -7721,28 +7734,28 @@
       </c>
       <c r="C12" s="21"/>
       <c r="E12" s="21" t="s">
-        <v>1827</v>
+        <v>1826</v>
       </c>
       <c r="F12" s="21" t="s">
-        <v>1808</v>
+        <v>1807</v>
       </c>
       <c r="G12" s="21"/>
     </row>
     <row r="13" spans="1:7" ht="24">
       <c r="E13" s="21" t="s">
-        <v>1828</v>
+        <v>1827</v>
       </c>
       <c r="F13" s="21" t="s">
-        <v>1809</v>
+        <v>1808</v>
       </c>
       <c r="G13" s="21"/>
     </row>
     <row r="14" spans="1:7" ht="24">
       <c r="E14" s="21" t="s">
-        <v>1829</v>
+        <v>1828</v>
       </c>
       <c r="F14" s="21" t="s">
-        <v>1810</v>
+        <v>1809</v>
       </c>
       <c r="G14" s="21"/>
     </row>
@@ -7751,19 +7764,19 @@
         <v>963</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>1830</v>
+        <v>1829</v>
       </c>
       <c r="F15" s="21" t="s">
-        <v>1811</v>
+        <v>1810</v>
       </c>
       <c r="G15" s="21"/>
     </row>
     <row r="16" spans="1:7" ht="24">
       <c r="E16" s="21" t="s">
-        <v>1831</v>
+        <v>1830</v>
       </c>
       <c r="F16" s="21" t="s">
-        <v>1812</v>
+        <v>1811</v>
       </c>
       <c r="G16" s="21"/>
     </row>
@@ -7778,10 +7791,10 @@
         <v>457</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>1832</v>
+        <v>1831</v>
       </c>
       <c r="F17" s="21" t="s">
-        <v>1813</v>
+        <v>1812</v>
       </c>
       <c r="G17" s="21"/>
     </row>
@@ -7794,10 +7807,10 @@
       </c>
       <c r="C18" s="21"/>
       <c r="E18" s="21" t="s">
-        <v>1833</v>
+        <v>1832</v>
       </c>
       <c r="F18" s="21" t="s">
-        <v>1814</v>
+        <v>1813</v>
       </c>
       <c r="G18" s="21"/>
     </row>
@@ -7810,10 +7823,10 @@
       </c>
       <c r="C19" s="21"/>
       <c r="E19" s="21" t="s">
-        <v>1834</v>
+        <v>1833</v>
       </c>
       <c r="F19" s="21" t="s">
-        <v>1815</v>
+        <v>1814</v>
       </c>
       <c r="G19" s="21"/>
     </row>
@@ -7826,10 +7839,10 @@
       </c>
       <c r="C20" s="21"/>
       <c r="E20" s="21" t="s">
-        <v>1835</v>
+        <v>1834</v>
       </c>
       <c r="F20" s="21" t="s">
-        <v>1816</v>
+        <v>1815</v>
       </c>
       <c r="G20" s="21"/>
     </row>
@@ -7842,10 +7855,10 @@
       </c>
       <c r="C21" s="21"/>
       <c r="E21" s="21" t="s">
-        <v>1836</v>
+        <v>1835</v>
       </c>
       <c r="F21" s="21" t="s">
-        <v>1817</v>
+        <v>1816</v>
       </c>
       <c r="G21" s="21"/>
     </row>
@@ -7858,10 +7871,10 @@
       </c>
       <c r="C22" s="21"/>
       <c r="E22" s="21" t="s">
-        <v>1837</v>
+        <v>1836</v>
       </c>
       <c r="F22" s="21" t="s">
-        <v>1818</v>
+        <v>1817</v>
       </c>
       <c r="G22" s="21"/>
     </row>
@@ -7874,10 +7887,10 @@
       </c>
       <c r="C23" s="21"/>
       <c r="E23" s="21" t="s">
-        <v>1838</v>
+        <v>1837</v>
       </c>
       <c r="F23" s="21" t="s">
-        <v>1819</v>
+        <v>1818</v>
       </c>
       <c r="G23" s="21"/>
     </row>
@@ -7890,10 +7903,10 @@
       </c>
       <c r="C24" s="21"/>
       <c r="E24" s="21" t="s">
-        <v>1839</v>
+        <v>1838</v>
       </c>
       <c r="F24" s="21" t="s">
-        <v>1820</v>
+        <v>1819</v>
       </c>
       <c r="G24" s="21"/>
     </row>
@@ -7906,10 +7919,10 @@
       </c>
       <c r="C25" s="21"/>
       <c r="E25" s="21" t="s">
-        <v>1840</v>
+        <v>1839</v>
       </c>
       <c r="F25" s="21" t="s">
-        <v>1821</v>
+        <v>1820</v>
       </c>
       <c r="G25" s="21"/>
     </row>
@@ -7922,10 +7935,10 @@
       </c>
       <c r="C26" s="21"/>
       <c r="E26" s="21" t="s">
-        <v>1841</v>
+        <v>1840</v>
       </c>
       <c r="F26" s="21" t="s">
-        <v>1822</v>
+        <v>1821</v>
       </c>
       <c r="G26" s="21"/>
     </row>
@@ -7938,10 +7951,10 @@
       </c>
       <c r="C27" s="21"/>
       <c r="E27" s="21" t="s">
+        <v>1841</v>
+      </c>
+      <c r="F27" s="21" t="s">
         <v>1842</v>
-      </c>
-      <c r="F27" s="21" t="s">
-        <v>1843</v>
       </c>
       <c r="G27" s="21"/>
     </row>
@@ -10236,10 +10249,10 @@
       </c>
       <c r="C20" s="1"/>
       <c r="D20" s="5" t="s">
+        <v>1796</v>
+      </c>
+      <c r="E20" s="5" t="s">
         <v>1797</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>1798</v>
       </c>
       <c r="F20" s="1"/>
       <c r="G20" s="7" t="s">
@@ -13312,7 +13325,7 @@
   <sheetData>
     <row r="2" spans="1:3" ht="24">
       <c r="A2" s="62" t="s">
-        <v>1791</v>
+        <v>1790</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="24">
@@ -13328,10 +13341,10 @@
     </row>
     <row r="6" spans="1:3" ht="24">
       <c r="A6" s="21" t="s">
+        <v>1788</v>
+      </c>
+      <c r="B6" s="21" t="s">
         <v>1789</v>
-      </c>
-      <c r="B6" s="21" t="s">
-        <v>1790</v>
       </c>
       <c r="C6" s="21"/>
     </row>
@@ -13340,16 +13353,16 @@
         <v>530</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>1792</v>
+        <v>1791</v>
       </c>
       <c r="C7" s="21"/>
     </row>
     <row r="8" spans="1:3" ht="24">
       <c r="A8" s="21" t="s">
+        <v>1792</v>
+      </c>
+      <c r="B8" s="21" t="s">
         <v>1793</v>
-      </c>
-      <c r="B8" s="21" t="s">
-        <v>1794</v>
       </c>
       <c r="C8" s="21"/>
     </row>
@@ -13567,10 +13580,10 @@
     </row>
     <row r="12" spans="1:15" ht="24">
       <c r="A12" s="21" t="s">
-        <v>164</v>
+        <v>1734</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>165</v>
+        <v>1722</v>
       </c>
       <c r="C12" s="21"/>
       <c r="D12" s="9"/>
@@ -13588,10 +13601,10 @@
     </row>
     <row r="13" spans="1:15" ht="24">
       <c r="A13" s="21" t="s">
-        <v>782</v>
+        <v>164</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>783</v>
+        <v>165</v>
       </c>
       <c r="C13" s="21"/>
       <c r="E13" s="9"/>
@@ -13608,10 +13621,10 @@
     </row>
     <row r="14" spans="1:15" ht="24">
       <c r="A14" s="21" t="s">
-        <v>406</v>
+        <v>782</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>407</v>
+        <v>783</v>
       </c>
       <c r="C14" s="21"/>
       <c r="E14" s="9"/>
@@ -13628,10 +13641,10 @@
     </row>
     <row r="15" spans="1:15" ht="24">
       <c r="A15" s="21" t="s">
-        <v>854</v>
+        <v>406</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>855</v>
+        <v>407</v>
       </c>
       <c r="C15" s="21"/>
       <c r="E15" s="9"/>
@@ -13648,10 +13661,10 @@
     </row>
     <row r="16" spans="1:15" ht="24">
       <c r="A16" s="21" t="s">
-        <v>801</v>
+        <v>854</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>802</v>
+        <v>855</v>
       </c>
       <c r="C16" s="21"/>
       <c r="E16" s="9"/>
@@ -13668,10 +13681,10 @@
     </row>
     <row r="17" spans="1:15" ht="24">
       <c r="A17" s="21" t="s">
-        <v>770</v>
+        <v>801</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>771</v>
+        <v>802</v>
       </c>
       <c r="C17" s="21"/>
       <c r="E17" s="9"/>
@@ -13688,10 +13701,10 @@
     </row>
     <row r="18" spans="1:15" ht="24">
       <c r="A18" s="21" t="s">
-        <v>1453</v>
+        <v>770</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>1454</v>
+        <v>771</v>
       </c>
       <c r="C18" s="21"/>
       <c r="E18" s="9"/>
@@ -13708,10 +13721,10 @@
     </row>
     <row r="19" spans="1:15" ht="24">
       <c r="A19" s="21" t="s">
-        <v>996</v>
+        <v>1453</v>
       </c>
       <c r="B19" s="21" t="s">
-        <v>997</v>
+        <v>1454</v>
       </c>
       <c r="C19" s="21"/>
       <c r="D19" s="9"/>
@@ -13729,10 +13742,10 @@
     </row>
     <row r="20" spans="1:15" ht="24">
       <c r="A20" s="21" t="s">
-        <v>796</v>
+        <v>996</v>
       </c>
       <c r="B20" s="21" t="s">
-        <v>282</v>
+        <v>997</v>
       </c>
       <c r="C20" s="21"/>
       <c r="E20" s="9"/>
@@ -13749,10 +13762,10 @@
     </row>
     <row r="21" spans="1:15" ht="24">
       <c r="A21" s="21" t="s">
-        <v>990</v>
+        <v>796</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>991</v>
+        <v>282</v>
       </c>
       <c r="C21" s="21"/>
       <c r="D21" s="9"/>
@@ -13768,12 +13781,12 @@
       <c r="N21" s="9"/>
       <c r="O21" s="9"/>
     </row>
-    <row r="22" spans="1:15" ht="25">
-      <c r="A22" s="47" t="s">
-        <v>1573</v>
-      </c>
-      <c r="B22" s="47" t="s">
-        <v>1574</v>
+    <row r="22" spans="1:15" ht="24">
+      <c r="A22" s="21" t="s">
+        <v>990</v>
+      </c>
+      <c r="B22" s="21" t="s">
+        <v>991</v>
       </c>
       <c r="C22" s="21"/>
       <c r="E22" s="9"/>
@@ -13790,10 +13803,10 @@
     </row>
     <row r="23" spans="1:15" ht="25">
       <c r="A23" s="47" t="s">
-        <v>1570</v>
+        <v>1573</v>
       </c>
       <c r="B23" s="47" t="s">
-        <v>1571</v>
+        <v>1574</v>
       </c>
       <c r="C23" s="21"/>
       <c r="D23" s="9"/>
@@ -13809,12 +13822,12 @@
       <c r="N23" s="9"/>
       <c r="O23" s="9"/>
     </row>
-    <row r="24" spans="1:15" ht="24">
-      <c r="A24" s="21" t="s">
-        <v>858</v>
-      </c>
-      <c r="B24" s="21" t="s">
-        <v>859</v>
+    <row r="24" spans="1:15" ht="25">
+      <c r="A24" s="47" t="s">
+        <v>1570</v>
+      </c>
+      <c r="B24" s="47" t="s">
+        <v>1571</v>
       </c>
       <c r="C24" s="21"/>
       <c r="E24" s="9"/>
@@ -13831,10 +13844,10 @@
     </row>
     <row r="25" spans="1:15" ht="24">
       <c r="A25" s="21" t="s">
-        <v>599</v>
+        <v>858</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>600</v>
+        <v>859</v>
       </c>
       <c r="C25" s="21"/>
       <c r="D25" s="9"/>
@@ -13852,10 +13865,10 @@
     </row>
     <row r="26" spans="1:15" ht="24">
       <c r="A26" s="21" t="s">
-        <v>920</v>
+        <v>1844</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>921</v>
+        <v>1845</v>
       </c>
       <c r="C26" s="21"/>
       <c r="E26" s="9"/>
@@ -13872,10 +13885,10 @@
     </row>
     <row r="27" spans="1:15" ht="24">
       <c r="A27" s="21" t="s">
-        <v>1128</v>
+        <v>599</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>1136</v>
+        <v>600</v>
       </c>
       <c r="C27" s="21"/>
       <c r="D27" s="9"/>
@@ -13893,10 +13906,10 @@
     </row>
     <row r="28" spans="1:15" ht="24">
       <c r="A28" s="21" t="s">
-        <v>177</v>
+        <v>920</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>195</v>
+        <v>921</v>
       </c>
       <c r="C28" s="21"/>
       <c r="E28" s="9"/>
@@ -13913,10 +13926,10 @@
     </row>
     <row r="29" spans="1:15" ht="24">
       <c r="A29" s="21" t="s">
-        <v>204</v>
+        <v>1128</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>931</v>
+        <v>1136</v>
       </c>
       <c r="C29" s="21"/>
       <c r="D29" s="9"/>
@@ -13934,10 +13947,10 @@
     </row>
     <row r="30" spans="1:15" ht="24">
       <c r="A30" s="21" t="s">
-        <v>200</v>
+        <v>177</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>218</v>
+        <v>195</v>
       </c>
       <c r="C30" s="21"/>
       <c r="E30" s="9"/>
@@ -13954,10 +13967,10 @@
     </row>
     <row r="31" spans="1:15" ht="24">
       <c r="A31" s="21" t="s">
-        <v>924</v>
+        <v>204</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>925</v>
+        <v>931</v>
       </c>
       <c r="C31" s="21"/>
       <c r="D31" s="9"/>
@@ -13973,12 +13986,12 @@
       <c r="N31" s="9"/>
       <c r="O31" s="9"/>
     </row>
-    <row r="32" spans="1:15" ht="25">
-      <c r="A32" s="47" t="s">
-        <v>1591</v>
-      </c>
-      <c r="B32" s="47" t="s">
-        <v>1592</v>
+    <row r="32" spans="1:15" ht="24">
+      <c r="A32" s="21" t="s">
+        <v>200</v>
+      </c>
+      <c r="B32" s="21" t="s">
+        <v>218</v>
       </c>
       <c r="C32" s="21"/>
       <c r="E32" s="9"/>
@@ -13995,10 +14008,10 @@
     </row>
     <row r="33" spans="1:15" ht="24">
       <c r="A33" s="21" t="s">
-        <v>1163</v>
+        <v>924</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>1164</v>
+        <v>925</v>
       </c>
       <c r="C33" s="21"/>
       <c r="D33" s="9"/>
@@ -14014,12 +14027,12 @@
       <c r="N33" s="9"/>
       <c r="O33" s="9"/>
     </row>
-    <row r="34" spans="1:15" ht="24">
-      <c r="A34" s="21" t="s">
-        <v>178</v>
-      </c>
-      <c r="B34" s="21" t="s">
-        <v>169</v>
+    <row r="34" spans="1:15" ht="25">
+      <c r="A34" s="47" t="s">
+        <v>1591</v>
+      </c>
+      <c r="B34" s="47" t="s">
+        <v>1592</v>
       </c>
       <c r="C34" s="21"/>
       <c r="E34" s="9"/>
@@ -14036,10 +14049,10 @@
     </row>
     <row r="35" spans="1:15" ht="24">
       <c r="A35" s="21" t="s">
-        <v>196</v>
+        <v>1163</v>
       </c>
       <c r="B35" s="21" t="s">
-        <v>197</v>
+        <v>1164</v>
       </c>
       <c r="C35" s="21"/>
       <c r="D35" s="9"/>
@@ -14057,10 +14070,10 @@
     </row>
     <row r="36" spans="1:15" ht="24">
       <c r="A36" s="21" t="s">
-        <v>589</v>
+        <v>178</v>
       </c>
       <c r="B36" s="21" t="s">
-        <v>590</v>
+        <v>169</v>
       </c>
       <c r="C36" s="21"/>
       <c r="E36" s="9"/>
@@ -14077,10 +14090,10 @@
     </row>
     <row r="37" spans="1:15" ht="24">
       <c r="A37" s="21" t="s">
-        <v>578</v>
+        <v>196</v>
       </c>
       <c r="B37" s="21" t="s">
-        <v>579</v>
+        <v>197</v>
       </c>
       <c r="C37" s="21"/>
       <c r="D37" s="9"/>
@@ -14098,21 +14111,19 @@
     </row>
     <row r="38" spans="1:15" ht="25" customHeight="1">
       <c r="A38" s="21" t="s">
-        <v>1137</v>
+        <v>589</v>
       </c>
       <c r="B38" s="21" t="s">
-        <v>1138</v>
-      </c>
-      <c r="C38" s="21" t="s">
-        <v>1139</v>
-      </c>
+        <v>590</v>
+      </c>
+      <c r="C38" s="21"/>
     </row>
     <row r="39" spans="1:15" ht="24">
       <c r="A39" s="21" t="s">
-        <v>247</v>
+        <v>578</v>
       </c>
       <c r="B39" s="21" t="s">
-        <v>248</v>
+        <v>579</v>
       </c>
       <c r="C39" s="21"/>
       <c r="D39" s="9"/>
@@ -14130,12 +14141,14 @@
     </row>
     <row r="40" spans="1:15" ht="24">
       <c r="A40" s="21" t="s">
-        <v>187</v>
+        <v>1137</v>
       </c>
       <c r="B40" s="21" t="s">
-        <v>999</v>
-      </c>
-      <c r="C40" s="21"/>
+        <v>1138</v>
+      </c>
+      <c r="C40" s="21" t="s">
+        <v>1139</v>
+      </c>
       <c r="E40" s="9"/>
       <c r="F40" s="9"/>
       <c r="G40" s="9"/>
@@ -14150,10 +14163,10 @@
     </row>
     <row r="41" spans="1:15" ht="24">
       <c r="A41" s="21" t="s">
-        <v>570</v>
+        <v>247</v>
       </c>
       <c r="B41" s="21" t="s">
-        <v>571</v>
+        <v>248</v>
       </c>
       <c r="C41" s="21"/>
       <c r="E41" s="9"/>
@@ -14170,10 +14183,10 @@
     </row>
     <row r="42" spans="1:15" ht="24">
       <c r="A42" s="21" t="s">
-        <v>1140</v>
+        <v>187</v>
       </c>
       <c r="B42" s="21" t="s">
-        <v>1141</v>
+        <v>999</v>
       </c>
       <c r="C42" s="21"/>
       <c r="D42" s="9"/>
@@ -14191,10 +14204,10 @@
     </row>
     <row r="43" spans="1:15" ht="24">
       <c r="A43" s="21" t="s">
-        <v>183</v>
+        <v>570</v>
       </c>
       <c r="B43" s="21" t="s">
-        <v>182</v>
+        <v>571</v>
       </c>
       <c r="C43" s="21"/>
       <c r="E43" s="9"/>
@@ -14211,14 +14224,12 @@
     </row>
     <row r="44" spans="1:15" ht="24">
       <c r="A44" s="21" t="s">
-        <v>181</v>
+        <v>1140</v>
       </c>
       <c r="B44" s="21" t="s">
-        <v>172</v>
-      </c>
-      <c r="C44" s="21" t="s">
-        <v>234</v>
-      </c>
+        <v>1141</v>
+      </c>
+      <c r="C44" s="21"/>
       <c r="D44" s="9"/>
       <c r="E44" s="9"/>
       <c r="F44" s="9"/>
@@ -14234,10 +14245,10 @@
     </row>
     <row r="45" spans="1:15" ht="24">
       <c r="A45" s="21" t="s">
-        <v>568</v>
+        <v>183</v>
       </c>
       <c r="B45" s="21" t="s">
-        <v>569</v>
+        <v>182</v>
       </c>
       <c r="C45" s="21"/>
       <c r="E45" s="9"/>
@@ -14254,12 +14265,14 @@
     </row>
     <row r="46" spans="1:15" ht="24">
       <c r="A46" s="21" t="s">
-        <v>402</v>
+        <v>181</v>
       </c>
       <c r="B46" s="21" t="s">
-        <v>403</v>
-      </c>
-      <c r="C46" s="21"/>
+        <v>172</v>
+      </c>
+      <c r="C46" s="21" t="s">
+        <v>234</v>
+      </c>
       <c r="D46" s="9"/>
       <c r="E46" s="9"/>
       <c r="F46" s="9"/>
@@ -14275,10 +14288,10 @@
     </row>
     <row r="47" spans="1:15" ht="24">
       <c r="A47" s="21" t="s">
-        <v>722</v>
+        <v>568</v>
       </c>
       <c r="B47" s="21" t="s">
-        <v>723</v>
+        <v>569</v>
       </c>
       <c r="C47" s="21"/>
       <c r="E47" s="9"/>
@@ -14293,12 +14306,12 @@
       <c r="N47" s="9"/>
       <c r="O47" s="9"/>
     </row>
-    <row r="48" spans="1:15" ht="25">
-      <c r="A48" s="47" t="s">
-        <v>1577</v>
-      </c>
-      <c r="B48" s="47" t="s">
-        <v>1578</v>
+    <row r="48" spans="1:15" ht="24">
+      <c r="A48" s="21" t="s">
+        <v>402</v>
+      </c>
+      <c r="B48" s="21" t="s">
+        <v>403</v>
       </c>
       <c r="C48" s="21"/>
       <c r="D48" s="9"/>
@@ -14316,10 +14329,10 @@
     </row>
     <row r="49" spans="1:15" ht="24">
       <c r="A49" s="21" t="s">
-        <v>930</v>
+        <v>722</v>
       </c>
       <c r="B49" s="21" t="s">
-        <v>1328</v>
+        <v>723</v>
       </c>
       <c r="C49" s="21"/>
       <c r="E49" s="9"/>
@@ -14334,12 +14347,12 @@
       <c r="N49" s="9"/>
       <c r="O49" s="9"/>
     </row>
-    <row r="50" spans="1:15" ht="24">
-      <c r="A50" s="21" t="s">
-        <v>188</v>
-      </c>
-      <c r="B50" s="21" t="s">
-        <v>1329</v>
+    <row r="50" spans="1:15" ht="25">
+      <c r="A50" s="47" t="s">
+        <v>1577</v>
+      </c>
+      <c r="B50" s="47" t="s">
+        <v>1578</v>
       </c>
       <c r="C50" s="21"/>
       <c r="E50" s="9"/>
@@ -14356,67 +14369,67 @@
     </row>
     <row r="51" spans="1:15" ht="24">
       <c r="A51" s="21" t="s">
-        <v>1142</v>
+        <v>930</v>
       </c>
       <c r="B51" s="21" t="s">
-        <v>1143</v>
+        <v>1328</v>
       </c>
       <c r="C51" s="21"/>
       <c r="D51" s="9"/>
     </row>
     <row r="52" spans="1:15" ht="24">
       <c r="A52" s="21" t="s">
-        <v>320</v>
+        <v>188</v>
       </c>
       <c r="B52" s="21" t="s">
-        <v>321</v>
+        <v>1329</v>
       </c>
       <c r="C52" s="21"/>
     </row>
     <row r="53" spans="1:15" ht="24">
       <c r="A53" s="21" t="s">
-        <v>780</v>
+        <v>1142</v>
       </c>
       <c r="B53" s="21" t="s">
-        <v>781</v>
+        <v>1143</v>
       </c>
       <c r="C53" s="21"/>
       <c r="D53" s="9"/>
     </row>
     <row r="54" spans="1:15" ht="24">
       <c r="A54" s="21" t="s">
-        <v>776</v>
+        <v>1737</v>
       </c>
       <c r="B54" s="21" t="s">
-        <v>777</v>
+        <v>1843</v>
       </c>
       <c r="C54" s="21"/>
     </row>
     <row r="55" spans="1:15" ht="24">
       <c r="A55" s="21" t="s">
-        <v>1144</v>
+        <v>1736</v>
       </c>
       <c r="B55" s="21" t="s">
-        <v>244</v>
+        <v>1735</v>
       </c>
       <c r="C55" s="21"/>
       <c r="D55" s="9"/>
     </row>
     <row r="56" spans="1:15" ht="24">
       <c r="A56" s="21" t="s">
-        <v>1145</v>
+        <v>320</v>
       </c>
       <c r="B56" s="21" t="s">
-        <v>1146</v>
+        <v>321</v>
       </c>
       <c r="C56" s="21"/>
     </row>
     <row r="57" spans="1:15" ht="24">
       <c r="A57" s="21" t="s">
-        <v>162</v>
+        <v>780</v>
       </c>
       <c r="B57" s="21" t="s">
-        <v>163</v>
+        <v>781</v>
       </c>
       <c r="C57" s="21"/>
       <c r="D57" s="9"/>
@@ -14434,1035 +14447,1053 @@
     </row>
     <row r="58" spans="1:15" ht="24">
       <c r="A58" s="21" t="s">
-        <v>201</v>
+        <v>776</v>
       </c>
       <c r="B58" s="21" t="s">
-        <v>219</v>
+        <v>777</v>
       </c>
       <c r="C58" s="21"/>
     </row>
     <row r="59" spans="1:15" ht="24">
       <c r="A59" s="21" t="s">
-        <v>228</v>
+        <v>1144</v>
       </c>
       <c r="B59" s="21" t="s">
-        <v>229</v>
+        <v>244</v>
       </c>
       <c r="C59" s="21"/>
       <c r="D59" s="9"/>
     </row>
     <row r="60" spans="1:15" ht="24">
       <c r="A60" s="21" t="s">
-        <v>191</v>
+        <v>1145</v>
       </c>
       <c r="B60" s="21" t="s">
-        <v>192</v>
+        <v>1146</v>
       </c>
       <c r="C60" s="21"/>
     </row>
     <row r="61" spans="1:15" ht="24">
       <c r="A61" s="21" t="s">
-        <v>193</v>
+        <v>162</v>
       </c>
       <c r="B61" s="21" t="s">
-        <v>194</v>
+        <v>163</v>
       </c>
       <c r="C61" s="21"/>
       <c r="D61" s="9"/>
     </row>
-    <row r="62" spans="1:15" ht="25">
-      <c r="A62" s="47" t="s">
-        <v>1581</v>
-      </c>
-      <c r="B62" s="47" t="s">
-        <v>1582</v>
+    <row r="62" spans="1:15" ht="24">
+      <c r="A62" s="21" t="s">
+        <v>201</v>
+      </c>
+      <c r="B62" s="21" t="s">
+        <v>219</v>
       </c>
       <c r="C62" s="21"/>
     </row>
     <row r="63" spans="1:15" ht="24">
       <c r="A63" s="21" t="s">
-        <v>794</v>
+        <v>228</v>
       </c>
       <c r="B63" s="21" t="s">
-        <v>795</v>
+        <v>229</v>
       </c>
       <c r="C63" s="21"/>
       <c r="D63" s="9"/>
     </row>
     <row r="64" spans="1:15" ht="24">
       <c r="A64" s="21" t="s">
-        <v>202</v>
+        <v>191</v>
       </c>
       <c r="B64" s="21" t="s">
-        <v>220</v>
+        <v>192</v>
       </c>
       <c r="C64" s="21"/>
     </row>
     <row r="65" spans="1:4" ht="24">
       <c r="A65" s="21" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="B65" s="21" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="C65" s="21"/>
     </row>
-    <row r="66" spans="1:4" ht="24">
-      <c r="A66" s="21" t="s">
-        <v>724</v>
-      </c>
-      <c r="B66" s="21" t="s">
-        <v>725</v>
+    <row r="66" spans="1:4" ht="25">
+      <c r="A66" s="47" t="s">
+        <v>1581</v>
+      </c>
+      <c r="B66" s="47" t="s">
+        <v>1582</v>
       </c>
       <c r="C66" s="21"/>
       <c r="D66" s="9"/>
     </row>
     <row r="67" spans="1:4" ht="24">
       <c r="A67" s="21" t="s">
-        <v>232</v>
+        <v>794</v>
       </c>
       <c r="B67" s="21" t="s">
-        <v>239</v>
+        <v>795</v>
       </c>
       <c r="C67" s="21"/>
     </row>
     <row r="68" spans="1:4" ht="24">
       <c r="A68" s="21" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B68" s="21" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="C68" s="21"/>
       <c r="D68" s="9"/>
     </row>
     <row r="69" spans="1:4" ht="24">
       <c r="A69" s="21" t="s">
-        <v>848</v>
+        <v>189</v>
       </c>
       <c r="B69" s="21" t="s">
-        <v>849</v>
+        <v>190</v>
       </c>
       <c r="C69" s="21"/>
     </row>
-    <row r="70" spans="1:4" ht="25">
-      <c r="A70" s="47" t="s">
-        <v>1583</v>
-      </c>
-      <c r="B70" s="47" t="s">
-        <v>1584</v>
-      </c>
-      <c r="C70" s="23"/>
+    <row r="70" spans="1:4" ht="24">
+      <c r="A70" s="21" t="s">
+        <v>724</v>
+      </c>
+      <c r="B70" s="21" t="s">
+        <v>725</v>
+      </c>
+      <c r="C70" s="21"/>
       <c r="D70" s="9"/>
     </row>
     <row r="71" spans="1:4" ht="24">
       <c r="A71" s="21" t="s">
-        <v>1147</v>
+        <v>232</v>
       </c>
       <c r="B71" s="21" t="s">
-        <v>562</v>
+        <v>239</v>
       </c>
       <c r="C71" s="21"/>
     </row>
     <row r="72" spans="1:4" ht="24">
       <c r="A72" s="21" t="s">
-        <v>856</v>
+        <v>203</v>
       </c>
       <c r="B72" s="21" t="s">
-        <v>857</v>
-      </c>
-      <c r="C72" s="23"/>
+        <v>216</v>
+      </c>
+      <c r="C72" s="21"/>
     </row>
     <row r="73" spans="1:4" ht="24">
       <c r="A73" s="21" t="s">
-        <v>1127</v>
+        <v>848</v>
       </c>
       <c r="B73" s="21" t="s">
-        <v>1126</v>
+        <v>849</v>
       </c>
       <c r="C73" s="21"/>
     </row>
-    <row r="74" spans="1:4" ht="24">
-      <c r="A74" s="21" t="s">
-        <v>1764</v>
-      </c>
-      <c r="B74" s="21" t="s">
-        <v>1765</v>
-      </c>
-      <c r="C74" s="21"/>
+    <row r="74" spans="1:4" ht="25">
+      <c r="A74" s="47" t="s">
+        <v>1583</v>
+      </c>
+      <c r="B74" s="47" t="s">
+        <v>1584</v>
+      </c>
+      <c r="C74" s="23"/>
       <c r="D74" s="9"/>
     </row>
     <row r="75" spans="1:4" ht="24">
       <c r="A75" s="21" t="s">
-        <v>199</v>
+        <v>1147</v>
       </c>
       <c r="B75" s="21" t="s">
-        <v>217</v>
+        <v>562</v>
       </c>
       <c r="C75" s="21"/>
     </row>
     <row r="76" spans="1:4" ht="24">
       <c r="A76" s="21" t="s">
-        <v>1159</v>
+        <v>856</v>
       </c>
       <c r="B76" s="21" t="s">
-        <v>1160</v>
-      </c>
-      <c r="C76" s="21"/>
+        <v>857</v>
+      </c>
+      <c r="C76" s="23"/>
       <c r="D76" s="9"/>
     </row>
     <row r="77" spans="1:4" ht="24">
       <c r="A77" s="21" t="s">
-        <v>249</v>
+        <v>1127</v>
       </c>
       <c r="B77" s="21" t="s">
-        <v>250</v>
+        <v>1126</v>
       </c>
       <c r="C77" s="21"/>
     </row>
     <row r="78" spans="1:4" ht="24">
-      <c r="A78" s="30" t="s">
-        <v>1347</v>
-      </c>
-      <c r="B78" s="30" t="s">
-        <v>1348</v>
+      <c r="A78" s="21" t="s">
+        <v>1764</v>
+      </c>
+      <c r="B78" s="21" t="s">
+        <v>1765</v>
       </c>
       <c r="C78" s="21"/>
     </row>
     <row r="79" spans="1:4" ht="24">
       <c r="A79" s="21" t="s">
-        <v>803</v>
+        <v>199</v>
       </c>
       <c r="B79" s="21" t="s">
-        <v>804</v>
+        <v>217</v>
       </c>
       <c r="C79" s="21"/>
       <c r="D79" s="9"/>
     </row>
     <row r="80" spans="1:4" ht="24">
       <c r="A80" s="21" t="s">
-        <v>798</v>
+        <v>1159</v>
       </c>
       <c r="B80" s="21" t="s">
-        <v>1106</v>
+        <v>1160</v>
       </c>
       <c r="C80" s="21"/>
     </row>
     <row r="81" spans="1:4" ht="24">
       <c r="A81" s="21" t="s">
-        <v>1161</v>
+        <v>249</v>
       </c>
       <c r="B81" s="21" t="s">
-        <v>1162</v>
+        <v>250</v>
       </c>
       <c r="C81" s="21"/>
     </row>
-    <row r="82" spans="1:4" ht="50">
-      <c r="A82" s="47" t="s">
-        <v>1593</v>
-      </c>
-      <c r="B82" s="49" t="s">
-        <v>1594</v>
+    <row r="82" spans="1:4" ht="24">
+      <c r="A82" s="30" t="s">
+        <v>1347</v>
+      </c>
+      <c r="B82" s="30" t="s">
+        <v>1348</v>
       </c>
       <c r="C82" s="21"/>
     </row>
     <row r="83" spans="1:4" ht="24">
       <c r="A83" s="21" t="s">
-        <v>916</v>
+        <v>803</v>
       </c>
       <c r="B83" s="21" t="s">
-        <v>573</v>
+        <v>804</v>
       </c>
       <c r="C83" s="21"/>
       <c r="D83" s="9"/>
     </row>
     <row r="84" spans="1:4" ht="24">
       <c r="A84" s="21" t="s">
-        <v>918</v>
+        <v>798</v>
       </c>
       <c r="B84" s="21" t="s">
-        <v>919</v>
+        <v>1106</v>
       </c>
       <c r="C84" s="21"/>
     </row>
     <row r="85" spans="1:4" ht="24">
       <c r="A85" s="21" t="s">
-        <v>206</v>
+        <v>1161</v>
       </c>
       <c r="B85" s="21" t="s">
-        <v>223</v>
-      </c>
-      <c r="C85" s="21" t="s">
-        <v>917</v>
-      </c>
+        <v>1162</v>
+      </c>
+      <c r="C85" s="21"/>
       <c r="D85" s="9"/>
     </row>
-    <row r="86" spans="1:4" ht="24">
-      <c r="A86" s="21" t="s">
-        <v>799</v>
-      </c>
-      <c r="B86" s="21" t="s">
-        <v>800</v>
+    <row r="86" spans="1:4" ht="50">
+      <c r="A86" s="47" t="s">
+        <v>1593</v>
+      </c>
+      <c r="B86" s="49" t="s">
+        <v>1594</v>
       </c>
       <c r="C86" s="21"/>
     </row>
     <row r="87" spans="1:4" ht="24">
       <c r="A87" s="21" t="s">
-        <v>993</v>
+        <v>916</v>
       </c>
       <c r="B87" s="21" t="s">
-        <v>992</v>
+        <v>573</v>
       </c>
       <c r="C87" s="21"/>
     </row>
-    <row r="88" spans="1:4" ht="25">
-      <c r="A88" s="47" t="s">
-        <v>1579</v>
-      </c>
-      <c r="B88" s="47" t="s">
-        <v>1580</v>
+    <row r="88" spans="1:4" ht="24">
+      <c r="A88" s="21" t="s">
+        <v>918</v>
+      </c>
+      <c r="B88" s="21" t="s">
+        <v>919</v>
       </c>
       <c r="C88" s="21"/>
       <c r="D88" s="9"/>
     </row>
     <row r="89" spans="1:4" ht="24">
       <c r="A89" s="21" t="s">
-        <v>1456</v>
+        <v>206</v>
       </c>
       <c r="B89" s="21" t="s">
-        <v>1457</v>
-      </c>
-      <c r="C89" s="21"/>
+        <v>223</v>
+      </c>
+      <c r="C89" s="21" t="s">
+        <v>917</v>
+      </c>
     </row>
     <row r="90" spans="1:4" ht="24">
       <c r="A90" s="21" t="s">
-        <v>283</v>
+        <v>799</v>
       </c>
       <c r="B90" s="21" t="s">
-        <v>284</v>
+        <v>800</v>
       </c>
       <c r="C90" s="21"/>
       <c r="D90" s="9"/>
     </row>
     <row r="91" spans="1:4" ht="24">
       <c r="A91" s="21" t="s">
-        <v>926</v>
+        <v>993</v>
       </c>
       <c r="B91" s="21" t="s">
-        <v>928</v>
+        <v>992</v>
       </c>
       <c r="C91" s="21"/>
     </row>
-    <row r="92" spans="1:4" ht="24">
-      <c r="A92" s="21" t="s">
-        <v>927</v>
-      </c>
-      <c r="B92" s="21" t="s">
-        <v>929</v>
+    <row r="92" spans="1:4" ht="25">
+      <c r="A92" s="47" t="s">
+        <v>1579</v>
+      </c>
+      <c r="B92" s="47" t="s">
+        <v>1580</v>
       </c>
       <c r="C92" s="21"/>
       <c r="D92" s="9"/>
     </row>
     <row r="93" spans="1:4" ht="24">
       <c r="A93" s="21" t="s">
-        <v>922</v>
+        <v>1456</v>
       </c>
       <c r="B93" s="21" t="s">
-        <v>923</v>
+        <v>1457</v>
       </c>
       <c r="C93" s="21"/>
     </row>
     <row r="94" spans="1:4" ht="24">
       <c r="A94" s="21" t="s">
-        <v>576</v>
+        <v>283</v>
       </c>
       <c r="B94" s="21" t="s">
-        <v>577</v>
+        <v>284</v>
       </c>
       <c r="C94" s="21"/>
       <c r="D94" s="9"/>
     </row>
     <row r="95" spans="1:4" ht="24">
       <c r="A95" s="21" t="s">
-        <v>587</v>
+        <v>926</v>
       </c>
       <c r="B95" s="21" t="s">
-        <v>588</v>
+        <v>928</v>
       </c>
       <c r="C95" s="21"/>
     </row>
     <row r="96" spans="1:4" ht="24">
       <c r="A96" s="21" t="s">
-        <v>335</v>
+        <v>927</v>
       </c>
       <c r="B96" s="21" t="s">
-        <v>242</v>
+        <v>929</v>
       </c>
       <c r="C96" s="21"/>
       <c r="D96" s="9"/>
     </row>
     <row r="97" spans="1:4" ht="24">
       <c r="A97" s="21" t="s">
-        <v>214</v>
+        <v>922</v>
       </c>
       <c r="B97" s="21" t="s">
-        <v>215</v>
+        <v>923</v>
       </c>
       <c r="C97" s="21"/>
     </row>
     <row r="98" spans="1:4" ht="24">
       <c r="A98" s="21" t="s">
-        <v>1324</v>
+        <v>576</v>
       </c>
       <c r="B98" s="21" t="s">
-        <v>1326</v>
-      </c>
-      <c r="C98" s="21" t="s">
-        <v>1327</v>
-      </c>
+        <v>577</v>
+      </c>
+      <c r="C98" s="21"/>
     </row>
     <row r="99" spans="1:4" ht="24">
       <c r="A99" s="21" t="s">
-        <v>592</v>
+        <v>587</v>
       </c>
       <c r="B99" s="21" t="s">
-        <v>593</v>
+        <v>588</v>
       </c>
       <c r="C99" s="21"/>
       <c r="D99" s="9"/>
     </row>
     <row r="100" spans="1:4" ht="24">
       <c r="A100" s="21" t="s">
-        <v>1769</v>
+        <v>335</v>
       </c>
       <c r="B100" s="21" t="s">
-        <v>1770</v>
+        <v>242</v>
       </c>
       <c r="C100" s="21"/>
     </row>
     <row r="101" spans="1:4" ht="24">
       <c r="A101" s="21" t="s">
-        <v>580</v>
+        <v>214</v>
       </c>
       <c r="B101" s="21" t="s">
-        <v>581</v>
+        <v>215</v>
       </c>
       <c r="C101" s="21"/>
       <c r="D101" s="9"/>
     </row>
-    <row r="102" spans="1:4" ht="25">
-      <c r="A102" s="47" t="s">
-        <v>1585</v>
-      </c>
-      <c r="B102" s="47" t="s">
-        <v>1586</v>
-      </c>
-      <c r="C102" s="21"/>
+    <row r="102" spans="1:4" ht="24">
+      <c r="A102" s="21" t="s">
+        <v>1324</v>
+      </c>
+      <c r="B102" s="21" t="s">
+        <v>1326</v>
+      </c>
+      <c r="C102" s="21" t="s">
+        <v>1327</v>
+      </c>
     </row>
     <row r="103" spans="1:4" ht="24">
       <c r="A103" s="21" t="s">
-        <v>852</v>
+        <v>592</v>
       </c>
       <c r="B103" s="21" t="s">
-        <v>853</v>
+        <v>593</v>
       </c>
       <c r="C103" s="21"/>
     </row>
     <row r="104" spans="1:4" ht="24">
       <c r="A104" s="21" t="s">
-        <v>1148</v>
+        <v>1769</v>
       </c>
       <c r="B104" s="21" t="s">
-        <v>1149</v>
+        <v>1770</v>
       </c>
       <c r="C104" s="21"/>
     </row>
     <row r="105" spans="1:4" ht="24">
       <c r="A105" s="21" t="s">
-        <v>720</v>
+        <v>580</v>
       </c>
       <c r="B105" s="21" t="s">
-        <v>721</v>
+        <v>581</v>
       </c>
       <c r="C105" s="21"/>
     </row>
-    <row r="106" spans="1:4" ht="24">
-      <c r="A106" s="21" t="s">
-        <v>230</v>
-      </c>
-      <c r="B106" s="21" t="s">
-        <v>231</v>
+    <row r="106" spans="1:4" ht="25">
+      <c r="A106" s="47" t="s">
+        <v>1585</v>
+      </c>
+      <c r="B106" s="47" t="s">
+        <v>1586</v>
       </c>
       <c r="C106" s="21"/>
     </row>
     <row r="107" spans="1:4" ht="24">
       <c r="A107" s="21" t="s">
-        <v>251</v>
+        <v>852</v>
       </c>
       <c r="B107" s="21" t="s">
-        <v>252</v>
+        <v>853</v>
       </c>
       <c r="C107" s="21"/>
     </row>
     <row r="108" spans="1:4" ht="24">
       <c r="A108" s="21" t="s">
-        <v>208</v>
+        <v>1148</v>
       </c>
       <c r="B108" s="21" t="s">
-        <v>225</v>
+        <v>1149</v>
       </c>
       <c r="C108" s="21"/>
     </row>
     <row r="109" spans="1:4" ht="24">
-      <c r="A109" s="30" t="s">
-        <v>1132</v>
-      </c>
-      <c r="B109" s="30" t="s">
-        <v>677</v>
+      <c r="A109" s="21" t="s">
+        <v>720</v>
+      </c>
+      <c r="B109" s="21" t="s">
+        <v>721</v>
       </c>
       <c r="C109" s="21"/>
     </row>
     <row r="110" spans="1:4" ht="24">
       <c r="A110" s="21" t="s">
-        <v>566</v>
+        <v>230</v>
       </c>
       <c r="B110" s="21" t="s">
-        <v>567</v>
+        <v>231</v>
       </c>
       <c r="C110" s="21"/>
     </row>
     <row r="111" spans="1:4" ht="24">
       <c r="A111" s="21" t="s">
-        <v>1320</v>
+        <v>1846</v>
       </c>
       <c r="B111" s="21" t="s">
-        <v>1321</v>
+        <v>1847</v>
       </c>
       <c r="C111" s="21"/>
     </row>
     <row r="112" spans="1:4" ht="24">
       <c r="A112" s="21" t="s">
-        <v>768</v>
+        <v>251</v>
       </c>
       <c r="B112" s="21" t="s">
-        <v>769</v>
+        <v>252</v>
       </c>
       <c r="C112" s="21"/>
     </row>
     <row r="113" spans="1:4" ht="24">
       <c r="A113" s="21" t="s">
-        <v>988</v>
+        <v>208</v>
       </c>
       <c r="B113" s="21" t="s">
-        <v>989</v>
+        <v>225</v>
       </c>
       <c r="C113" s="21"/>
     </row>
     <row r="114" spans="1:4" ht="24">
-      <c r="A114" s="21" t="s">
-        <v>1165</v>
-      </c>
-      <c r="B114" s="21" t="s">
-        <v>586</v>
+      <c r="A114" s="30" t="s">
+        <v>1132</v>
+      </c>
+      <c r="B114" s="30" t="s">
+        <v>677</v>
       </c>
       <c r="C114" s="21"/>
     </row>
     <row r="115" spans="1:4" ht="24">
       <c r="A115" s="21" t="s">
-        <v>582</v>
+        <v>566</v>
       </c>
       <c r="B115" s="21" t="s">
-        <v>583</v>
+        <v>567</v>
       </c>
       <c r="C115" s="21"/>
     </row>
     <row r="116" spans="1:4" ht="24">
       <c r="A116" s="21" t="s">
-        <v>792</v>
+        <v>1320</v>
       </c>
       <c r="B116" s="21" t="s">
-        <v>793</v>
+        <v>1321</v>
       </c>
       <c r="C116" s="21"/>
       <c r="D116" s="9"/>
     </row>
     <row r="117" spans="1:4" ht="24">
       <c r="A117" s="21" t="s">
-        <v>241</v>
+        <v>768</v>
       </c>
       <c r="B117" s="21" t="s">
-        <v>243</v>
+        <v>769</v>
       </c>
       <c r="C117" s="21"/>
     </row>
     <row r="118" spans="1:4" ht="24">
       <c r="A118" s="21" t="s">
-        <v>1166</v>
+        <v>988</v>
       </c>
       <c r="B118" s="21" t="s">
-        <v>1156</v>
+        <v>989</v>
       </c>
       <c r="C118" s="21"/>
     </row>
     <row r="119" spans="1:4" ht="24">
       <c r="A119" s="21" t="s">
-        <v>313</v>
+        <v>1165</v>
       </c>
       <c r="B119" s="21" t="s">
-        <v>594</v>
+        <v>586</v>
       </c>
       <c r="C119" s="21"/>
     </row>
     <row r="120" spans="1:4" ht="24">
       <c r="A120" s="21" t="s">
-        <v>726</v>
+        <v>582</v>
       </c>
       <c r="B120" s="21" t="s">
-        <v>727</v>
+        <v>583</v>
       </c>
       <c r="C120" s="21"/>
     </row>
     <row r="121" spans="1:4" ht="24">
       <c r="A121" s="21" t="s">
-        <v>207</v>
+        <v>792</v>
       </c>
       <c r="B121" s="21" t="s">
-        <v>224</v>
+        <v>793</v>
       </c>
       <c r="C121" s="21"/>
     </row>
     <row r="122" spans="1:4" ht="24">
       <c r="A122" s="21" t="s">
-        <v>1150</v>
+        <v>241</v>
       </c>
       <c r="B122" s="21" t="s">
-        <v>1151</v>
+        <v>243</v>
       </c>
       <c r="C122" s="21"/>
     </row>
     <row r="123" spans="1:4" ht="24">
       <c r="A123" s="21" t="s">
-        <v>1152</v>
+        <v>1166</v>
       </c>
       <c r="B123" s="21" t="s">
-        <v>1153</v>
+        <v>1156</v>
       </c>
       <c r="C123" s="21"/>
     </row>
     <row r="124" spans="1:4" ht="24">
       <c r="A124" s="21" t="s">
-        <v>1154</v>
+        <v>313</v>
       </c>
       <c r="B124" s="21" t="s">
-        <v>1155</v>
+        <v>594</v>
       </c>
       <c r="C124" s="21"/>
     </row>
     <row r="125" spans="1:4" ht="24">
       <c r="A125" s="21" t="s">
-        <v>597</v>
+        <v>726</v>
       </c>
       <c r="B125" s="21" t="s">
-        <v>598</v>
+        <v>727</v>
       </c>
       <c r="C125" s="21"/>
     </row>
     <row r="126" spans="1:4" ht="24">
       <c r="A126" s="21" t="s">
-        <v>240</v>
+        <v>207</v>
       </c>
       <c r="B126" s="21" t="s">
-        <v>242</v>
+        <v>224</v>
       </c>
       <c r="C126" s="21"/>
     </row>
     <row r="127" spans="1:4" ht="24">
       <c r="A127" s="21" t="s">
-        <v>788</v>
+        <v>1150</v>
       </c>
       <c r="B127" s="21" t="s">
-        <v>789</v>
+        <v>1151</v>
       </c>
       <c r="C127" s="21"/>
     </row>
     <row r="128" spans="1:4" ht="24">
       <c r="A128" s="21" t="s">
-        <v>786</v>
+        <v>1152</v>
       </c>
       <c r="B128" s="21" t="s">
-        <v>787</v>
+        <v>1153</v>
       </c>
       <c r="C128" s="21"/>
     </row>
     <row r="129" spans="1:3" ht="24">
       <c r="A129" s="21" t="s">
-        <v>850</v>
+        <v>1154</v>
       </c>
       <c r="B129" s="21" t="s">
-        <v>851</v>
+        <v>1155</v>
       </c>
       <c r="C129" s="21"/>
     </row>
     <row r="130" spans="1:3" ht="24">
       <c r="A130" s="21" t="s">
-        <v>790</v>
+        <v>597</v>
       </c>
       <c r="B130" s="21" t="s">
-        <v>791</v>
+        <v>598</v>
       </c>
       <c r="C130" s="21"/>
     </row>
     <row r="131" spans="1:3" ht="24">
       <c r="A131" s="21" t="s">
-        <v>574</v>
+        <v>240</v>
       </c>
       <c r="B131" s="21" t="s">
-        <v>575</v>
+        <v>242</v>
       </c>
       <c r="C131" s="21"/>
     </row>
     <row r="132" spans="1:3" ht="24">
       <c r="A132" s="21" t="s">
-        <v>205</v>
+        <v>788</v>
       </c>
       <c r="B132" s="21" t="s">
-        <v>221</v>
-      </c>
-      <c r="C132" s="21" t="s">
-        <v>222</v>
-      </c>
+        <v>789</v>
+      </c>
+      <c r="C132" s="21"/>
     </row>
     <row r="133" spans="1:3" ht="24">
       <c r="A133" s="21" t="s">
-        <v>245</v>
+        <v>786</v>
       </c>
       <c r="B133" s="21" t="s">
-        <v>246</v>
+        <v>787</v>
       </c>
       <c r="C133" s="21"/>
     </row>
-    <row r="134" spans="1:3" ht="25">
-      <c r="A134" s="47" t="s">
-        <v>1575</v>
-      </c>
-      <c r="B134" s="47" t="s">
-        <v>1576</v>
+    <row r="134" spans="1:3" ht="24">
+      <c r="A134" s="21" t="s">
+        <v>850</v>
+      </c>
+      <c r="B134" s="21" t="s">
+        <v>851</v>
       </c>
       <c r="C134" s="21"/>
     </row>
     <row r="135" spans="1:3" ht="24">
       <c r="A135" s="21" t="s">
-        <v>994</v>
+        <v>790</v>
       </c>
       <c r="B135" s="21" t="s">
-        <v>995</v>
+        <v>791</v>
       </c>
       <c r="C135" s="21"/>
     </row>
     <row r="136" spans="1:3" ht="24">
       <c r="A136" s="21" t="s">
-        <v>774</v>
+        <v>574</v>
       </c>
       <c r="B136" s="21" t="s">
-        <v>775</v>
+        <v>575</v>
       </c>
       <c r="C136" s="21"/>
     </row>
     <row r="137" spans="1:3" ht="24">
       <c r="A137" s="21" t="s">
-        <v>584</v>
+        <v>205</v>
       </c>
       <c r="B137" s="21" t="s">
-        <v>585</v>
-      </c>
-      <c r="C137" s="21"/>
-    </row>
-    <row r="138" spans="1:3" ht="25">
-      <c r="A138" s="47" t="s">
-        <v>1589</v>
-      </c>
-      <c r="B138" s="47" t="s">
-        <v>1590</v>
+        <v>221</v>
+      </c>
+      <c r="C137" s="21" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" ht="24">
+      <c r="A138" s="21" t="s">
+        <v>245</v>
+      </c>
+      <c r="B138" s="21" t="s">
+        <v>246</v>
       </c>
       <c r="C138" s="21"/>
     </row>
-    <row r="139" spans="1:3" ht="24">
-      <c r="A139" s="21" t="s">
-        <v>185</v>
-      </c>
-      <c r="B139" s="21" t="s">
-        <v>186</v>
+    <row r="139" spans="1:3" ht="25">
+      <c r="A139" s="47" t="s">
+        <v>1575</v>
+      </c>
+      <c r="B139" s="47" t="s">
+        <v>1576</v>
       </c>
       <c r="C139" s="21"/>
     </row>
     <row r="140" spans="1:3" ht="24">
       <c r="A140" s="21" t="s">
-        <v>226</v>
+        <v>994</v>
       </c>
       <c r="B140" s="21" t="s">
-        <v>227</v>
+        <v>995</v>
       </c>
       <c r="C140" s="21"/>
     </row>
-    <row r="141" spans="1:3" ht="25">
-      <c r="A141" s="47" t="s">
-        <v>1595</v>
-      </c>
-      <c r="B141" s="47" t="s">
-        <v>1596</v>
+    <row r="141" spans="1:3" ht="24">
+      <c r="A141" s="21" t="s">
+        <v>774</v>
+      </c>
+      <c r="B141" s="21" t="s">
+        <v>775</v>
       </c>
       <c r="C141" s="21"/>
     </row>
-    <row r="142" spans="1:3" ht="25">
-      <c r="A142" s="47" t="s">
-        <v>1442</v>
-      </c>
-      <c r="B142" s="47" t="s">
-        <v>1572</v>
+    <row r="142" spans="1:3" ht="24">
+      <c r="A142" s="21" t="s">
+        <v>584</v>
+      </c>
+      <c r="B142" s="21" t="s">
+        <v>585</v>
       </c>
       <c r="C142" s="21"/>
     </row>
-    <row r="143" spans="1:3" ht="24">
-      <c r="A143" s="21" t="s">
-        <v>1325</v>
-      </c>
-      <c r="B143" s="21" t="s">
-        <v>237</v>
+    <row r="143" spans="1:3" ht="25">
+      <c r="A143" s="47" t="s">
+        <v>1589</v>
+      </c>
+      <c r="B143" s="47" t="s">
+        <v>1590</v>
       </c>
       <c r="C143" s="21"/>
     </row>
     <row r="144" spans="1:3" ht="24">
       <c r="A144" s="21" t="s">
-        <v>238</v>
+        <v>185</v>
       </c>
       <c r="B144" s="21" t="s">
-        <v>237</v>
+        <v>186</v>
       </c>
       <c r="C144" s="21"/>
     </row>
     <row r="145" spans="1:3" ht="24">
       <c r="A145" s="21" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
       <c r="B145" s="21" t="s">
-        <v>236</v>
+        <v>227</v>
       </c>
       <c r="C145" s="21"/>
     </row>
-    <row r="146" spans="1:3" ht="24">
-      <c r="A146" s="21" t="s">
-        <v>860</v>
-      </c>
-      <c r="B146" s="21" t="s">
-        <v>861</v>
+    <row r="146" spans="1:3" ht="25">
+      <c r="A146" s="47" t="s">
+        <v>1595</v>
+      </c>
+      <c r="B146" s="47" t="s">
+        <v>1596</v>
       </c>
       <c r="C146" s="21"/>
     </row>
     <row r="147" spans="1:3" ht="25">
       <c r="A147" s="47" t="s">
-        <v>1597</v>
+        <v>1442</v>
       </c>
       <c r="B147" s="47" t="s">
-        <v>1598</v>
+        <v>1572</v>
       </c>
       <c r="C147" s="21"/>
     </row>
     <row r="148" spans="1:3" ht="24">
       <c r="A148" s="21" t="s">
-        <v>784</v>
+        <v>1325</v>
       </c>
       <c r="B148" s="21" t="s">
-        <v>785</v>
+        <v>237</v>
       </c>
       <c r="C148" s="21"/>
     </row>
     <row r="149" spans="1:3" ht="24">
       <c r="A149" s="21" t="s">
-        <v>743</v>
+        <v>238</v>
       </c>
       <c r="B149" s="21" t="s">
-        <v>998</v>
+        <v>237</v>
       </c>
       <c r="C149" s="21"/>
     </row>
-    <row r="150" spans="1:3" ht="25">
-      <c r="A150" s="60" t="s">
-        <v>1587</v>
-      </c>
-      <c r="B150" s="60" t="s">
-        <v>1588</v>
+    <row r="150" spans="1:3" ht="24">
+      <c r="A150" s="48" t="s">
+        <v>235</v>
+      </c>
+      <c r="B150" s="48" t="s">
+        <v>236</v>
       </c>
       <c r="C150" s="21"/>
     </row>
     <row r="151" spans="1:3" ht="24">
       <c r="A151" s="48" t="s">
-        <v>184</v>
+        <v>860</v>
       </c>
       <c r="B151" s="48" t="s">
-        <v>1768</v>
+        <v>861</v>
       </c>
       <c r="C151" s="21"/>
     </row>
-    <row r="152" spans="1:3" ht="24">
-      <c r="A152" s="48" t="s">
-        <v>209</v>
-      </c>
-      <c r="B152" s="48" t="s">
-        <v>210</v>
+    <row r="152" spans="1:3" ht="25">
+      <c r="A152" s="60" t="s">
+        <v>1597</v>
+      </c>
+      <c r="B152" s="60" t="s">
+        <v>1598</v>
       </c>
       <c r="C152" s="21"/>
     </row>
     <row r="153" spans="1:3" ht="24">
       <c r="A153" s="48" t="s">
-        <v>179</v>
+        <v>784</v>
       </c>
       <c r="B153" s="48" t="s">
-        <v>170</v>
+        <v>785</v>
       </c>
       <c r="C153" s="21"/>
     </row>
     <row r="154" spans="1:3" ht="24">
       <c r="A154" s="48" t="s">
-        <v>387</v>
+        <v>743</v>
       </c>
       <c r="B154" s="48" t="s">
-        <v>399</v>
+        <v>998</v>
       </c>
       <c r="C154" s="21"/>
     </row>
-    <row r="155" spans="1:3" ht="24">
-      <c r="A155" s="48" t="s">
-        <v>1167</v>
-      </c>
-      <c r="B155" s="48" t="s">
-        <v>591</v>
+    <row r="155" spans="1:3" ht="25">
+      <c r="A155" s="60" t="s">
+        <v>1587</v>
+      </c>
+      <c r="B155" s="60" t="s">
+        <v>1588</v>
       </c>
       <c r="C155" s="21"/>
     </row>
     <row r="156" spans="1:3" ht="24">
       <c r="A156" s="48" t="s">
-        <v>797</v>
+        <v>184</v>
       </c>
       <c r="B156" s="48" t="s">
-        <v>286</v>
+        <v>1768</v>
       </c>
       <c r="C156" s="21"/>
     </row>
     <row r="157" spans="1:3" ht="24">
       <c r="A157" s="48" t="s">
-        <v>1000</v>
+        <v>209</v>
       </c>
       <c r="B157" s="48" t="s">
-        <v>1001</v>
+        <v>210</v>
       </c>
       <c r="C157" s="21"/>
     </row>
     <row r="158" spans="1:3" ht="24">
       <c r="A158" s="48" t="s">
-        <v>1157</v>
+        <v>179</v>
       </c>
       <c r="B158" s="48" t="s">
-        <v>1158</v>
+        <v>170</v>
       </c>
       <c r="C158" s="21"/>
     </row>
     <row r="159" spans="1:3" ht="24">
       <c r="A159" s="48" t="s">
-        <v>166</v>
+        <v>387</v>
       </c>
       <c r="B159" s="48" t="s">
-        <v>167</v>
+        <v>399</v>
       </c>
       <c r="C159" s="21"/>
     </row>
     <row r="160" spans="1:3" ht="24">
       <c r="A160" s="48" t="s">
-        <v>408</v>
+        <v>1167</v>
       </c>
       <c r="B160" s="48" t="s">
-        <v>719</v>
-      </c>
-      <c r="C160" s="9"/>
+        <v>591</v>
+      </c>
+      <c r="C160" s="63"/>
     </row>
     <row r="161" spans="1:3" ht="24">
       <c r="A161" s="48" t="s">
-        <v>211</v>
+        <v>797</v>
       </c>
       <c r="B161" s="48" t="s">
-        <v>212</v>
+        <v>286</v>
       </c>
       <c r="C161" s="21"/>
     </row>
     <row r="162" spans="1:3" ht="24">
       <c r="A162" s="48" t="s">
-        <v>1105</v>
+        <v>1000</v>
       </c>
       <c r="B162" s="48" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="C162" s="21"/>
     </row>
     <row r="163" spans="1:3" ht="24">
       <c r="A163" s="48" t="s">
-        <v>778</v>
+        <v>1157</v>
       </c>
       <c r="B163" s="48" t="s">
-        <v>779</v>
+        <v>1158</v>
       </c>
       <c r="C163" s="21"/>
     </row>
     <row r="164" spans="1:3" ht="24">
       <c r="A164" s="48" t="s">
-        <v>198</v>
+        <v>166</v>
       </c>
       <c r="B164" s="48" t="s">
-        <v>213</v>
+        <v>167</v>
       </c>
       <c r="C164" s="21"/>
     </row>
     <row r="165" spans="1:3" ht="24">
       <c r="A165" s="21" t="s">
-        <v>175</v>
+        <v>408</v>
       </c>
       <c r="B165" s="61" t="s">
-        <v>176</v>
+        <v>719</v>
       </c>
       <c r="C165" s="21"/>
     </row>
     <row r="166" spans="1:3" ht="24">
       <c r="A166" s="59" t="s">
-        <v>174</v>
+        <v>211</v>
       </c>
       <c r="B166" s="59" t="s">
-        <v>173</v>
+        <v>212</v>
       </c>
       <c r="C166" s="21"/>
     </row>
     <row r="167" spans="1:3" ht="24">
-      <c r="A167" s="58"/>
-      <c r="B167" s="59"/>
+      <c r="A167" s="58" t="s">
+        <v>1105</v>
+      </c>
+      <c r="B167" s="59" t="s">
+        <v>1002</v>
+      </c>
       <c r="C167" s="21"/>
     </row>
     <row r="168" spans="1:3" ht="24">
       <c r="A168" s="21" t="s">
-        <v>1788</v>
-      </c>
-      <c r="B168" s="21"/>
+        <v>778</v>
+      </c>
+      <c r="B168" s="21" t="s">
+        <v>779</v>
+      </c>
       <c r="C168" s="21"/>
     </row>
     <row r="169" spans="1:3" ht="24">
-      <c r="A169" s="21"/>
-      <c r="B169" s="21"/>
+      <c r="A169" s="21" t="s">
+        <v>198</v>
+      </c>
+      <c r="B169" s="21" t="s">
+        <v>213</v>
+      </c>
       <c r="C169" s="21"/>
     </row>
     <row r="170" spans="1:3" ht="24">
-      <c r="A170" s="21"/>
-      <c r="B170" s="21"/>
+      <c r="A170" s="21" t="s">
+        <v>175</v>
+      </c>
+      <c r="B170" s="21" t="s">
+        <v>176</v>
+      </c>
       <c r="C170" s="21"/>
     </row>
     <row r="171" spans="1:3" ht="24">
-      <c r="A171" s="21"/>
-      <c r="B171" s="21"/>
+      <c r="A171" s="21" t="s">
+        <v>174</v>
+      </c>
+      <c r="B171" s="21" t="s">
+        <v>173</v>
+      </c>
       <c r="C171" s="21"/>
     </row>
     <row r="172" spans="1:3" ht="24">
@@ -15841,8 +15872,8 @@
       <c r="C246" s="21"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A5:C167">
-    <sortCondition ref="A167"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A6:C173">
+    <sortCondition ref="A6:A173"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
Resorted Vocab sheet to accommodate new additions.
Signed-off-by: Connor Graydon <connorj@bully4u.com>
</commit_message>
<xml_diff>
--- a/chinuk_vocab_gold.xlsx
+++ b/chinuk_vocab_gold.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/connor/Work/chinuk_vocab_repo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC8F3473-ED31-1E45-A6FF-73A09F9BE15D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2ED5A52-E5BF-B54B-8674-76EC4911C4B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-52500" yWindow="4020" windowWidth="46560" windowHeight="24520" activeTab="3" xr2:uid="{7DFB5DAA-41FE-8F4C-ADA0-7B74441B15D5}"/>
+    <workbookView xWindow="-52500" yWindow="4020" windowWidth="46560" windowHeight="24520" activeTab="2" xr2:uid="{7DFB5DAA-41FE-8F4C-ADA0-7B74441B15D5}"/>
   </bookViews>
   <sheets>
     <sheet name="Grammar" sheetId="33" r:id="rId1"/>
@@ -5848,7 +5848,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -5985,6 +5985,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -14437,10 +14438,10 @@
     </row>
     <row r="31" spans="1:15" ht="24">
       <c r="A31" s="21" t="s">
-        <v>204</v>
+        <v>1787</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>931</v>
+        <v>1788</v>
       </c>
       <c r="C31" s="21"/>
       <c r="D31" s="9"/>
@@ -14458,10 +14459,10 @@
     </row>
     <row r="32" spans="1:15" ht="24">
       <c r="A32" s="21" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="B32" s="21" t="s">
-        <v>218</v>
+        <v>931</v>
       </c>
       <c r="C32" s="21"/>
       <c r="E32" s="9"/>
@@ -14478,10 +14479,10 @@
     </row>
     <row r="33" spans="1:15" ht="24">
       <c r="A33" s="21" t="s">
-        <v>924</v>
+        <v>200</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>925</v>
+        <v>218</v>
       </c>
       <c r="C33" s="21"/>
       <c r="D33" s="9"/>
@@ -14497,12 +14498,12 @@
       <c r="N33" s="9"/>
       <c r="O33" s="9"/>
     </row>
-    <row r="34" spans="1:15" ht="25">
-      <c r="A34" s="47" t="s">
-        <v>1497</v>
-      </c>
-      <c r="B34" s="47" t="s">
-        <v>1498</v>
+    <row r="34" spans="1:15" ht="24">
+      <c r="A34" s="21" t="s">
+        <v>924</v>
+      </c>
+      <c r="B34" s="21" t="s">
+        <v>925</v>
       </c>
       <c r="C34" s="21"/>
       <c r="E34" s="9"/>
@@ -14517,12 +14518,12 @@
       <c r="N34" s="9"/>
       <c r="O34" s="9"/>
     </row>
-    <row r="35" spans="1:15" ht="24">
-      <c r="A35" s="21" t="s">
-        <v>1163</v>
-      </c>
-      <c r="B35" s="21" t="s">
-        <v>1164</v>
+    <row r="35" spans="1:15" ht="25">
+      <c r="A35" s="47" t="s">
+        <v>1497</v>
+      </c>
+      <c r="B35" s="47" t="s">
+        <v>1498</v>
       </c>
       <c r="C35" s="21"/>
       <c r="D35" s="9"/>
@@ -14540,10 +14541,10 @@
     </row>
     <row r="36" spans="1:15" ht="24">
       <c r="A36" s="21" t="s">
-        <v>178</v>
+        <v>1163</v>
       </c>
       <c r="B36" s="21" t="s">
-        <v>169</v>
+        <v>1164</v>
       </c>
       <c r="C36" s="21"/>
       <c r="E36" s="9"/>
@@ -14560,10 +14561,10 @@
     </row>
     <row r="37" spans="1:15" ht="24">
       <c r="A37" s="21" t="s">
-        <v>196</v>
+        <v>178</v>
       </c>
       <c r="B37" s="21" t="s">
-        <v>197</v>
+        <v>169</v>
       </c>
       <c r="C37" s="21"/>
       <c r="D37" s="9"/>
@@ -14581,19 +14582,19 @@
     </row>
     <row r="38" spans="1:15" ht="25" customHeight="1">
       <c r="A38" s="21" t="s">
-        <v>589</v>
+        <v>196</v>
       </c>
       <c r="B38" s="21" t="s">
-        <v>590</v>
+        <v>197</v>
       </c>
       <c r="C38" s="21"/>
     </row>
     <row r="39" spans="1:15" ht="24">
       <c r="A39" s="21" t="s">
-        <v>578</v>
+        <v>589</v>
       </c>
       <c r="B39" s="21" t="s">
-        <v>579</v>
+        <v>590</v>
       </c>
       <c r="C39" s="21"/>
       <c r="D39" s="9"/>
@@ -14611,14 +14612,12 @@
     </row>
     <row r="40" spans="1:15" ht="24">
       <c r="A40" s="21" t="s">
-        <v>1137</v>
+        <v>578</v>
       </c>
       <c r="B40" s="21" t="s">
-        <v>1138</v>
-      </c>
-      <c r="C40" s="21" t="s">
-        <v>1139</v>
-      </c>
+        <v>579</v>
+      </c>
+      <c r="C40" s="21"/>
       <c r="E40" s="9"/>
       <c r="F40" s="9"/>
       <c r="G40" s="9"/>
@@ -14633,10 +14632,10 @@
     </row>
     <row r="41" spans="1:15" ht="24">
       <c r="A41" s="21" t="s">
-        <v>247</v>
+        <v>1792</v>
       </c>
       <c r="B41" s="21" t="s">
-        <v>248</v>
+        <v>680</v>
       </c>
       <c r="C41" s="21"/>
       <c r="E41" s="9"/>
@@ -14653,12 +14652,14 @@
     </row>
     <row r="42" spans="1:15" ht="24">
       <c r="A42" s="21" t="s">
-        <v>187</v>
+        <v>1137</v>
       </c>
       <c r="B42" s="21" t="s">
-        <v>999</v>
-      </c>
-      <c r="C42" s="21"/>
+        <v>1138</v>
+      </c>
+      <c r="C42" s="21" t="s">
+        <v>1139</v>
+      </c>
       <c r="D42" s="9"/>
       <c r="E42" s="9"/>
       <c r="F42" s="9"/>
@@ -14674,10 +14675,10 @@
     </row>
     <row r="43" spans="1:15" ht="24">
       <c r="A43" s="21" t="s">
-        <v>570</v>
+        <v>247</v>
       </c>
       <c r="B43" s="21" t="s">
-        <v>571</v>
+        <v>248</v>
       </c>
       <c r="C43" s="21"/>
       <c r="E43" s="9"/>
@@ -14694,10 +14695,10 @@
     </row>
     <row r="44" spans="1:15" ht="24">
       <c r="A44" s="21" t="s">
-        <v>1140</v>
+        <v>187</v>
       </c>
       <c r="B44" s="21" t="s">
-        <v>1141</v>
+        <v>999</v>
       </c>
       <c r="C44" s="21"/>
       <c r="D44" s="9"/>
@@ -14715,10 +14716,10 @@
     </row>
     <row r="45" spans="1:15" ht="24">
       <c r="A45" s="21" t="s">
-        <v>183</v>
+        <v>570</v>
       </c>
       <c r="B45" s="21" t="s">
-        <v>182</v>
+        <v>571</v>
       </c>
       <c r="C45" s="21"/>
       <c r="E45" s="9"/>
@@ -14735,14 +14736,12 @@
     </row>
     <row r="46" spans="1:15" ht="24">
       <c r="A46" s="21" t="s">
-        <v>181</v>
+        <v>1140</v>
       </c>
       <c r="B46" s="21" t="s">
-        <v>172</v>
-      </c>
-      <c r="C46" s="21" t="s">
-        <v>234</v>
-      </c>
+        <v>1141</v>
+      </c>
+      <c r="C46" s="21"/>
       <c r="D46" s="9"/>
       <c r="E46" s="9"/>
       <c r="F46" s="9"/>
@@ -14758,10 +14757,10 @@
     </row>
     <row r="47" spans="1:15" ht="24">
       <c r="A47" s="21" t="s">
-        <v>568</v>
+        <v>183</v>
       </c>
       <c r="B47" s="21" t="s">
-        <v>569</v>
+        <v>182</v>
       </c>
       <c r="C47" s="21"/>
       <c r="E47" s="9"/>
@@ -14778,12 +14777,14 @@
     </row>
     <row r="48" spans="1:15" ht="24">
       <c r="A48" s="21" t="s">
-        <v>402</v>
+        <v>181</v>
       </c>
       <c r="B48" s="21" t="s">
-        <v>403</v>
-      </c>
-      <c r="C48" s="21"/>
+        <v>172</v>
+      </c>
+      <c r="C48" s="21" t="s">
+        <v>234</v>
+      </c>
       <c r="D48" s="9"/>
       <c r="E48" s="9"/>
       <c r="F48" s="9"/>
@@ -14799,10 +14800,10 @@
     </row>
     <row r="49" spans="1:15" ht="24">
       <c r="A49" s="21" t="s">
-        <v>722</v>
+        <v>568</v>
       </c>
       <c r="B49" s="21" t="s">
-        <v>723</v>
+        <v>569</v>
       </c>
       <c r="C49" s="21"/>
       <c r="E49" s="9"/>
@@ -14817,12 +14818,12 @@
       <c r="N49" s="9"/>
       <c r="O49" s="9"/>
     </row>
-    <row r="50" spans="1:15" ht="25">
-      <c r="A50" s="47" t="s">
-        <v>1483</v>
-      </c>
-      <c r="B50" s="47" t="s">
-        <v>1484</v>
+    <row r="50" spans="1:15" ht="24">
+      <c r="A50" s="21" t="s">
+        <v>402</v>
+      </c>
+      <c r="B50" s="21" t="s">
+        <v>403</v>
       </c>
       <c r="C50" s="21"/>
       <c r="E50" s="9"/>
@@ -14839,67 +14840,67 @@
     </row>
     <row r="51" spans="1:15" ht="24">
       <c r="A51" s="21" t="s">
-        <v>930</v>
+        <v>722</v>
       </c>
       <c r="B51" s="21" t="s">
-        <v>1328</v>
+        <v>723</v>
       </c>
       <c r="C51" s="21"/>
       <c r="D51" s="9"/>
     </row>
-    <row r="52" spans="1:15" ht="24">
-      <c r="A52" s="21" t="s">
-        <v>188</v>
-      </c>
-      <c r="B52" s="21" t="s">
-        <v>1329</v>
+    <row r="52" spans="1:15" ht="25">
+      <c r="A52" s="47" t="s">
+        <v>1483</v>
+      </c>
+      <c r="B52" s="47" t="s">
+        <v>1484</v>
       </c>
       <c r="C52" s="21"/>
     </row>
     <row r="53" spans="1:15" ht="24">
       <c r="A53" s="21" t="s">
-        <v>1142</v>
+        <v>930</v>
       </c>
       <c r="B53" s="21" t="s">
-        <v>1143</v>
+        <v>1328</v>
       </c>
       <c r="C53" s="21"/>
       <c r="D53" s="9"/>
     </row>
     <row r="54" spans="1:15" ht="24">
       <c r="A54" s="21" t="s">
-        <v>1643</v>
+        <v>188</v>
       </c>
       <c r="B54" s="21" t="s">
-        <v>1749</v>
+        <v>1329</v>
       </c>
       <c r="C54" s="21"/>
     </row>
     <row r="55" spans="1:15" ht="24">
       <c r="A55" s="21" t="s">
-        <v>1642</v>
+        <v>1142</v>
       </c>
       <c r="B55" s="21" t="s">
-        <v>1641</v>
+        <v>1143</v>
       </c>
       <c r="C55" s="21"/>
       <c r="D55" s="9"/>
     </row>
     <row r="56" spans="1:15" ht="24">
       <c r="A56" s="21" t="s">
-        <v>320</v>
+        <v>1643</v>
       </c>
       <c r="B56" s="21" t="s">
-        <v>321</v>
+        <v>1749</v>
       </c>
       <c r="C56" s="21"/>
     </row>
     <row r="57" spans="1:15" ht="24">
       <c r="A57" s="21" t="s">
-        <v>780</v>
+        <v>1754</v>
       </c>
       <c r="B57" s="21" t="s">
-        <v>781</v>
+        <v>1755</v>
       </c>
       <c r="C57" s="21"/>
       <c r="D57" s="9"/>
@@ -14917,1112 +14918,1110 @@
     </row>
     <row r="58" spans="1:15" ht="24">
       <c r="A58" s="21" t="s">
-        <v>776</v>
+        <v>1642</v>
       </c>
       <c r="B58" s="21" t="s">
-        <v>777</v>
+        <v>1641</v>
       </c>
       <c r="C58" s="21"/>
     </row>
     <row r="59" spans="1:15" ht="24">
       <c r="A59" s="21" t="s">
-        <v>1144</v>
+        <v>320</v>
       </c>
       <c r="B59" s="21" t="s">
-        <v>244</v>
+        <v>321</v>
       </c>
       <c r="C59" s="21"/>
       <c r="D59" s="9"/>
     </row>
     <row r="60" spans="1:15" ht="24">
       <c r="A60" s="21" t="s">
-        <v>1145</v>
+        <v>780</v>
       </c>
       <c r="B60" s="21" t="s">
-        <v>1146</v>
+        <v>781</v>
       </c>
       <c r="C60" s="21"/>
     </row>
     <row r="61" spans="1:15" ht="24">
       <c r="A61" s="21" t="s">
-        <v>162</v>
+        <v>776</v>
       </c>
       <c r="B61" s="21" t="s">
-        <v>163</v>
+        <v>777</v>
       </c>
       <c r="C61" s="21"/>
       <c r="D61" s="9"/>
     </row>
     <row r="62" spans="1:15" ht="24">
       <c r="A62" s="21" t="s">
-        <v>201</v>
+        <v>1144</v>
       </c>
       <c r="B62" s="21" t="s">
-        <v>219</v>
+        <v>244</v>
       </c>
       <c r="C62" s="21"/>
     </row>
     <row r="63" spans="1:15" ht="24">
       <c r="A63" s="21" t="s">
-        <v>228</v>
+        <v>1145</v>
       </c>
       <c r="B63" s="21" t="s">
-        <v>229</v>
+        <v>1146</v>
       </c>
       <c r="C63" s="21"/>
       <c r="D63" s="9"/>
     </row>
     <row r="64" spans="1:15" ht="24">
       <c r="A64" s="21" t="s">
-        <v>191</v>
+        <v>162</v>
       </c>
       <c r="B64" s="21" t="s">
-        <v>192</v>
+        <v>163</v>
       </c>
       <c r="C64" s="21"/>
     </row>
     <row r="65" spans="1:4" ht="24">
       <c r="A65" s="21" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="B65" s="21" t="s">
-        <v>194</v>
+        <v>219</v>
       </c>
       <c r="C65" s="21"/>
     </row>
-    <row r="66" spans="1:4" ht="25">
-      <c r="A66" s="47" t="s">
-        <v>1487</v>
-      </c>
-      <c r="B66" s="47" t="s">
-        <v>1488</v>
+    <row r="66" spans="1:4" ht="24">
+      <c r="A66" s="21" t="s">
+        <v>228</v>
+      </c>
+      <c r="B66" s="21" t="s">
+        <v>229</v>
       </c>
       <c r="C66" s="21"/>
       <c r="D66" s="9"/>
     </row>
     <row r="67" spans="1:4" ht="24">
       <c r="A67" s="21" t="s">
-        <v>794</v>
+        <v>191</v>
       </c>
       <c r="B67" s="21" t="s">
-        <v>795</v>
+        <v>192</v>
       </c>
       <c r="C67" s="21"/>
     </row>
     <row r="68" spans="1:4" ht="24">
       <c r="A68" s="21" t="s">
-        <v>202</v>
+        <v>193</v>
       </c>
       <c r="B68" s="21" t="s">
-        <v>220</v>
+        <v>194</v>
       </c>
       <c r="C68" s="21"/>
       <c r="D68" s="9"/>
     </row>
-    <row r="69" spans="1:4" ht="24">
-      <c r="A69" s="21" t="s">
-        <v>189</v>
-      </c>
-      <c r="B69" s="21" t="s">
-        <v>190</v>
+    <row r="69" spans="1:4" ht="25">
+      <c r="A69" s="47" t="s">
+        <v>1487</v>
+      </c>
+      <c r="B69" s="47" t="s">
+        <v>1488</v>
       </c>
       <c r="C69" s="21"/>
     </row>
     <row r="70" spans="1:4" ht="24">
       <c r="A70" s="21" t="s">
-        <v>724</v>
+        <v>794</v>
       </c>
       <c r="B70" s="21" t="s">
-        <v>725</v>
+        <v>795</v>
       </c>
       <c r="C70" s="21"/>
       <c r="D70" s="9"/>
     </row>
     <row r="71" spans="1:4" ht="24">
       <c r="A71" s="21" t="s">
-        <v>232</v>
+        <v>202</v>
       </c>
       <c r="B71" s="21" t="s">
-        <v>239</v>
+        <v>220</v>
       </c>
       <c r="C71" s="21"/>
     </row>
     <row r="72" spans="1:4" ht="24">
       <c r="A72" s="21" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="B72" s="21" t="s">
-        <v>216</v>
+        <v>190</v>
       </c>
       <c r="C72" s="21"/>
     </row>
     <row r="73" spans="1:4" ht="24">
       <c r="A73" s="21" t="s">
-        <v>848</v>
+        <v>724</v>
       </c>
       <c r="B73" s="21" t="s">
-        <v>849</v>
+        <v>725</v>
       </c>
       <c r="C73" s="21"/>
     </row>
-    <row r="74" spans="1:4" ht="25">
-      <c r="A74" s="47" t="s">
-        <v>1489</v>
-      </c>
-      <c r="B74" s="47" t="s">
-        <v>1490</v>
-      </c>
-      <c r="C74" s="23"/>
+    <row r="74" spans="1:4" ht="24">
+      <c r="A74" s="21" t="s">
+        <v>232</v>
+      </c>
+      <c r="B74" s="21" t="s">
+        <v>239</v>
+      </c>
+      <c r="C74" s="21"/>
       <c r="D74" s="9"/>
     </row>
     <row r="75" spans="1:4" ht="24">
       <c r="A75" s="21" t="s">
-        <v>1147</v>
+        <v>203</v>
       </c>
       <c r="B75" s="21" t="s">
-        <v>562</v>
+        <v>216</v>
       </c>
       <c r="C75" s="21"/>
     </row>
     <row r="76" spans="1:4" ht="24">
       <c r="A76" s="21" t="s">
-        <v>856</v>
+        <v>848</v>
       </c>
       <c r="B76" s="21" t="s">
-        <v>857</v>
-      </c>
-      <c r="C76" s="23"/>
+        <v>849</v>
+      </c>
+      <c r="C76" s="21"/>
       <c r="D76" s="9"/>
     </row>
     <row r="77" spans="1:4" ht="24">
       <c r="A77" s="21" t="s">
-        <v>1127</v>
+        <v>1789</v>
       </c>
       <c r="B77" s="21" t="s">
-        <v>1126</v>
+        <v>664</v>
       </c>
       <c r="C77" s="21"/>
     </row>
-    <row r="78" spans="1:4" ht="24">
-      <c r="A78" s="21" t="s">
-        <v>1670</v>
-      </c>
-      <c r="B78" s="21" t="s">
-        <v>1671</v>
-      </c>
-      <c r="C78" s="21"/>
+    <row r="78" spans="1:4" ht="25">
+      <c r="A78" s="47" t="s">
+        <v>1489</v>
+      </c>
+      <c r="B78" s="47" t="s">
+        <v>1490</v>
+      </c>
+      <c r="C78" s="23"/>
     </row>
     <row r="79" spans="1:4" ht="24">
       <c r="A79" s="21" t="s">
-        <v>199</v>
+        <v>1790</v>
       </c>
       <c r="B79" s="21" t="s">
-        <v>217</v>
+        <v>672</v>
       </c>
       <c r="C79" s="21"/>
       <c r="D79" s="9"/>
     </row>
     <row r="80" spans="1:4" ht="24">
       <c r="A80" s="21" t="s">
-        <v>1159</v>
+        <v>1147</v>
       </c>
       <c r="B80" s="21" t="s">
-        <v>1160</v>
+        <v>562</v>
       </c>
       <c r="C80" s="21"/>
     </row>
     <row r="81" spans="1:4" ht="24">
       <c r="A81" s="21" t="s">
-        <v>249</v>
+        <v>856</v>
       </c>
       <c r="B81" s="21" t="s">
-        <v>250</v>
-      </c>
-      <c r="C81" s="21"/>
+        <v>857</v>
+      </c>
+      <c r="C81" s="23"/>
     </row>
     <row r="82" spans="1:4" ht="24">
-      <c r="A82" s="30" t="s">
-        <v>1347</v>
-      </c>
-      <c r="B82" s="30" t="s">
-        <v>1348</v>
+      <c r="A82" s="21" t="s">
+        <v>1127</v>
+      </c>
+      <c r="B82" s="21" t="s">
+        <v>1126</v>
       </c>
       <c r="C82" s="21"/>
     </row>
     <row r="83" spans="1:4" ht="24">
       <c r="A83" s="21" t="s">
-        <v>803</v>
+        <v>1670</v>
       </c>
       <c r="B83" s="21" t="s">
-        <v>804</v>
+        <v>1671</v>
       </c>
       <c r="C83" s="21"/>
       <c r="D83" s="9"/>
     </row>
     <row r="84" spans="1:4" ht="24">
       <c r="A84" s="21" t="s">
-        <v>798</v>
+        <v>199</v>
       </c>
       <c r="B84" s="21" t="s">
-        <v>1106</v>
+        <v>217</v>
       </c>
       <c r="C84" s="21"/>
     </row>
     <row r="85" spans="1:4" ht="24">
       <c r="A85" s="21" t="s">
-        <v>1161</v>
+        <v>1159</v>
       </c>
       <c r="B85" s="21" t="s">
-        <v>1162</v>
+        <v>1160</v>
       </c>
       <c r="C85" s="21"/>
       <c r="D85" s="9"/>
     </row>
-    <row r="86" spans="1:4" ht="50">
-      <c r="A86" s="47" t="s">
-        <v>1499</v>
-      </c>
-      <c r="B86" s="49" t="s">
-        <v>1500</v>
+    <row r="86" spans="1:4" ht="24">
+      <c r="A86" s="21" t="s">
+        <v>249</v>
+      </c>
+      <c r="B86" s="21" t="s">
+        <v>250</v>
       </c>
       <c r="C86" s="21"/>
     </row>
     <row r="87" spans="1:4" ht="24">
-      <c r="A87" s="21" t="s">
-        <v>916</v>
-      </c>
-      <c r="B87" s="21" t="s">
-        <v>573</v>
+      <c r="A87" s="30" t="s">
+        <v>1347</v>
+      </c>
+      <c r="B87" s="30" t="s">
+        <v>1348</v>
       </c>
       <c r="C87" s="21"/>
     </row>
     <row r="88" spans="1:4" ht="24">
       <c r="A88" s="21" t="s">
-        <v>918</v>
+        <v>803</v>
       </c>
       <c r="B88" s="21" t="s">
-        <v>919</v>
+        <v>804</v>
       </c>
       <c r="C88" s="21"/>
       <c r="D88" s="9"/>
     </row>
     <row r="89" spans="1:4" ht="24">
       <c r="A89" s="21" t="s">
-        <v>206</v>
+        <v>798</v>
       </c>
       <c r="B89" s="21" t="s">
-        <v>223</v>
-      </c>
-      <c r="C89" s="21" t="s">
-        <v>917</v>
-      </c>
+        <v>1106</v>
+      </c>
+      <c r="C89" s="21"/>
     </row>
     <row r="90" spans="1:4" ht="24">
       <c r="A90" s="21" t="s">
-        <v>799</v>
+        <v>1161</v>
       </c>
       <c r="B90" s="21" t="s">
-        <v>800</v>
+        <v>1162</v>
       </c>
       <c r="C90" s="21"/>
       <c r="D90" s="9"/>
     </row>
-    <row r="91" spans="1:4" ht="24">
-      <c r="A91" s="21" t="s">
-        <v>993</v>
-      </c>
-      <c r="B91" s="21" t="s">
-        <v>992</v>
+    <row r="91" spans="1:4" ht="50">
+      <c r="A91" s="47" t="s">
+        <v>1499</v>
+      </c>
+      <c r="B91" s="49" t="s">
+        <v>1500</v>
       </c>
       <c r="C91" s="21"/>
     </row>
-    <row r="92" spans="1:4" ht="25">
-      <c r="A92" s="47" t="s">
-        <v>1485</v>
-      </c>
-      <c r="B92" s="47" t="s">
-        <v>1486</v>
+    <row r="92" spans="1:4" ht="24">
+      <c r="A92" s="21" t="s">
+        <v>916</v>
+      </c>
+      <c r="B92" s="21" t="s">
+        <v>573</v>
       </c>
       <c r="C92" s="21"/>
       <c r="D92" s="9"/>
     </row>
     <row r="93" spans="1:4" ht="24">
       <c r="A93" s="21" t="s">
-        <v>1456</v>
+        <v>918</v>
       </c>
       <c r="B93" s="21" t="s">
-        <v>1457</v>
+        <v>919</v>
       </c>
       <c r="C93" s="21"/>
     </row>
     <row r="94" spans="1:4" ht="24">
       <c r="A94" s="21" t="s">
-        <v>283</v>
+        <v>206</v>
       </c>
       <c r="B94" s="21" t="s">
-        <v>284</v>
-      </c>
-      <c r="C94" s="21"/>
+        <v>223</v>
+      </c>
+      <c r="C94" s="21" t="s">
+        <v>917</v>
+      </c>
       <c r="D94" s="9"/>
     </row>
     <row r="95" spans="1:4" ht="24">
       <c r="A95" s="21" t="s">
-        <v>926</v>
+        <v>799</v>
       </c>
       <c r="B95" s="21" t="s">
-        <v>928</v>
+        <v>800</v>
       </c>
       <c r="C95" s="21"/>
     </row>
     <row r="96" spans="1:4" ht="24">
       <c r="A96" s="21" t="s">
-        <v>927</v>
+        <v>993</v>
       </c>
       <c r="B96" s="21" t="s">
-        <v>929</v>
+        <v>992</v>
       </c>
       <c r="C96" s="21"/>
       <c r="D96" s="9"/>
     </row>
-    <row r="97" spans="1:4" ht="24">
-      <c r="A97" s="21" t="s">
-        <v>922</v>
-      </c>
-      <c r="B97" s="21" t="s">
-        <v>923</v>
+    <row r="97" spans="1:4" ht="25">
+      <c r="A97" s="47" t="s">
+        <v>1485</v>
+      </c>
+      <c r="B97" s="47" t="s">
+        <v>1486</v>
       </c>
       <c r="C97" s="21"/>
     </row>
     <row r="98" spans="1:4" ht="24">
       <c r="A98" s="21" t="s">
-        <v>576</v>
+        <v>1456</v>
       </c>
       <c r="B98" s="21" t="s">
-        <v>577</v>
+        <v>1457</v>
       </c>
       <c r="C98" s="21"/>
     </row>
     <row r="99" spans="1:4" ht="24">
       <c r="A99" s="21" t="s">
-        <v>587</v>
+        <v>283</v>
       </c>
       <c r="B99" s="21" t="s">
-        <v>588</v>
+        <v>284</v>
       </c>
       <c r="C99" s="21"/>
       <c r="D99" s="9"/>
     </row>
     <row r="100" spans="1:4" ht="24">
       <c r="A100" s="21" t="s">
-        <v>335</v>
+        <v>926</v>
       </c>
       <c r="B100" s="21" t="s">
-        <v>242</v>
+        <v>928</v>
       </c>
       <c r="C100" s="21"/>
     </row>
     <row r="101" spans="1:4" ht="24">
       <c r="A101" s="21" t="s">
-        <v>214</v>
+        <v>927</v>
       </c>
       <c r="B101" s="21" t="s">
-        <v>215</v>
+        <v>929</v>
       </c>
       <c r="C101" s="21"/>
       <c r="D101" s="9"/>
     </row>
     <row r="102" spans="1:4" ht="24">
       <c r="A102" s="21" t="s">
-        <v>1324</v>
+        <v>922</v>
       </c>
       <c r="B102" s="21" t="s">
-        <v>1326</v>
-      </c>
-      <c r="C102" s="21" t="s">
-        <v>1327</v>
-      </c>
+        <v>923</v>
+      </c>
+      <c r="C102" s="21"/>
     </row>
     <row r="103" spans="1:4" ht="24">
       <c r="A103" s="21" t="s">
-        <v>592</v>
+        <v>576</v>
       </c>
       <c r="B103" s="21" t="s">
-        <v>593</v>
+        <v>577</v>
       </c>
       <c r="C103" s="21"/>
     </row>
     <row r="104" spans="1:4" ht="24">
       <c r="A104" s="21" t="s">
-        <v>1675</v>
+        <v>587</v>
       </c>
       <c r="B104" s="21" t="s">
-        <v>1676</v>
+        <v>588</v>
       </c>
       <c r="C104" s="21"/>
     </row>
     <row r="105" spans="1:4" ht="24">
       <c r="A105" s="21" t="s">
-        <v>580</v>
+        <v>335</v>
       </c>
       <c r="B105" s="21" t="s">
-        <v>581</v>
+        <v>242</v>
       </c>
       <c r="C105" s="21"/>
     </row>
-    <row r="106" spans="1:4" ht="25">
-      <c r="A106" s="47" t="s">
-        <v>1491</v>
-      </c>
-      <c r="B106" s="47" t="s">
-        <v>1492</v>
+    <row r="106" spans="1:4" ht="24">
+      <c r="A106" s="21" t="s">
+        <v>214</v>
+      </c>
+      <c r="B106" s="21" t="s">
+        <v>215</v>
       </c>
       <c r="C106" s="21"/>
     </row>
     <row r="107" spans="1:4" ht="24">
       <c r="A107" s="21" t="s">
-        <v>852</v>
+        <v>1324</v>
       </c>
       <c r="B107" s="21" t="s">
-        <v>853</v>
-      </c>
-      <c r="C107" s="21"/>
+        <v>1326</v>
+      </c>
+      <c r="C107" s="21" t="s">
+        <v>1327</v>
+      </c>
     </row>
     <row r="108" spans="1:4" ht="24">
       <c r="A108" s="21" t="s">
-        <v>1148</v>
+        <v>592</v>
       </c>
       <c r="B108" s="21" t="s">
-        <v>1149</v>
+        <v>593</v>
       </c>
       <c r="C108" s="21"/>
     </row>
     <row r="109" spans="1:4" ht="24">
       <c r="A109" s="21" t="s">
-        <v>720</v>
+        <v>1675</v>
       </c>
       <c r="B109" s="21" t="s">
-        <v>721</v>
+        <v>1676</v>
       </c>
       <c r="C109" s="21"/>
     </row>
     <row r="110" spans="1:4" ht="24">
       <c r="A110" s="21" t="s">
-        <v>230</v>
+        <v>580</v>
       </c>
       <c r="B110" s="21" t="s">
-        <v>231</v>
+        <v>581</v>
       </c>
       <c r="C110" s="21"/>
     </row>
-    <row r="111" spans="1:4" ht="24">
-      <c r="A111" s="21" t="s">
-        <v>1752</v>
-      </c>
-      <c r="B111" s="21" t="s">
-        <v>1753</v>
+    <row r="111" spans="1:4" ht="25">
+      <c r="A111" s="47" t="s">
+        <v>1491</v>
+      </c>
+      <c r="B111" s="47" t="s">
+        <v>1492</v>
       </c>
       <c r="C111" s="21"/>
     </row>
     <row r="112" spans="1:4" ht="24">
       <c r="A112" s="21" t="s">
-        <v>251</v>
+        <v>852</v>
       </c>
       <c r="B112" s="21" t="s">
-        <v>252</v>
+        <v>853</v>
       </c>
       <c r="C112" s="21"/>
     </row>
     <row r="113" spans="1:4" ht="24">
       <c r="A113" s="21" t="s">
-        <v>208</v>
+        <v>1148</v>
       </c>
       <c r="B113" s="21" t="s">
-        <v>225</v>
+        <v>1149</v>
       </c>
       <c r="C113" s="21"/>
     </row>
     <row r="114" spans="1:4" ht="24">
-      <c r="A114" s="30" t="s">
-        <v>1132</v>
-      </c>
-      <c r="B114" s="30" t="s">
-        <v>677</v>
+      <c r="A114" s="21" t="s">
+        <v>720</v>
+      </c>
+      <c r="B114" s="21" t="s">
+        <v>721</v>
       </c>
       <c r="C114" s="21"/>
     </row>
     <row r="115" spans="1:4" ht="24">
       <c r="A115" s="21" t="s">
-        <v>566</v>
+        <v>230</v>
       </c>
       <c r="B115" s="21" t="s">
-        <v>567</v>
+        <v>231</v>
       </c>
       <c r="C115" s="21"/>
     </row>
     <row r="116" spans="1:4" ht="24">
       <c r="A116" s="21" t="s">
-        <v>1320</v>
+        <v>1752</v>
       </c>
       <c r="B116" s="21" t="s">
-        <v>1321</v>
+        <v>1753</v>
       </c>
       <c r="C116" s="21"/>
       <c r="D116" s="9"/>
     </row>
     <row r="117" spans="1:4" ht="24">
       <c r="A117" s="21" t="s">
-        <v>768</v>
+        <v>251</v>
       </c>
       <c r="B117" s="21" t="s">
-        <v>769</v>
+        <v>252</v>
       </c>
       <c r="C117" s="21"/>
     </row>
     <row r="118" spans="1:4" ht="24">
       <c r="A118" s="21" t="s">
-        <v>988</v>
+        <v>208</v>
       </c>
       <c r="B118" s="21" t="s">
-        <v>989</v>
+        <v>225</v>
       </c>
       <c r="C118" s="21"/>
     </row>
     <row r="119" spans="1:4" ht="24">
-      <c r="A119" s="21" t="s">
-        <v>1165</v>
-      </c>
-      <c r="B119" s="21" t="s">
-        <v>586</v>
+      <c r="A119" s="30" t="s">
+        <v>1132</v>
+      </c>
+      <c r="B119" s="30" t="s">
+        <v>677</v>
       </c>
       <c r="C119" s="21"/>
     </row>
     <row r="120" spans="1:4" ht="24">
       <c r="A120" s="21" t="s">
-        <v>582</v>
+        <v>566</v>
       </c>
       <c r="B120" s="21" t="s">
-        <v>583</v>
+        <v>567</v>
       </c>
       <c r="C120" s="21"/>
     </row>
     <row r="121" spans="1:4" ht="24">
       <c r="A121" s="21" t="s">
-        <v>792</v>
+        <v>1320</v>
       </c>
       <c r="B121" s="21" t="s">
-        <v>793</v>
+        <v>1321</v>
       </c>
       <c r="C121" s="21"/>
     </row>
     <row r="122" spans="1:4" ht="24">
       <c r="A122" s="21" t="s">
-        <v>241</v>
+        <v>768</v>
       </c>
       <c r="B122" s="21" t="s">
-        <v>243</v>
+        <v>769</v>
       </c>
       <c r="C122" s="21"/>
     </row>
     <row r="123" spans="1:4" ht="24">
       <c r="A123" s="21" t="s">
-        <v>1166</v>
+        <v>988</v>
       </c>
       <c r="B123" s="21" t="s">
-        <v>1156</v>
+        <v>989</v>
       </c>
       <c r="C123" s="21"/>
     </row>
     <row r="124" spans="1:4" ht="24">
       <c r="A124" s="21" t="s">
-        <v>313</v>
+        <v>1165</v>
       </c>
       <c r="B124" s="21" t="s">
-        <v>594</v>
+        <v>586</v>
       </c>
       <c r="C124" s="21"/>
     </row>
     <row r="125" spans="1:4" ht="24">
       <c r="A125" s="21" t="s">
-        <v>726</v>
+        <v>582</v>
       </c>
       <c r="B125" s="21" t="s">
-        <v>727</v>
+        <v>583</v>
       </c>
       <c r="C125" s="21"/>
     </row>
     <row r="126" spans="1:4" ht="24">
       <c r="A126" s="21" t="s">
-        <v>207</v>
+        <v>792</v>
       </c>
       <c r="B126" s="21" t="s">
-        <v>224</v>
+        <v>793</v>
       </c>
       <c r="C126" s="21"/>
     </row>
     <row r="127" spans="1:4" ht="24">
       <c r="A127" s="21" t="s">
-        <v>1150</v>
+        <v>241</v>
       </c>
       <c r="B127" s="21" t="s">
-        <v>1151</v>
+        <v>243</v>
       </c>
       <c r="C127" s="21"/>
     </row>
     <row r="128" spans="1:4" ht="24">
       <c r="A128" s="21" t="s">
-        <v>1152</v>
+        <v>1166</v>
       </c>
       <c r="B128" s="21" t="s">
-        <v>1153</v>
+        <v>1156</v>
       </c>
       <c r="C128" s="21"/>
     </row>
     <row r="129" spans="1:3" ht="24">
       <c r="A129" s="21" t="s">
-        <v>1154</v>
+        <v>313</v>
       </c>
       <c r="B129" s="21" t="s">
-        <v>1155</v>
+        <v>594</v>
       </c>
       <c r="C129" s="21"/>
     </row>
     <row r="130" spans="1:3" ht="24">
       <c r="A130" s="21" t="s">
-        <v>597</v>
+        <v>726</v>
       </c>
       <c r="B130" s="21" t="s">
-        <v>598</v>
+        <v>727</v>
       </c>
       <c r="C130" s="21"/>
     </row>
     <row r="131" spans="1:3" ht="24">
       <c r="A131" s="21" t="s">
-        <v>240</v>
+        <v>207</v>
       </c>
       <c r="B131" s="21" t="s">
-        <v>242</v>
+        <v>224</v>
       </c>
       <c r="C131" s="21"/>
     </row>
     <row r="132" spans="1:3" ht="24">
       <c r="A132" s="21" t="s">
-        <v>788</v>
+        <v>1150</v>
       </c>
       <c r="B132" s="21" t="s">
-        <v>789</v>
+        <v>1151</v>
       </c>
       <c r="C132" s="21"/>
     </row>
     <row r="133" spans="1:3" ht="24">
       <c r="A133" s="21" t="s">
-        <v>786</v>
+        <v>1152</v>
       </c>
       <c r="B133" s="21" t="s">
-        <v>787</v>
+        <v>1153</v>
       </c>
       <c r="C133" s="21"/>
     </row>
     <row r="134" spans="1:3" ht="24">
       <c r="A134" s="21" t="s">
-        <v>850</v>
+        <v>1154</v>
       </c>
       <c r="B134" s="21" t="s">
-        <v>851</v>
+        <v>1155</v>
       </c>
       <c r="C134" s="21"/>
     </row>
     <row r="135" spans="1:3" ht="24">
       <c r="A135" s="21" t="s">
-        <v>790</v>
+        <v>597</v>
       </c>
       <c r="B135" s="21" t="s">
-        <v>791</v>
+        <v>598</v>
       </c>
       <c r="C135" s="21"/>
     </row>
     <row r="136" spans="1:3" ht="24">
       <c r="A136" s="21" t="s">
-        <v>574</v>
+        <v>240</v>
       </c>
       <c r="B136" s="21" t="s">
-        <v>575</v>
+        <v>242</v>
       </c>
       <c r="C136" s="21"/>
     </row>
     <row r="137" spans="1:3" ht="24">
       <c r="A137" s="21" t="s">
-        <v>205</v>
+        <v>788</v>
       </c>
       <c r="B137" s="21" t="s">
-        <v>221</v>
-      </c>
-      <c r="C137" s="21" t="s">
-        <v>222</v>
-      </c>
+        <v>789</v>
+      </c>
+      <c r="C137" s="21"/>
     </row>
     <row r="138" spans="1:3" ht="24">
       <c r="A138" s="21" t="s">
-        <v>245</v>
+        <v>786</v>
       </c>
       <c r="B138" s="21" t="s">
-        <v>246</v>
+        <v>787</v>
       </c>
       <c r="C138" s="21"/>
     </row>
-    <row r="139" spans="1:3" ht="25">
-      <c r="A139" s="47" t="s">
-        <v>1481</v>
-      </c>
-      <c r="B139" s="47" t="s">
-        <v>1482</v>
+    <row r="139" spans="1:3" ht="24">
+      <c r="A139" s="21" t="s">
+        <v>850</v>
+      </c>
+      <c r="B139" s="21" t="s">
+        <v>851</v>
       </c>
       <c r="C139" s="21"/>
     </row>
     <row r="140" spans="1:3" ht="24">
       <c r="A140" s="21" t="s">
-        <v>994</v>
+        <v>790</v>
       </c>
       <c r="B140" s="21" t="s">
-        <v>995</v>
+        <v>791</v>
       </c>
       <c r="C140" s="21"/>
     </row>
     <row r="141" spans="1:3" ht="24">
       <c r="A141" s="21" t="s">
-        <v>774</v>
+        <v>574</v>
       </c>
       <c r="B141" s="21" t="s">
-        <v>775</v>
+        <v>575</v>
       </c>
       <c r="C141" s="21"/>
     </row>
     <row r="142" spans="1:3" ht="24">
       <c r="A142" s="21" t="s">
-        <v>584</v>
+        <v>205</v>
       </c>
       <c r="B142" s="21" t="s">
-        <v>585</v>
-      </c>
-      <c r="C142" s="21"/>
-    </row>
-    <row r="143" spans="1:3" ht="25">
-      <c r="A143" s="47" t="s">
-        <v>1495</v>
-      </c>
-      <c r="B143" s="47" t="s">
-        <v>1496</v>
+        <v>221</v>
+      </c>
+      <c r="C142" s="21" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" ht="24">
+      <c r="A143" s="21" t="s">
+        <v>245</v>
+      </c>
+      <c r="B143" s="21" t="s">
+        <v>246</v>
       </c>
       <c r="C143" s="21"/>
     </row>
-    <row r="144" spans="1:3" ht="24">
-      <c r="A144" s="21" t="s">
-        <v>185</v>
-      </c>
-      <c r="B144" s="21" t="s">
-        <v>186</v>
+    <row r="144" spans="1:3" ht="25">
+      <c r="A144" s="47" t="s">
+        <v>1481</v>
+      </c>
+      <c r="B144" s="47" t="s">
+        <v>1482</v>
       </c>
       <c r="C144" s="21"/>
     </row>
     <row r="145" spans="1:3" ht="24">
       <c r="A145" s="21" t="s">
-        <v>226</v>
+        <v>1791</v>
       </c>
       <c r="B145" s="21" t="s">
-        <v>227</v>
+        <v>711</v>
       </c>
       <c r="C145" s="21"/>
     </row>
-    <row r="146" spans="1:3" ht="25">
-      <c r="A146" s="47" t="s">
-        <v>1501</v>
-      </c>
-      <c r="B146" s="47" t="s">
-        <v>1502</v>
+    <row r="146" spans="1:3" ht="24">
+      <c r="A146" s="21" t="s">
+        <v>994</v>
+      </c>
+      <c r="B146" s="21" t="s">
+        <v>995</v>
       </c>
       <c r="C146" s="21"/>
     </row>
-    <row r="147" spans="1:3" ht="25">
-      <c r="A147" s="47" t="s">
-        <v>1442</v>
-      </c>
-      <c r="B147" s="47" t="s">
-        <v>1478</v>
+    <row r="147" spans="1:3" ht="24">
+      <c r="A147" s="21" t="s">
+        <v>774</v>
+      </c>
+      <c r="B147" s="21" t="s">
+        <v>775</v>
       </c>
       <c r="C147" s="21"/>
     </row>
     <row r="148" spans="1:3" ht="24">
       <c r="A148" s="21" t="s">
-        <v>1325</v>
+        <v>584</v>
       </c>
       <c r="B148" s="21" t="s">
-        <v>237</v>
+        <v>585</v>
       </c>
       <c r="C148" s="21"/>
     </row>
-    <row r="149" spans="1:3" ht="24">
-      <c r="A149" s="21" t="s">
-        <v>238</v>
-      </c>
-      <c r="B149" s="21" t="s">
-        <v>237</v>
+    <row r="149" spans="1:3" ht="25">
+      <c r="A149" s="47" t="s">
+        <v>1495</v>
+      </c>
+      <c r="B149" s="47" t="s">
+        <v>1496</v>
       </c>
       <c r="C149" s="21"/>
     </row>
     <row r="150" spans="1:3" ht="24">
       <c r="A150" s="48" t="s">
-        <v>235</v>
+        <v>185</v>
       </c>
       <c r="B150" s="48" t="s">
-        <v>236</v>
+        <v>186</v>
       </c>
       <c r="C150" s="21"/>
     </row>
     <row r="151" spans="1:3" ht="24">
       <c r="A151" s="48" t="s">
-        <v>860</v>
+        <v>226</v>
       </c>
       <c r="B151" s="48" t="s">
-        <v>861</v>
+        <v>227</v>
       </c>
       <c r="C151" s="21"/>
     </row>
     <row r="152" spans="1:3" ht="25">
       <c r="A152" s="60" t="s">
-        <v>1503</v>
+        <v>1501</v>
       </c>
       <c r="B152" s="60" t="s">
-        <v>1504</v>
+        <v>1502</v>
       </c>
       <c r="C152" s="21"/>
     </row>
-    <row r="153" spans="1:3" ht="24">
-      <c r="A153" s="48" t="s">
-        <v>784</v>
-      </c>
-      <c r="B153" s="48" t="s">
-        <v>785</v>
+    <row r="153" spans="1:3" ht="25">
+      <c r="A153" s="60" t="s">
+        <v>1442</v>
+      </c>
+      <c r="B153" s="60" t="s">
+        <v>1478</v>
       </c>
       <c r="C153" s="21"/>
     </row>
     <row r="154" spans="1:3" ht="24">
       <c r="A154" s="48" t="s">
-        <v>743</v>
+        <v>1325</v>
       </c>
       <c r="B154" s="48" t="s">
-        <v>998</v>
+        <v>237</v>
       </c>
       <c r="C154" s="21"/>
     </row>
-    <row r="155" spans="1:3" ht="25">
-      <c r="A155" s="60" t="s">
-        <v>1493</v>
-      </c>
-      <c r="B155" s="60" t="s">
-        <v>1494</v>
+    <row r="155" spans="1:3" ht="24">
+      <c r="A155" s="48" t="s">
+        <v>238</v>
+      </c>
+      <c r="B155" s="48" t="s">
+        <v>237</v>
       </c>
       <c r="C155" s="21"/>
     </row>
     <row r="156" spans="1:3" ht="24">
       <c r="A156" s="48" t="s">
-        <v>184</v>
+        <v>235</v>
       </c>
       <c r="B156" s="48" t="s">
-        <v>1674</v>
+        <v>236</v>
       </c>
       <c r="C156" s="21"/>
     </row>
     <row r="157" spans="1:3" ht="24">
       <c r="A157" s="48" t="s">
-        <v>209</v>
+        <v>860</v>
       </c>
       <c r="B157" s="48" t="s">
-        <v>210</v>
+        <v>861</v>
       </c>
       <c r="C157" s="21"/>
     </row>
-    <row r="158" spans="1:3" ht="24">
-      <c r="A158" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="B158" s="48" t="s">
-        <v>170</v>
+    <row r="158" spans="1:3" ht="25">
+      <c r="A158" s="60" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B158" s="60" t="s">
+        <v>1504</v>
       </c>
       <c r="C158" s="21"/>
     </row>
     <row r="159" spans="1:3" ht="24">
       <c r="A159" s="48" t="s">
-        <v>387</v>
+        <v>784</v>
       </c>
       <c r="B159" s="48" t="s">
-        <v>399</v>
+        <v>785</v>
       </c>
       <c r="C159" s="21"/>
     </row>
     <row r="160" spans="1:3" ht="24">
       <c r="A160" s="48" t="s">
-        <v>1167</v>
+        <v>743</v>
       </c>
       <c r="B160" s="48" t="s">
-        <v>591</v>
-      </c>
-      <c r="C160" s="9"/>
-    </row>
-    <row r="161" spans="1:3" ht="24">
-      <c r="A161" s="48" t="s">
-        <v>797</v>
-      </c>
-      <c r="B161" s="48" t="s">
-        <v>286</v>
+        <v>998</v>
+      </c>
+      <c r="C160" s="66"/>
+    </row>
+    <row r="161" spans="1:3" ht="25">
+      <c r="A161" s="60" t="s">
+        <v>1493</v>
+      </c>
+      <c r="B161" s="60" t="s">
+        <v>1494</v>
       </c>
       <c r="C161" s="21"/>
     </row>
     <row r="162" spans="1:3" ht="24">
       <c r="A162" s="48" t="s">
-        <v>1000</v>
+        <v>184</v>
       </c>
       <c r="B162" s="48" t="s">
-        <v>1001</v>
+        <v>1674</v>
       </c>
       <c r="C162" s="21"/>
     </row>
     <row r="163" spans="1:3" ht="24">
       <c r="A163" s="48" t="s">
-        <v>1157</v>
+        <v>209</v>
       </c>
       <c r="B163" s="48" t="s">
-        <v>1158</v>
+        <v>210</v>
       </c>
       <c r="C163" s="21"/>
     </row>
     <row r="164" spans="1:3" ht="24">
       <c r="A164" s="48" t="s">
-        <v>166</v>
+        <v>179</v>
       </c>
       <c r="B164" s="48" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="C164" s="21"/>
     </row>
     <row r="165" spans="1:3" ht="24">
       <c r="A165" s="21" t="s">
-        <v>408</v>
+        <v>387</v>
       </c>
       <c r="B165" s="61" t="s">
-        <v>719</v>
+        <v>399</v>
       </c>
       <c r="C165" s="21"/>
     </row>
     <row r="166" spans="1:3" ht="24">
       <c r="A166" s="59" t="s">
-        <v>211</v>
+        <v>1167</v>
       </c>
       <c r="B166" s="59" t="s">
-        <v>212</v>
+        <v>591</v>
       </c>
       <c r="C166" s="21"/>
     </row>
     <row r="167" spans="1:3" ht="24">
       <c r="A167" s="58" t="s">
-        <v>1105</v>
+        <v>797</v>
       </c>
       <c r="B167" s="59" t="s">
-        <v>1002</v>
+        <v>286</v>
       </c>
       <c r="C167" s="21"/>
     </row>
     <row r="168" spans="1:3" ht="24">
       <c r="A168" s="21" t="s">
-        <v>778</v>
+        <v>1000</v>
       </c>
       <c r="B168" s="21" t="s">
-        <v>779</v>
+        <v>1001</v>
       </c>
       <c r="C168" s="21"/>
     </row>
     <row r="169" spans="1:3" ht="24">
       <c r="A169" s="21" t="s">
-        <v>198</v>
+        <v>1157</v>
       </c>
       <c r="B169" s="21" t="s">
-        <v>213</v>
+        <v>1158</v>
       </c>
       <c r="C169" s="21"/>
     </row>
     <row r="170" spans="1:3" ht="24">
       <c r="A170" s="21" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="B170" s="21" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="C170" s="21"/>
     </row>
     <row r="171" spans="1:3" ht="24">
       <c r="A171" s="21" t="s">
-        <v>174</v>
+        <v>408</v>
       </c>
       <c r="B171" s="21" t="s">
-        <v>173</v>
+        <v>719</v>
       </c>
       <c r="C171" s="21"/>
     </row>
     <row r="172" spans="1:3" ht="24">
       <c r="A172" s="21" t="s">
-        <v>1754</v>
+        <v>211</v>
       </c>
       <c r="B172" s="21" t="s">
-        <v>1755</v>
+        <v>212</v>
       </c>
       <c r="C172" s="21"/>
     </row>
     <row r="173" spans="1:3" ht="24">
-      <c r="A173" s="21"/>
-      <c r="B173" s="21"/>
+      <c r="A173" s="21" t="s">
+        <v>1105</v>
+      </c>
+      <c r="B173" s="21" t="s">
+        <v>1002</v>
+      </c>
       <c r="C173" s="21"/>
     </row>
     <row r="174" spans="1:3" ht="24">
       <c r="A174" s="21" t="s">
-        <v>1787</v>
+        <v>778</v>
       </c>
       <c r="B174" s="21" t="s">
-        <v>1788</v>
+        <v>779</v>
       </c>
       <c r="C174" s="21"/>
     </row>
     <row r="175" spans="1:3" ht="24">
       <c r="A175" s="21" t="s">
-        <v>1789</v>
+        <v>198</v>
       </c>
       <c r="B175" s="21" t="s">
-        <v>664</v>
+        <v>213</v>
       </c>
       <c r="C175" s="21"/>
     </row>
     <row r="176" spans="1:3" ht="24">
       <c r="A176" s="21" t="s">
-        <v>1790</v>
+        <v>175</v>
       </c>
       <c r="B176" s="21" t="s">
-        <v>672</v>
+        <v>176</v>
       </c>
       <c r="C176" s="21"/>
     </row>
     <row r="177" spans="1:3" ht="24">
       <c r="A177" s="21" t="s">
-        <v>1791</v>
+        <v>174</v>
       </c>
       <c r="B177" s="21" t="s">
-        <v>711</v>
+        <v>173</v>
       </c>
       <c r="C177" s="21"/>
     </row>
     <row r="178" spans="1:3" ht="24">
-      <c r="A178" s="21" t="s">
-        <v>1792</v>
-      </c>
-      <c r="B178" s="21" t="s">
-        <v>680</v>
-      </c>
       <c r="C178" s="21"/>
     </row>
     <row r="179" spans="1:3" ht="24">
@@ -16366,8 +16365,8 @@
       <c r="C246" s="21"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A6:C173">
-    <sortCondition ref="A6:A173"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A5:C178">
+    <sortCondition ref="A5:A178"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>